<commit_message>
ANW-3030 Use numbered file version columns in the archival object import
Replace the rep_* and nonrep_* columns of the archival object import template
with file_version_<field>_<N> columns, numbered at the end like the rest of the
template, with the fields and the Make Display Thumbnail / Make Display Link
flags of the digital object import. The template has two file versions; more
can be added with _3, _4, ... columns.

A spreadsheet with the old rep_* or nonrep_* columns, or a file_version column
for a field that does not exist, now aborts the import: the importer ignores
unknown columns, so such a spreadsheet would otherwise create no file versions.

The fixtures move their rep data to file version 1 as the Display Thumbnail and
their nonrep data to file version 2, which is the Display Link when published,
as the old columns meant.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/spec/fixtures/bulk_import/bulk_import_VFIRST01_test01.xlsx
+++ b/backend/spec/fixtures/bulk_import/bulk_import_VFIRST01_test01.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:sst xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="545">
+<ns0:sst xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="650">
   <ns0:si>
     <ns0:t>Mapping - ArchivesSpace Resource record SECTION</ns0:t>
   </ns0:si>
@@ -1668,6 +1668,327 @@
   </ns0:si>
   <ns0:si>
     <ns0:t>Accession URI (link to existing accession record)</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version Linked-to URL
+Duplicate the columns and increment the index to add more versions.
+file_version_*_3
+file_version_*_4, etc.</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Publish file version? A Display Thumbnail or Display Link file version is always published.</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Use Statement</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Xlink actuate attribute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Xlink show attribute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Format Name</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Format Version</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File size (bytes)</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Checksum</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Checksum Method</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Make Display Thumbnail?</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Make Display Link?</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Caption</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version Linked-to URL
+Duplicate the columns and increment the index to add more versions.
+file_version_*_3
+file_version_*_4, etc.</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Publish file version? A Display Thumbnail or Display Link file version is always published.</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Use Statement</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Xlink actuate attribute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Xlink show attribute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Format Name</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Format Version</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File size (bytes)</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Checksum</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Checksum Method</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Make Display Thumbnail?</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Make Display Link?</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Caption</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_file_uri_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_publish_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_use_statement_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_xlink_actuate_attribute_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_xlink_show_attribute_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_file_format_name_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_file_format_version_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_file_size_bytes_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_checksum_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_checksum_method_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_is_display_thumbnail_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_is_display_link_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_caption_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_file_uri_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_publish_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_use_statement_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_xlink_actuate_attribute_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_xlink_show_attribute_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_file_format_name_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_file_format_version_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_file_size_bytes_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_checksum_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_checksum_method_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_is_display_thumbnail_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_is_display_link_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">file_version_caption_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(1) URI</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(1) Publish</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(1) Use Statement</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(1) xlink actuate attribute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(1) xlink show attribute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(1) File Format Name</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(1) File Format Version</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(1) File Size Bytes</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(1) Checksum</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(1) Checksum Method</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(1) Make Display Thumbnail</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(1) Make Display Link</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(1) Caption</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(2) URI</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(2) Publish</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(2) Use Statement</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(2) xlink actuate attribute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(2) xlink show attribute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(2) File Format Name</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(2) File Format Version</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(2) File Size Bytes</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(2) Checksum</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(2) Checksum Method</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(2) Make Display Thumbnail</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(2) Make Display Link</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">File Version(2) Caption</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">TRUE</ns0:t>
   </ns0:si>
 </ns0:sst>
 </file>
@@ -2622,7 +2943,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns6="http://schemas.microsoft.com/office/excel/2006/main" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
-  <ns0:dimension ref="A1:ASK7"/>
+  <ns0:dimension ref="A1:ASP7"/>
   <ns0:sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" ns3:dyDescent="0.2"/>
   <ns0:cols>
     <ns0:col min="1" max="1" width="13.1640625" style="30" customWidth="1"/>
@@ -2674,108 +2995,126 @@
     <ns0:col min="66" max="66" width="15.83203125" style="1" customWidth="1"/>
     <ns0:col min="67" max="67" width="10.5" style="1" customWidth="1"/>
     <ns0:col min="68" max="68" width="20.6640625" customWidth="1"/>
-    <ns0:col min="69" max="80" width="12" style="1" customWidth="1"/>
-    <ns0:col min="81" max="81" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="82" max="83" width="12" style="1" customWidth="1"/>
-    <ns0:col min="84" max="84" width="22.6640625" style="1" customWidth="1"/>
-    <ns0:col min="85" max="85" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="86" max="86" width="13" style="1" customWidth="1"/>
-    <ns0:col min="87" max="87" width="15.5" style="1" customWidth="1"/>
-    <ns0:col min="88" max="88" width="22.6640625" style="1" customWidth="1"/>
-    <ns0:col min="89" max="90" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="91" max="91" width="22.6640625" style="1"/>
-    <ns0:col min="92" max="92" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="93" max="93" width="13" style="1" customWidth="1"/>
-    <ns0:col min="94" max="94" width="15.5" style="1" customWidth="1"/>
-    <ns0:col min="95" max="95" width="22.6640625" style="1"/>
-    <ns0:col min="96" max="96" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="97" max="97" width="9.1640625" style="1"/>
-    <ns0:col min="98" max="98" width="15.1640625" style="1" customWidth="1"/>
-    <ns0:col min="99" max="99" width="20.1640625" style="1" customWidth="1"/>
-    <ns0:col min="100" max="100" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="101" max="101" width="12.83203125" style="1" customWidth="1"/>
-    <ns0:col min="102" max="102" width="15.1640625" style="1" customWidth="1"/>
-    <ns0:col min="103" max="103" width="20.1640625" style="1" customWidth="1"/>
-    <ns0:col min="104" max="104" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="105" max="105" width="12.83203125" style="1" customWidth="1"/>
-    <ns0:col min="106" max="106" width="15.1640625" style="1" customWidth="1"/>
-    <ns0:col min="107" max="107" width="20.1640625" style="1" customWidth="1"/>
-    <ns0:col min="108" max="108" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="109" max="109" width="12.83203125" style="1" customWidth="1"/>
-    <ns0:col min="110" max="110" width="9.1640625" style="1"/>
-    <ns0:col min="111" max="111" width="11.5" style="1" customWidth="1"/>
-    <ns0:col min="112" max="112" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="113" max="114" width="9.1640625" style="1"/>
-    <ns0:col min="115" max="115" width="11.5" style="1" customWidth="1"/>
-    <ns0:col min="116" max="116" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="117" max="119" width="9.1640625" style="1"/>
-    <ns0:col min="120" max="120" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="121" max="123" width="9.1640625" style="1"/>
-    <ns0:col min="124" max="124" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="125" max="127" width="9.1640625" style="1"/>
-    <ns0:col min="128" max="128" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="129" max="129" width="9.1640625" style="1"/>
-    <ns0:col min="130" max="130" width="11.5" style="1" customWidth="1"/>
-    <ns0:col min="131" max="131" width="12.33203125" style="1" customWidth="1"/>
-    <ns0:col min="132" max="134" width="13.5" style="1" customWidth="1"/>
-    <ns0:col min="135" max="136" width="10.83203125" style="1" customWidth="1"/>
-    <ns0:col min="137" max="137" width="15.5" style="1" customWidth="1"/>
-    <ns0:col min="138" max="138" width="9.33203125" style="1"/>
-    <ns0:col min="139" max="139" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="140" max="140" width="17.6640625" customWidth="1"/>
-    <ns0:col min="141" max="141" width="17" style="1" customWidth="1"/>
-    <ns0:col min="142" max="142" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="143" max="143" width="17.6640625" customWidth="1"/>
-    <ns0:col min="144" max="145" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="146" max="147" width="12.33203125" style="1" customWidth="1"/>
-    <ns0:col min="148" max="148" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="149" max="149" width="17.6640625" customWidth="1"/>
-    <ns0:col min="150" max="150" width="11.6640625" style="1" customWidth="1"/>
-    <ns0:col min="151" max="151" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="152" max="152" width="17.6640625" customWidth="1"/>
-    <ns0:col min="153" max="153" width="16" style="1" customWidth="1"/>
-    <ns0:col min="154" max="154" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="155" max="155" width="17.6640625" customWidth="1"/>
-    <ns0:col min="156" max="156" width="9.1640625" style="1"/>
-    <ns0:col min="157" max="157" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="158" max="158" width="17.6640625" customWidth="1"/>
-    <ns0:col min="159" max="159" width="12" customWidth="1"/>
-    <ns0:col min="160" max="160" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="161" max="161" width="17.6640625" customWidth="1"/>
-    <ns0:col min="162" max="162" width="11.83203125" style="1" customWidth="1"/>
-    <ns0:col min="163" max="163" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="164" max="164" width="17.6640625" customWidth="1"/>
-    <ns0:col min="165" max="165" width="11.83203125" style="1" customWidth="1"/>
-    <ns0:col min="166" max="166" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="167" max="167" width="17.6640625" customWidth="1"/>
-    <ns0:col min="168" max="168" width="11.83203125" style="1" customWidth="1"/>
-    <ns0:col min="169" max="169" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="69" max="69" width="24" customWidth="1"/>
+    <ns0:col min="70" max="70" width="24" customWidth="1"/>
+    <ns0:col min="71" max="71" width="24" customWidth="1"/>
+    <ns0:col min="72" max="72" width="24" customWidth="1"/>
+    <ns0:col min="73" max="73" width="24" customWidth="1"/>
+    <ns0:col min="74" max="74" width="24" customWidth="1"/>
+    <ns0:col min="75" max="75" width="24" customWidth="1"/>
+    <ns0:col min="76" max="76" width="24" customWidth="1"/>
+    <ns0:col min="77" max="77" width="24" customWidth="1"/>
+    <ns0:col min="78" max="78" width="24" customWidth="1"/>
+    <ns0:col min="79" max="79" width="24" customWidth="1"/>
+    <ns0:col min="80" max="80" width="24" customWidth="1"/>
+    <ns0:col min="81" max="81" width="24" customWidth="1"/>
+    <ns0:col min="82" max="82" width="24" customWidth="1"/>
+    <ns0:col min="83" max="83" width="24" customWidth="1"/>
+    <ns0:col min="84" max="84" width="24" customWidth="1"/>
+    <ns0:col min="85" max="85" width="24" customWidth="1"/>
+    <ns0:col min="86" max="86" width="24" customWidth="1"/>
+    <ns0:col min="87" max="87" width="24" customWidth="1"/>
+    <ns0:col min="88" max="88" width="24" customWidth="1"/>
+    <ns0:col min="89" max="89" width="24" customWidth="1"/>
+    <ns0:col min="90" max="90" width="24" customWidth="1"/>
+    <ns0:col min="91" max="91" width="24" customWidth="1"/>
+    <ns0:col min="92" max="92" width="24" customWidth="1"/>
+    <ns0:col min="93" max="93" width="24" customWidth="1"/>
+    <ns0:col min="94" max="94" width="24" customWidth="1"/>
+    <ns0:col min="95" max="95" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="96" max="96" width="22.6640625" style="1"/>
+    <ns0:col min="97" max="97" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="98" max="98" width="13" style="1" customWidth="1"/>
+    <ns0:col min="99" max="99" width="15.5" style="1" customWidth="1"/>
+    <ns0:col min="100" max="100" width="22.6640625" style="1"/>
+    <ns0:col min="101" max="101" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="102" max="102" width="9.1640625" style="1"/>
+    <ns0:col min="103" max="103" width="15.1640625" style="1" customWidth="1"/>
+    <ns0:col min="104" max="104" width="20.1640625" style="1" customWidth="1"/>
+    <ns0:col min="105" max="105" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="106" max="106" width="12.83203125" style="1" customWidth="1"/>
+    <ns0:col min="107" max="107" width="15.1640625" style="1" customWidth="1"/>
+    <ns0:col min="108" max="108" width="20.1640625" style="1" customWidth="1"/>
+    <ns0:col min="109" max="109" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="110" max="110" width="12.83203125" style="1" customWidth="1"/>
+    <ns0:col min="111" max="111" width="15.1640625" style="1" customWidth="1"/>
+    <ns0:col min="112" max="112" width="20.1640625" style="1" customWidth="1"/>
+    <ns0:col min="113" max="113" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="114" max="114" width="12.83203125" style="1" customWidth="1"/>
+    <ns0:col min="115" max="115" width="9.1640625" style="1"/>
+    <ns0:col min="116" max="116" width="11.5" style="1" customWidth="1"/>
+    <ns0:col min="117" max="117" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="118" max="119" width="9.1640625" style="1"/>
+    <ns0:col min="120" max="120" width="11.5" style="1" customWidth="1"/>
+    <ns0:col min="121" max="121" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="122" max="124" width="9.1640625" style="1"/>
+    <ns0:col min="125" max="125" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="126" max="128" width="9.1640625" style="1"/>
+    <ns0:col min="129" max="129" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="130" max="132" width="9.1640625" style="1"/>
+    <ns0:col min="133" max="133" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="134" max="134" width="9.1640625" style="1"/>
+    <ns0:col min="135" max="135" width="11.5" style="1" customWidth="1"/>
+    <ns0:col min="136" max="136" width="12.33203125" style="1" customWidth="1"/>
+    <ns0:col min="137" max="139" width="13.5" style="1" customWidth="1"/>
+    <ns0:col min="140" max="141" width="10.83203125" style="1" customWidth="1"/>
+    <ns0:col min="142" max="142" width="15.5" style="1" customWidth="1"/>
+    <ns0:col min="143" max="143" width="9.33203125" style="1"/>
+    <ns0:col min="144" max="144" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="145" max="145" width="17.6640625" customWidth="1"/>
+    <ns0:col min="146" max="146" width="17" style="1" customWidth="1"/>
+    <ns0:col min="147" max="147" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="148" max="148" width="17.6640625" customWidth="1"/>
+    <ns0:col min="149" max="150" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="151" max="152" width="12.33203125" style="1" customWidth="1"/>
+    <ns0:col min="153" max="153" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="154" max="154" width="17.6640625" customWidth="1"/>
+    <ns0:col min="155" max="155" width="11.6640625" style="1" customWidth="1"/>
+    <ns0:col min="156" max="156" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="157" max="157" width="17.6640625" customWidth="1"/>
+    <ns0:col min="158" max="158" width="16" style="1" customWidth="1"/>
+    <ns0:col min="159" max="159" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="160" max="160" width="17.6640625" customWidth="1"/>
+    <ns0:col min="161" max="161" width="9.1640625" style="1"/>
+    <ns0:col min="162" max="162" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="163" max="163" width="17.6640625" customWidth="1"/>
+    <ns0:col min="164" max="164" width="12" customWidth="1"/>
+    <ns0:col min="165" max="165" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="166" max="166" width="17.6640625" customWidth="1"/>
+    <ns0:col min="167" max="167" width="11.83203125" style="1" customWidth="1"/>
+    <ns0:col min="168" max="168" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="169" max="169" width="17.6640625" customWidth="1"/>
     <ns0:col min="170" max="170" width="11.83203125" style="1" customWidth="1"/>
-    <ns0:col min="171" max="171" width="17.6640625" customWidth="1"/>
-    <ns0:col min="172" max="172" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="173" max="173" width="17.6640625" customWidth="1"/>
-    <ns0:col min="174" max="174" width="14.83203125" style="1" customWidth="1"/>
-    <ns0:col min="175" max="175" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="171" max="171" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="172" max="172" width="17.6640625" customWidth="1"/>
+    <ns0:col min="173" max="173" width="11.83203125" style="1" customWidth="1"/>
+    <ns0:col min="174" max="174" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="175" max="175" width="11.83203125" style="1" customWidth="1"/>
     <ns0:col min="176" max="176" width="17.6640625" customWidth="1"/>
-    <ns0:col min="177" max="177" width="12.33203125" style="1" customWidth="1"/>
-    <ns0:col min="178" max="178" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="179" max="179" width="17.6640625" customWidth="1"/>
-    <ns0:col min="180" max="180" width="9.1640625" style="1"/>
-    <ns0:col min="181" max="181" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="182" max="182" width="17.6640625" customWidth="1"/>
-    <ns0:col min="183" max="183" width="9.1640625" style="1"/>
-    <ns0:col min="184" max="184" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="185" max="185" width="17.6640625" customWidth="1"/>
-    <ns0:col min="186" max="186" width="18.5" style="1" customWidth="1"/>
-    <ns0:col min="187" max="187" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="188" max="188" width="17.6640625" customWidth="1"/>
-    <ns0:col min="189" max="189" width="10.1640625" style="1" customWidth="1"/>
-    <ns0:col min="190" max="190" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="191" max="193" width="17.6640625" customWidth="1"/>
-    <ns0:col min="194" max="1180" width="9.33203125" style="1"/>
+    <ns0:col min="177" max="177" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="178" max="178" width="17.6640625" customWidth="1"/>
+    <ns0:col min="179" max="179" width="14.83203125" style="1" customWidth="1"/>
+    <ns0:col min="180" max="180" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="181" max="181" width="17.6640625" customWidth="1"/>
+    <ns0:col min="182" max="182" width="12.33203125" style="1" customWidth="1"/>
+    <ns0:col min="183" max="183" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="184" max="184" width="17.6640625" customWidth="1"/>
+    <ns0:col min="185" max="185" width="9.1640625" style="1"/>
+    <ns0:col min="186" max="186" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="187" max="187" width="17.6640625" customWidth="1"/>
+    <ns0:col min="188" max="188" width="9.1640625" style="1"/>
+    <ns0:col min="189" max="189" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="190" max="190" width="17.6640625" customWidth="1"/>
+    <ns0:col min="191" max="191" width="18.5" style="1" customWidth="1"/>
+    <ns0:col min="192" max="192" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="193" max="193" width="17.6640625" customWidth="1"/>
+    <ns0:col min="194" max="194" width="10.1640625" style="1" customWidth="1"/>
+    <ns0:col min="195" max="195" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="196" max="198" width="17.6640625" customWidth="1"/>
+    <ns0:col min="199" max="1185" width="9.33203125" style="1"/>
   </ns0:cols>
   <ns0:sheetData>
-    <ns0:row r="1" spans="1:193" ht="16" thickBot="1" ns3:dyDescent="0.25">
+    <ns0:row r="1" spans="1:198" ht="16" thickBot="1" ns3:dyDescent="0.25">
       <ns0:c r="A1" s="30" t="s">
         <ns0:v>385</ns0:v>
       </ns0:c>
@@ -2785,27 +3124,27 @@
       <ns0:c r="R1"/>
       <ns0:c r="S1"/>
       <ns0:c r="T1"/>
-      <ns0:c r="EK1" s="1"/>
-      <ns0:c r="EN1" s="1"/>
-      <ns0:c r="ET1" s="1"/>
-      <ns0:c r="EW1" s="1"/>
-      <ns0:c r="EZ1" s="1"/>
-      <ns0:c r="FC1" s="1"/>
-      <ns0:c r="FF1" s="1"/>
-      <ns0:c r="FI1" s="1"/>
-      <ns0:c r="FL1" s="1"/>
-      <ns0:c r="FP1" s="1"/>
-      <ns0:c r="FR1" s="1"/>
+      <ns0:c r="EP1" s="1"/>
+      <ns0:c r="ES1" s="1"/>
+      <ns0:c r="EY1" s="1"/>
+      <ns0:c r="FB1" s="1"/>
+      <ns0:c r="FE1" s="1"/>
+      <ns0:c r="FH1" s="1"/>
+      <ns0:c r="FK1" s="1"/>
+      <ns0:c r="FN1" s="1"/>
+      <ns0:c r="FQ1" s="1"/>
       <ns0:c r="FU1" s="1"/>
-      <ns0:c r="FX1" s="1"/>
-      <ns0:c r="GA1" s="1"/>
-      <ns0:c r="GD1" s="1"/>
-      <ns0:c r="GG1" s="1"/>
-      <ns0:c r="GJ1" s="1"/>
-      <ns0:c r="GK1" s="1"/>
+      <ns0:c r="FW1" s="1"/>
+      <ns0:c r="FZ1" s="1"/>
+      <ns0:c r="GC1" s="1"/>
+      <ns0:c r="GF1" s="1"/>
+      <ns0:c r="GI1" s="1"/>
       <ns0:c r="GL1" s="1"/>
+      <ns0:c r="GO1" s="1"/>
+      <ns0:c r="GP1" s="1"/>
+      <ns0:c r="GQ1" s="1"/>
     </ns0:row>
-    <ns0:row r="2" spans="1:193" s="1" customFormat="1" ht="61" thickTop="1" ns3:dyDescent="0.2">
+    <ns0:row r="2" spans="1:198" s="1" customFormat="1" ht="61" thickTop="1" ns3:dyDescent="0.2">
       <ns0:c r="A2" s="32" t="s">
         <ns0:v>0</ns0:v>
       </ns0:c>
@@ -3011,90 +3350,90 @@
         <ns0:v>37</ns0:v>
       </ns0:c>
       <ns0:c r="BQ2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>545</ns0:v>
       </ns0:c>
       <ns0:c r="BR2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>546</ns0:v>
       </ns0:c>
       <ns0:c r="BS2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>547</ns0:v>
       </ns0:c>
       <ns0:c r="BT2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>548</ns0:v>
       </ns0:c>
       <ns0:c r="BU2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>549</ns0:v>
       </ns0:c>
       <ns0:c r="BV2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>550</ns0:v>
       </ns0:c>
       <ns0:c r="BW2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>551</ns0:v>
       </ns0:c>
       <ns0:c r="BX2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>552</ns0:v>
       </ns0:c>
       <ns0:c r="BY2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>553</ns0:v>
       </ns0:c>
       <ns0:c r="BZ2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>554</ns0:v>
       </ns0:c>
       <ns0:c r="CA2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>555</ns0:v>
       </ns0:c>
       <ns0:c r="CB2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>556</ns0:v>
       </ns0:c>
       <ns0:c r="CC2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>557</ns0:v>
       </ns0:c>
       <ns0:c r="CD2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>558</ns0:v>
       </ns0:c>
       <ns0:c r="CE2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>559</ns0:v>
       </ns0:c>
       <ns0:c r="CF2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>560</ns0:v>
       </ns0:c>
       <ns0:c r="CG2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>561</ns0:v>
       </ns0:c>
       <ns0:c r="CH2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>562</ns0:v>
       </ns0:c>
       <ns0:c r="CI2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>563</ns0:v>
       </ns0:c>
       <ns0:c r="CJ2" s="70" t="s">
-        <ns0:v>37</ns0:v>
+        <ns0:v>564</ns0:v>
       </ns0:c>
       <ns0:c r="CK2" s="70" t="s">
-        <ns0:v>37</ns0:v>
-      </ns0:c>
-      <ns0:c r="CL2" s="47" t="s">
+        <ns0:v>565</ns0:v>
+      </ns0:c>
+      <ns0:c r="CL2" s="70" t="s">
+        <ns0:v>566</ns0:v>
+      </ns0:c>
+      <ns0:c r="CM2" s="70" t="s">
+        <ns0:v>567</ns0:v>
+      </ns0:c>
+      <ns0:c r="CN2" s="70" t="s">
+        <ns0:v>568</ns0:v>
+      </ns0:c>
+      <ns0:c r="CO2" s="70" t="s">
+        <ns0:v>569</ns0:v>
+      </ns0:c>
+      <ns0:c r="CP2" s="70" t="s">
+        <ns0:v>570</ns0:v>
+      </ns0:c>
+      <ns0:c r="CQ2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="CM2" s="19" t="s">
+      <ns0:c r="CR2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="CN2" s="47" t="s">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="CO2" s="19" t="s">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="CP2" s="19" t="s">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="CQ2" s="19" t="s">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="CR2" s="47" t="s">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="CS2" s="19" t="s">
+      <ns0:c r="CS2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="CT2" s="19" t="s">
@@ -3103,10 +3442,10 @@
       <ns0:c r="CU2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="CV2" s="47" t="s">
+      <ns0:c r="CV2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="CW2" s="19" t="s">
+      <ns0:c r="CW2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="CX2" s="19" t="s">
@@ -3115,10 +3454,10 @@
       <ns0:c r="CY2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="CZ2" s="47" t="s">
+      <ns0:c r="CZ2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DA2" s="19" t="s">
+      <ns0:c r="DA2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="DB2" s="19" t="s">
@@ -3127,10 +3466,10 @@
       <ns0:c r="DC2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DD2" s="47" t="s">
+      <ns0:c r="DD2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DE2" s="19" t="s">
+      <ns0:c r="DE2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="DF2" s="19" t="s">
@@ -3139,10 +3478,10 @@
       <ns0:c r="DG2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DH2" s="47" t="s">
+      <ns0:c r="DH2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DI2" s="19" t="s">
+      <ns0:c r="DI2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="DJ2" s="19" t="s">
@@ -3151,10 +3490,10 @@
       <ns0:c r="DK2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DL2" s="47" t="s">
+      <ns0:c r="DL2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DM2" s="19" t="s">
+      <ns0:c r="DM2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="DN2" s="19" t="s">
@@ -3163,10 +3502,10 @@
       <ns0:c r="DO2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DP2" s="47" t="s">
+      <ns0:c r="DP2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DQ2" s="19" t="s">
+      <ns0:c r="DQ2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="DR2" s="19" t="s">
@@ -3175,10 +3514,10 @@
       <ns0:c r="DS2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DT2" s="47" t="s">
+      <ns0:c r="DT2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DU2" s="19" t="s">
+      <ns0:c r="DU2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="DV2" s="19" t="s">
@@ -3187,26 +3526,29 @@
       <ns0:c r="DW2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DX2" s="47" t="s">
+      <ns0:c r="DX2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DY2" s="19" t="s">
+      <ns0:c r="DY2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="EA2" s="21" t="s">
-        <ns0:v>108</ns0:v>
-      </ns0:c>
-      <ns0:c r="EB2" s="21" t="s">
-        <ns0:v>108</ns0:v>
-      </ns0:c>
-      <ns0:c r="EC2" s="21" t="s">
-        <ns0:v>108</ns0:v>
-      </ns0:c>
-      <ns0:c r="ED2" s="21" t="s">
-        <ns0:v>108</ns0:v>
-      </ns0:c>
-      <ns0:c r="EE2" s="21" t="s">
-        <ns0:v>108</ns0:v>
+      <ns0:c r="DZ2" s="19" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="EA2" s="19" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="EB2" s="19" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="EC2" s="47" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="ED2" s="19" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="EE2" t="s">
+        <ns0:v>543</ns0:v>
       </ns0:c>
       <ns0:c r="EF2" s="21" t="s">
         <ns0:v>108</ns0:v>
@@ -3217,115 +3559,115 @@
       <ns0:c r="EH2" s="21" t="s">
         <ns0:v>108</ns0:v>
       </ns0:c>
-      <ns0:c r="EI2" s="28" t="s">
+      <ns0:c r="EI2" s="21" t="s">
+        <ns0:v>108</ns0:v>
+      </ns0:c>
+      <ns0:c r="EJ2" s="21" t="s">
+        <ns0:v>108</ns0:v>
+      </ns0:c>
+      <ns0:c r="EK2" s="21" t="s">
+        <ns0:v>108</ns0:v>
+      </ns0:c>
+      <ns0:c r="EL2" s="21" t="s">
+        <ns0:v>108</ns0:v>
+      </ns0:c>
+      <ns0:c r="EM2" s="21" t="s">
+        <ns0:v>108</ns0:v>
+      </ns0:c>
+      <ns0:c r="EN2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EJ2" s="28" t="s">
+      <ns0:c r="EO2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EK2" s="67" t="s">
+      <ns0:c r="EP2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EL2" s="28" t="s">
-        <ns0:v>58</ns0:v>
-      </ns0:c>
-      <ns0:c r="EM2" s="28" t="s">
-        <ns0:v>58</ns0:v>
-      </ns0:c>
-      <ns0:c r="EN2" s="67" t="s">
-        <ns0:v>58</ns0:v>
-      </ns0:c>
-      <ns0:c r="EO2" s="66" t="s">
-        <ns0:v>58</ns0:v>
-      </ns0:c>
-      <ns0:c r="EP2" s="66" t="s">
-        <ns0:v>58</ns0:v>
-      </ns0:c>
-      <ns0:c r="EQ2" s="67" t="s">
+      <ns0:c r="EQ2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="ER2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="ES2" s="28" t="s">
+      <ns0:c r="ES2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="ET2" s="67" t="s">
+      <ns0:c r="ET2" s="66" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EU2" s="28" t="s">
+      <ns0:c r="EU2" s="66" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EV2" s="28" t="s">
+      <ns0:c r="EV2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EW2" s="67" t="s">
+      <ns0:c r="EW2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EX2" s="27" t="s">
+      <ns0:c r="EX2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EY2" s="28" t="s">
+      <ns0:c r="EY2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EZ2" s="67" t="s">
+      <ns0:c r="EZ2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FA2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FB2" s="28" t="s">
+      <ns0:c r="FB2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FC2" s="67" t="s">
+      <ns0:c r="FC2" s="27" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FD2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FE2" s="28" t="s">
+      <ns0:c r="FE2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FF2" s="67" t="s">
+      <ns0:c r="FF2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FG2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FH2" s="28" t="s">
+      <ns0:c r="FH2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FI2" s="67" t="s">
+      <ns0:c r="FI2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FJ2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FK2" s="28" t="s">
+      <ns0:c r="FK2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FL2" s="67" t="s">
+      <ns0:c r="FL2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FM2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FN2" s="28" t="s">
+      <ns0:c r="FN2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FO2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FP2" s="67" t="s">
+      <ns0:c r="FP2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FQ2" s="28" t="s">
+      <ns0:c r="FQ2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FR2" s="67" t="s">
+      <ns0:c r="FR2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FS2" s="29" t="s">
+      <ns0:c r="FS2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FT2" s="28" t="s">
@@ -3337,59 +3679,71 @@
       <ns0:c r="FV2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FW2" s="28" t="s">
+      <ns0:c r="FW2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FX2" s="67" t="s">
+      <ns0:c r="FX2" s="29" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FY2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FZ2" s="28" t="s">
+      <ns0:c r="FZ2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GA2" s="67" t="s">
+      <ns0:c r="GA2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="GB2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GC2" s="28" t="s">
+      <ns0:c r="GC2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GD2" s="67" t="s">
+      <ns0:c r="GD2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="GE2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GF2" s="28" t="s">
+      <ns0:c r="GF2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GG2" s="67" t="s">
+      <ns0:c r="GG2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="GH2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GI2" s="28" t="s">
+      <ns0:c r="GI2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GJ2" s="67" t="s">
+      <ns0:c r="GJ2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GK2" s="67" t="s">
+      <ns0:c r="GK2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="GL2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="DZ2" t="s">
-        <ns0:v>543</ns0:v>
+      <ns0:c r="GM2" s="28" t="s">
+        <ns0:v>58</ns0:v>
+      </ns0:c>
+      <ns0:c r="GN2" s="28" t="s">
+        <ns0:v>58</ns0:v>
+      </ns0:c>
+      <ns0:c r="GO2" s="67" t="s">
+        <ns0:v>58</ns0:v>
+      </ns0:c>
+      <ns0:c r="GP2" s="67" t="s">
+        <ns0:v>58</ns0:v>
+      </ns0:c>
+      <ns0:c r="GQ2" s="67" t="s">
+        <ns0:v>58</ns0:v>
       </ns0:c>
     </ns0:row>
-    <ns0:row r="3" spans="1:193" ht="105.75" customHeight="1" thickBot="1" ns3:dyDescent="0.25">
+    <ns0:row r="3" spans="1:198" ht="105.75" customHeight="1" thickBot="1" ns3:dyDescent="0.25">
       <ns0:c r="A3" s="33" t="s">
         <ns0:v>61</ns0:v>
       </ns0:c>
@@ -3593,385 +3947,400 @@
         <ns0:v>415</ns0:v>
       </ns0:c>
       <ns0:c r="BQ3" s="71" t="s">
-        <ns0:v>463</ns0:v>
+        <ns0:v>571</ns0:v>
       </ns0:c>
       <ns0:c r="BR3" s="71" t="s">
-        <ns0:v>464</ns0:v>
+        <ns0:v>572</ns0:v>
       </ns0:c>
       <ns0:c r="BS3" s="71" t="s">
-        <ns0:v>465</ns0:v>
+        <ns0:v>573</ns0:v>
       </ns0:c>
       <ns0:c r="BT3" s="71" t="s">
-        <ns0:v>466</ns0:v>
+        <ns0:v>574</ns0:v>
       </ns0:c>
       <ns0:c r="BU3" s="71" t="s">
-        <ns0:v>467</ns0:v>
+        <ns0:v>575</ns0:v>
       </ns0:c>
       <ns0:c r="BV3" s="71" t="s">
-        <ns0:v>468</ns0:v>
+        <ns0:v>576</ns0:v>
       </ns0:c>
       <ns0:c r="BW3" s="71" t="s">
-        <ns0:v>469</ns0:v>
+        <ns0:v>577</ns0:v>
       </ns0:c>
       <ns0:c r="BX3" s="71" t="s">
-        <ns0:v>470</ns0:v>
+        <ns0:v>578</ns0:v>
       </ns0:c>
       <ns0:c r="BY3" s="71" t="s">
-        <ns0:v>471</ns0:v>
+        <ns0:v>579</ns0:v>
       </ns0:c>
       <ns0:c r="BZ3" s="71" t="s">
-        <ns0:v>472</ns0:v>
+        <ns0:v>580</ns0:v>
       </ns0:c>
       <ns0:c r="CA3" s="71" t="s">
-        <ns0:v>473</ns0:v>
+        <ns0:v>581</ns0:v>
       </ns0:c>
       <ns0:c r="CB3" s="71" t="s">
-        <ns0:v>474</ns0:v>
+        <ns0:v>582</ns0:v>
       </ns0:c>
       <ns0:c r="CC3" s="71" t="s">
-        <ns0:v>475</ns0:v>
+        <ns0:v>583</ns0:v>
       </ns0:c>
       <ns0:c r="CD3" s="71" t="s">
-        <ns0:v>476</ns0:v>
+        <ns0:v>584</ns0:v>
       </ns0:c>
       <ns0:c r="CE3" s="71" t="s">
-        <ns0:v>477</ns0:v>
+        <ns0:v>585</ns0:v>
       </ns0:c>
       <ns0:c r="CF3" s="71" t="s">
-        <ns0:v>478</ns0:v>
+        <ns0:v>586</ns0:v>
       </ns0:c>
       <ns0:c r="CG3" s="71" t="s">
-        <ns0:v>479</ns0:v>
+        <ns0:v>587</ns0:v>
       </ns0:c>
       <ns0:c r="CH3" s="71" t="s">
-        <ns0:v>480</ns0:v>
+        <ns0:v>588</ns0:v>
       </ns0:c>
       <ns0:c r="CI3" s="71" t="s">
-        <ns0:v>481</ns0:v>
+        <ns0:v>589</ns0:v>
       </ns0:c>
       <ns0:c r="CJ3" s="71" t="s">
-        <ns0:v>482</ns0:v>
+        <ns0:v>590</ns0:v>
       </ns0:c>
       <ns0:c r="CK3" s="71" t="s">
-        <ns0:v>483</ns0:v>
-      </ns0:c>
-      <ns0:c r="CL3" s="26" t="s">
+        <ns0:v>591</ns0:v>
+      </ns0:c>
+      <ns0:c r="CL3" s="71" t="s">
+        <ns0:v>592</ns0:v>
+      </ns0:c>
+      <ns0:c r="CM3" s="71" t="s">
+        <ns0:v>593</ns0:v>
+      </ns0:c>
+      <ns0:c r="CN3" s="71" t="s">
+        <ns0:v>594</ns0:v>
+      </ns0:c>
+      <ns0:c r="CO3" s="71" t="s">
+        <ns0:v>595</ns0:v>
+      </ns0:c>
+      <ns0:c r="CP3" s="71" t="s">
+        <ns0:v>596</ns0:v>
+      </ns0:c>
+      <ns0:c r="CQ3" s="26" t="s">
         <ns0:v>160</ns0:v>
       </ns0:c>
-      <ns0:c r="CM3" s="26" t="s">
+      <ns0:c r="CR3" s="26" t="s">
         <ns0:v>162</ns0:v>
       </ns0:c>
-      <ns0:c r="CN3" s="26" t="s">
+      <ns0:c r="CS3" s="26" t="s">
         <ns0:v>247</ns0:v>
       </ns0:c>
-      <ns0:c r="CO3" s="26" t="s">
+      <ns0:c r="CT3" s="26" t="s">
         <ns0:v>275</ns0:v>
       </ns0:c>
-      <ns0:c r="CP3" s="26" t="s">
+      <ns0:c r="CU3" s="26" t="s">
         <ns0:v>160</ns0:v>
       </ns0:c>
-      <ns0:c r="CQ3" s="26" t="s">
+      <ns0:c r="CV3" s="26" t="s">
         <ns0:v>162</ns0:v>
       </ns0:c>
-      <ns0:c r="CR3" s="26" t="s">
+      <ns0:c r="CW3" s="26" t="s">
         <ns0:v>247</ns0:v>
       </ns0:c>
-      <ns0:c r="CS3" s="26" t="s">
+      <ns0:c r="CX3" s="26" t="s">
         <ns0:v>276</ns0:v>
       </ns0:c>
-      <ns0:c r="CT3" s="26" t="s">
+      <ns0:c r="CY3" s="26" t="s">
         <ns0:v>160</ns0:v>
       </ns0:c>
-      <ns0:c r="CU3" s="26" t="s">
+      <ns0:c r="CZ3" s="26" t="s">
         <ns0:v>162</ns0:v>
       </ns0:c>
-      <ns0:c r="CV3" s="26" t="s">
+      <ns0:c r="DA3" s="26" t="s">
         <ns0:v>247</ns0:v>
       </ns0:c>
-      <ns0:c r="CW3" s="26" t="s">
+      <ns0:c r="DB3" s="26" t="s">
         <ns0:v>300</ns0:v>
       </ns0:c>
-      <ns0:c r="CX3" s="26" t="s">
+      <ns0:c r="DC3" s="26" t="s">
         <ns0:v>160</ns0:v>
       </ns0:c>
-      <ns0:c r="CY3" s="26" t="s">
+      <ns0:c r="DD3" s="26" t="s">
         <ns0:v>162</ns0:v>
       </ns0:c>
-      <ns0:c r="CZ3" s="26" t="s">
+      <ns0:c r="DE3" s="26" t="s">
         <ns0:v>247</ns0:v>
       </ns0:c>
-      <ns0:c r="DA3" s="26" t="s">
+      <ns0:c r="DF3" s="26" t="s">
         <ns0:v>300</ns0:v>
       </ns0:c>
-      <ns0:c r="DB3" s="26" t="s">
+      <ns0:c r="DG3" s="26" t="s">
         <ns0:v>160</ns0:v>
       </ns0:c>
-      <ns0:c r="DC3" s="26" t="s">
+      <ns0:c r="DH3" s="26" t="s">
         <ns0:v>162</ns0:v>
       </ns0:c>
-      <ns0:c r="DD3" s="26" t="s">
+      <ns0:c r="DI3" s="26" t="s">
         <ns0:v>247</ns0:v>
       </ns0:c>
-      <ns0:c r="DE3" s="26" t="s">
+      <ns0:c r="DJ3" s="26" t="s">
         <ns0:v>300</ns0:v>
       </ns0:c>
-      <ns0:c r="DF3" s="26" t="s">
+      <ns0:c r="DK3" s="26" t="s">
         <ns0:v>161</ns0:v>
       </ns0:c>
-      <ns0:c r="DG3" s="26" t="s">
+      <ns0:c r="DL3" s="26" t="s">
         <ns0:v>163</ns0:v>
       </ns0:c>
-      <ns0:c r="DH3" s="26" t="s">
+      <ns0:c r="DM3" s="26" t="s">
         <ns0:v>267</ns0:v>
       </ns0:c>
-      <ns0:c r="DI3" s="26" t="s">
+      <ns0:c r="DN3" s="26" t="s">
         <ns0:v>269</ns0:v>
       </ns0:c>
-      <ns0:c r="DJ3" s="26" t="s">
+      <ns0:c r="DO3" s="26" t="s">
         <ns0:v>161</ns0:v>
       </ns0:c>
-      <ns0:c r="DK3" s="26" t="s">
+      <ns0:c r="DP3" s="26" t="s">
         <ns0:v>163</ns0:v>
       </ns0:c>
-      <ns0:c r="DL3" s="26" t="s">
+      <ns0:c r="DQ3" s="26" t="s">
         <ns0:v>267</ns0:v>
       </ns0:c>
-      <ns0:c r="DM3" s="26" t="s">
+      <ns0:c r="DR3" s="26" t="s">
         <ns0:v>269</ns0:v>
       </ns0:c>
-      <ns0:c r="DN3" s="26" t="s">
+      <ns0:c r="DS3" s="26" t="s">
         <ns0:v>165</ns0:v>
       </ns0:c>
-      <ns0:c r="DO3" s="26" t="s">
+      <ns0:c r="DT3" s="26" t="s">
         <ns0:v>164</ns0:v>
       </ns0:c>
-      <ns0:c r="DP3" s="26" t="s">
+      <ns0:c r="DU3" s="26" t="s">
         <ns0:v>271</ns0:v>
       </ns0:c>
-      <ns0:c r="DQ3" s="26" t="s">
+      <ns0:c r="DV3" s="26" t="s">
         <ns0:v>166</ns0:v>
       </ns0:c>
-      <ns0:c r="DR3" s="26" t="s">
+      <ns0:c r="DW3" s="26" t="s">
         <ns0:v>165</ns0:v>
       </ns0:c>
-      <ns0:c r="DS3" s="26" t="s">
+      <ns0:c r="DX3" s="26" t="s">
         <ns0:v>164</ns0:v>
       </ns0:c>
-      <ns0:c r="DT3" s="26" t="s">
+      <ns0:c r="DY3" s="26" t="s">
         <ns0:v>271</ns0:v>
       </ns0:c>
-      <ns0:c r="DU3" s="26" t="s">
+      <ns0:c r="DZ3" s="26" t="s">
         <ns0:v>166</ns0:v>
       </ns0:c>
-      <ns0:c r="DV3" s="26" t="s">
+      <ns0:c r="EA3" s="26" t="s">
         <ns0:v>165</ns0:v>
       </ns0:c>
-      <ns0:c r="DW3" s="26" t="s">
+      <ns0:c r="EB3" s="26" t="s">
         <ns0:v>164</ns0:v>
       </ns0:c>
-      <ns0:c r="DX3" s="26" t="s">
+      <ns0:c r="EC3" s="26" t="s">
         <ns0:v>271</ns0:v>
       </ns0:c>
-      <ns0:c r="DY3" s="26" t="s">
+      <ns0:c r="ED3" s="26" t="s">
         <ns0:v>166</ns0:v>
       </ns0:c>
-      <ns0:c r="EA3" s="61" t="s">
+      <ns0:c r="EE3" t="s">
+        <ns0:v>544</ns0:v>
+      </ns0:c>
+      <ns0:c r="EF3" s="61" t="s">
         <ns0:v>151</ns0:v>
       </ns0:c>
-      <ns0:c r="EB3" s="61" t="s">
+      <ns0:c r="EG3" s="61" t="s">
         <ns0:v>397</ns0:v>
       </ns0:c>
-      <ns0:c r="EC3" s="61" t="s">
+      <ns0:c r="EH3" s="61" t="s">
         <ns0:v>398</ns0:v>
       </ns0:c>
-      <ns0:c r="ED3" s="61" t="s">
+      <ns0:c r="EI3" s="61" t="s">
         <ns0:v>167</ns0:v>
       </ns0:c>
-      <ns0:c r="EE3" s="61" t="s">
+      <ns0:c r="EJ3" s="61" t="s">
         <ns0:v>151</ns0:v>
       </ns0:c>
-      <ns0:c r="EF3" s="61" t="s">
+      <ns0:c r="EK3" s="61" t="s">
         <ns0:v>407</ns0:v>
       </ns0:c>
-      <ns0:c r="EG3" s="61" t="s">
+      <ns0:c r="EL3" s="61" t="s">
         <ns0:v>406</ns0:v>
       </ns0:c>
-      <ns0:c r="EH3" s="61" t="s">
+      <ns0:c r="EM3" s="61" t="s">
         <ns0:v>167</ns0:v>
       </ns0:c>
-      <ns0:c r="EI3" s="25" t="s">
+      <ns0:c r="EN3" s="25" t="s">
         <ns0:v>125</ns0:v>
       </ns0:c>
-      <ns0:c r="EJ3" s="58" t="s">
+      <ns0:c r="EO3" s="58" t="s">
         <ns0:v>227</ns0:v>
       </ns0:c>
-      <ns0:c r="EK3" s="68" t="s">
+      <ns0:c r="EP3" s="68" t="s">
         <ns0:v>428</ns0:v>
       </ns0:c>
-      <ns0:c r="EL3" s="25" t="s">
+      <ns0:c r="EQ3" s="25" t="s">
         <ns0:v>126</ns0:v>
       </ns0:c>
-      <ns0:c r="EM3" s="58" t="s">
+      <ns0:c r="ER3" s="58" t="s">
         <ns0:v>225</ns0:v>
       </ns0:c>
-      <ns0:c r="EN3" s="68" t="s">
+      <ns0:c r="ES3" s="68" t="s">
         <ns0:v>430</ns0:v>
       </ns0:c>
-      <ns0:c r="EO3" s="58" t="s">
+      <ns0:c r="ET3" s="58" t="s">
         <ns0:v>418</ns0:v>
       </ns0:c>
-      <ns0:c r="EP3" s="58" t="s">
+      <ns0:c r="EU3" s="58" t="s">
         <ns0:v>419</ns0:v>
       </ns0:c>
-      <ns0:c r="EQ3" s="68" t="s">
+      <ns0:c r="EV3" s="68" t="s">
         <ns0:v>446</ns0:v>
       </ns0:c>
-      <ns0:c r="ER3" s="25" t="s">
+      <ns0:c r="EW3" s="25" t="s">
         <ns0:v>127</ns0:v>
       </ns0:c>
-      <ns0:c r="ES3" s="58" t="s">
+      <ns0:c r="EX3" s="58" t="s">
         <ns0:v>223</ns0:v>
       </ns0:c>
-      <ns0:c r="ET3" s="68" t="s">
+      <ns0:c r="EY3" s="68" t="s">
         <ns0:v>432</ns0:v>
       </ns0:c>
-      <ns0:c r="EU3" s="25" t="s">
+      <ns0:c r="EZ3" s="25" t="s">
         <ns0:v>128</ns0:v>
       </ns0:c>
-      <ns0:c r="EV3" s="58" t="s">
+      <ns0:c r="FA3" s="58" t="s">
         <ns0:v>221</ns0:v>
       </ns0:c>
-      <ns0:c r="EW3" s="68" t="s">
+      <ns0:c r="FB3" s="68" t="s">
         <ns0:v>434</ns0:v>
       </ns0:c>
-      <ns0:c r="EX3" s="25" t="s">
+      <ns0:c r="FC3" s="25" t="s">
         <ns0:v>129</ns0:v>
       </ns0:c>
-      <ns0:c r="EY3" s="58" t="s">
+      <ns0:c r="FD3" s="58" t="s">
         <ns0:v>219</ns0:v>
       </ns0:c>
-      <ns0:c r="EZ3" s="68" t="s">
+      <ns0:c r="FE3" s="68" t="s">
         <ns0:v>436</ns0:v>
       </ns0:c>
-      <ns0:c r="FA3" s="25" t="s">
+      <ns0:c r="FF3" s="25" t="s">
         <ns0:v>130</ns0:v>
       </ns0:c>
-      <ns0:c r="FB3" s="58" t="s">
+      <ns0:c r="FG3" s="58" t="s">
         <ns0:v>217</ns0:v>
       </ns0:c>
-      <ns0:c r="FC3" s="68" t="s">
+      <ns0:c r="FH3" s="68" t="s">
         <ns0:v>447</ns0:v>
       </ns0:c>
-      <ns0:c r="FD3" s="25" t="s">
+      <ns0:c r="FI3" s="25" t="s">
         <ns0:v>131</ns0:v>
       </ns0:c>
-      <ns0:c r="FE3" s="58" t="s">
+      <ns0:c r="FJ3" s="58" t="s">
         <ns0:v>215</ns0:v>
       </ns0:c>
-      <ns0:c r="FF3" s="68" t="s">
+      <ns0:c r="FK3" s="68" t="s">
         <ns0:v>449</ns0:v>
       </ns0:c>
-      <ns0:c r="FG3" s="25" t="s">
+      <ns0:c r="FL3" s="25" t="s">
         <ns0:v>132</ns0:v>
       </ns0:c>
-      <ns0:c r="FH3" s="58" t="s">
+      <ns0:c r="FM3" s="58" t="s">
         <ns0:v>213</ns0:v>
       </ns0:c>
-      <ns0:c r="FI3" s="68" t="s">
+      <ns0:c r="FN3" s="68" t="s">
         <ns0:v>451</ns0:v>
       </ns0:c>
-      <ns0:c r="FJ3" s="25" t="s">
+      <ns0:c r="FO3" s="25" t="s">
         <ns0:v>133</ns0:v>
       </ns0:c>
-      <ns0:c r="FK3" s="58" t="s">
+      <ns0:c r="FP3" s="58" t="s">
         <ns0:v>211</ns0:v>
       </ns0:c>
-      <ns0:c r="FL3" s="68" t="s">
+      <ns0:c r="FQ3" s="68" t="s">
         <ns0:v>453</ns0:v>
       </ns0:c>
-      <ns0:c r="FM3" s="25" t="s">
+      <ns0:c r="FR3" s="25" t="s">
         <ns0:v>135</ns0:v>
       </ns0:c>
-      <ns0:c r="FN3" s="58" t="s">
+      <ns0:c r="FS3" s="58" t="s">
         <ns0:v>209</ns0:v>
       </ns0:c>
-      <ns0:c r="FO3" s="25" t="s">
+      <ns0:c r="FT3" s="25" t="s">
         <ns0:v>136</ns0:v>
       </ns0:c>
-      <ns0:c r="FP3" s="68" t="s">
+      <ns0:c r="FU3" s="68" t="s">
         <ns0:v>461</ns0:v>
       </ns0:c>
-      <ns0:c r="FQ3" s="58" t="s">
+      <ns0:c r="FV3" s="58" t="s">
         <ns0:v>207</ns0:v>
       </ns0:c>
-      <ns0:c r="FR3" s="68" t="s">
+      <ns0:c r="FW3" s="68" t="s">
         <ns0:v>455</ns0:v>
       </ns0:c>
-      <ns0:c r="FS3" s="25" t="s">
+      <ns0:c r="FX3" s="25" t="s">
         <ns0:v>137</ns0:v>
       </ns0:c>
-      <ns0:c r="FT3" s="58" t="s">
+      <ns0:c r="FY3" s="58" t="s">
         <ns0:v>205</ns0:v>
       </ns0:c>
-      <ns0:c r="FU3" s="68" t="s">
+      <ns0:c r="FZ3" s="68" t="s">
         <ns0:v>457</ns0:v>
       </ns0:c>
-      <ns0:c r="FV3" s="25" t="s">
+      <ns0:c r="GA3" s="25" t="s">
         <ns0:v>138</ns0:v>
       </ns0:c>
-      <ns0:c r="FW3" s="58" t="s">
+      <ns0:c r="GB3" s="58" t="s">
         <ns0:v>204</ns0:v>
       </ns0:c>
-      <ns0:c r="FX3" s="68" t="s">
+      <ns0:c r="GC3" s="68" t="s">
         <ns0:v>438</ns0:v>
       </ns0:c>
-      <ns0:c r="FY3" s="25" t="s">
+      <ns0:c r="GD3" s="25" t="s">
         <ns0:v>139</ns0:v>
       </ns0:c>
-      <ns0:c r="FZ3" s="58" t="s">
+      <ns0:c r="GE3" s="58" t="s">
         <ns0:v>200</ns0:v>
       </ns0:c>
-      <ns0:c r="GA3" s="68" t="s">
+      <ns0:c r="GF3" s="68" t="s">
         <ns0:v>440</ns0:v>
       </ns0:c>
-      <ns0:c r="GB3" s="25" t="s">
+      <ns0:c r="GG3" s="25" t="s">
         <ns0:v>141</ns0:v>
       </ns0:c>
-      <ns0:c r="GC3" s="58" t="s">
+      <ns0:c r="GH3" s="58" t="s">
         <ns0:v>199</ns0:v>
       </ns0:c>
-      <ns0:c r="GD3" s="68" t="s">
+      <ns0:c r="GI3" s="68" t="s">
         <ns0:v>442</ns0:v>
       </ns0:c>
-      <ns0:c r="GE3" s="25" t="s">
+      <ns0:c r="GJ3" s="25" t="s">
         <ns0:v>143</ns0:v>
       </ns0:c>
-      <ns0:c r="GF3" s="58" t="s">
+      <ns0:c r="GK3" s="58" t="s">
         <ns0:v>197</ns0:v>
       </ns0:c>
-      <ns0:c r="GG3" s="68" t="s">
+      <ns0:c r="GL3" s="68" t="s">
         <ns0:v>444</ns0:v>
       </ns0:c>
-      <ns0:c r="GH3" s="25" t="s">
+      <ns0:c r="GM3" s="25" t="s">
         <ns0:v>145</ns0:v>
       </ns0:c>
-      <ns0:c r="GI3" s="58" t="s">
+      <ns0:c r="GN3" s="58" t="s">
         <ns0:v>195</ns0:v>
       </ns0:c>
-      <ns0:c r="GJ3" s="68" t="s">
+      <ns0:c r="GO3" s="68" t="s">
         <ns0:v>459</ns0:v>
       </ns0:c>
-      <ns0:c r="GK3" s="68" t="s">
+      <ns0:c r="GP3" s="68" t="s">
         <ns0:v>520</ns0:v>
       </ns0:c>
-      <ns0:c r="GL3" s="68" t="s">
+      <ns0:c r="GQ3" s="68" t="s">
         <ns0:v>521</ns0:v>
       </ns0:c>
-      <ns0:c r="DZ3" t="s">
-        <ns0:v>544</ns0:v>
-      </ns0:c>
     </ns0:row>
-    <ns0:row r="4" spans="1:193" s="59" customFormat="1" ht="56.25" customHeight="1" thickTop="1" thickBot="1" ns3:dyDescent="0.25">
+    <ns0:row r="4" spans="1:198" s="59" customFormat="1" ht="56.25" customHeight="1" thickTop="1" thickBot="1" ns3:dyDescent="0.25">
       <ns0:c r="A4" s="35" t="s">
         <ns0:v>5</ns0:v>
       </ns0:c>
@@ -4177,385 +4546,400 @@
         <ns0:v>424</ns0:v>
       </ns0:c>
       <ns0:c r="BQ4" s="69" t="s">
-        <ns0:v>484</ns0:v>
+        <ns0:v>597</ns0:v>
       </ns0:c>
       <ns0:c r="BR4" s="69" t="s">
-        <ns0:v>485</ns0:v>
+        <ns0:v>598</ns0:v>
       </ns0:c>
       <ns0:c r="BS4" s="69" t="s">
-        <ns0:v>486</ns0:v>
+        <ns0:v>599</ns0:v>
       </ns0:c>
       <ns0:c r="BT4" s="69" t="s">
-        <ns0:v>487</ns0:v>
+        <ns0:v>600</ns0:v>
       </ns0:c>
       <ns0:c r="BU4" s="69" t="s">
-        <ns0:v>488</ns0:v>
+        <ns0:v>601</ns0:v>
       </ns0:c>
       <ns0:c r="BV4" s="69" t="s">
-        <ns0:v>489</ns0:v>
+        <ns0:v>602</ns0:v>
       </ns0:c>
       <ns0:c r="BW4" s="69" t="s">
-        <ns0:v>490</ns0:v>
+        <ns0:v>603</ns0:v>
       </ns0:c>
       <ns0:c r="BX4" s="69" t="s">
-        <ns0:v>491</ns0:v>
+        <ns0:v>604</ns0:v>
       </ns0:c>
       <ns0:c r="BY4" s="69" t="s">
-        <ns0:v>492</ns0:v>
+        <ns0:v>605</ns0:v>
       </ns0:c>
       <ns0:c r="BZ4" s="69" t="s">
-        <ns0:v>493</ns0:v>
+        <ns0:v>606</ns0:v>
       </ns0:c>
       <ns0:c r="CA4" s="69" t="s">
-        <ns0:v>494</ns0:v>
+        <ns0:v>607</ns0:v>
       </ns0:c>
       <ns0:c r="CB4" s="69" t="s">
-        <ns0:v>495</ns0:v>
+        <ns0:v>608</ns0:v>
       </ns0:c>
       <ns0:c r="CC4" s="69" t="s">
-        <ns0:v>496</ns0:v>
+        <ns0:v>609</ns0:v>
       </ns0:c>
       <ns0:c r="CD4" s="69" t="s">
-        <ns0:v>497</ns0:v>
+        <ns0:v>610</ns0:v>
       </ns0:c>
       <ns0:c r="CE4" s="69" t="s">
-        <ns0:v>498</ns0:v>
+        <ns0:v>611</ns0:v>
       </ns0:c>
       <ns0:c r="CF4" s="69" t="s">
-        <ns0:v>499</ns0:v>
+        <ns0:v>612</ns0:v>
       </ns0:c>
       <ns0:c r="CG4" s="69" t="s">
-        <ns0:v>500</ns0:v>
+        <ns0:v>613</ns0:v>
       </ns0:c>
       <ns0:c r="CH4" s="69" t="s">
-        <ns0:v>501</ns0:v>
+        <ns0:v>614</ns0:v>
       </ns0:c>
       <ns0:c r="CI4" s="69" t="s">
-        <ns0:v>502</ns0:v>
+        <ns0:v>615</ns0:v>
       </ns0:c>
       <ns0:c r="CJ4" s="69" t="s">
-        <ns0:v>503</ns0:v>
+        <ns0:v>616</ns0:v>
       </ns0:c>
       <ns0:c r="CK4" s="69" t="s">
-        <ns0:v>504</ns0:v>
-      </ns0:c>
-      <ns0:c r="CL4" s="37" t="s">
+        <ns0:v>617</ns0:v>
+      </ns0:c>
+      <ns0:c r="CL4" s="69" t="s">
+        <ns0:v>618</ns0:v>
+      </ns0:c>
+      <ns0:c r="CM4" s="69" t="s">
+        <ns0:v>619</ns0:v>
+      </ns0:c>
+      <ns0:c r="CN4" s="69" t="s">
+        <ns0:v>620</ns0:v>
+      </ns0:c>
+      <ns0:c r="CO4" s="69" t="s">
+        <ns0:v>621</ns0:v>
+      </ns0:c>
+      <ns0:c r="CP4" s="69" t="s">
+        <ns0:v>622</ns0:v>
+      </ns0:c>
+      <ns0:c r="CQ4" s="37" t="s">
         <ns0:v>184</ns0:v>
       </ns0:c>
-      <ns0:c r="CM4" s="37" t="s">
+      <ns0:c r="CR4" s="37" t="s">
         <ns0:v>168</ns0:v>
       </ns0:c>
-      <ns0:c r="CN4" s="37" t="s">
+      <ns0:c r="CS4" s="37" t="s">
         <ns0:v>248</ns0:v>
       </ns0:c>
-      <ns0:c r="CO4" s="37" t="s">
+      <ns0:c r="CT4" s="37" t="s">
         <ns0:v>169</ns0:v>
       </ns0:c>
-      <ns0:c r="CP4" s="37" t="s">
+      <ns0:c r="CU4" s="37" t="s">
         <ns0:v>170</ns0:v>
       </ns0:c>
-      <ns0:c r="CQ4" s="37" t="s">
+      <ns0:c r="CV4" s="37" t="s">
         <ns0:v>171</ns0:v>
       </ns0:c>
-      <ns0:c r="CR4" s="37" t="s">
+      <ns0:c r="CW4" s="37" t="s">
         <ns0:v>262</ns0:v>
       </ns0:c>
-      <ns0:c r="CS4" s="37" t="s">
+      <ns0:c r="CX4" s="37" t="s">
         <ns0:v>172</ns0:v>
       </ns0:c>
-      <ns0:c r="CT4" s="37" t="s">
+      <ns0:c r="CY4" s="37" t="s">
         <ns0:v>173</ns0:v>
       </ns0:c>
-      <ns0:c r="CU4" s="37" t="s">
+      <ns0:c r="CZ4" s="37" t="s">
         <ns0:v>174</ns0:v>
       </ns0:c>
-      <ns0:c r="CV4" s="37" t="s">
+      <ns0:c r="DA4" s="37" t="s">
         <ns0:v>265</ns0:v>
       </ns0:c>
-      <ns0:c r="CW4" s="37" t="s">
+      <ns0:c r="DB4" s="37" t="s">
         <ns0:v>175</ns0:v>
       </ns0:c>
-      <ns0:c r="CX4" s="37" t="s">
+      <ns0:c r="DC4" s="37" t="s">
         <ns0:v>301</ns0:v>
       </ns0:c>
-      <ns0:c r="CY4" s="37" t="s">
+      <ns0:c r="DD4" s="37" t="s">
         <ns0:v>303</ns0:v>
       </ns0:c>
-      <ns0:c r="CZ4" s="37" t="s">
+      <ns0:c r="DE4" s="37" t="s">
         <ns0:v>305</ns0:v>
       </ns0:c>
-      <ns0:c r="DA4" s="37" t="s">
+      <ns0:c r="DF4" s="37" t="s">
         <ns0:v>307</ns0:v>
       </ns0:c>
-      <ns0:c r="DB4" s="37" t="s">
+      <ns0:c r="DG4" s="37" t="s">
         <ns0:v>309</ns0:v>
       </ns0:c>
-      <ns0:c r="DC4" s="37" t="s">
+      <ns0:c r="DH4" s="37" t="s">
         <ns0:v>311</ns0:v>
       </ns0:c>
-      <ns0:c r="DD4" s="37" t="s">
+      <ns0:c r="DI4" s="37" t="s">
         <ns0:v>313</ns0:v>
       </ns0:c>
-      <ns0:c r="DE4" s="37" t="s">
+      <ns0:c r="DJ4" s="37" t="s">
         <ns0:v>315</ns0:v>
       </ns0:c>
-      <ns0:c r="DF4" s="37" t="s">
+      <ns0:c r="DK4" s="37" t="s">
         <ns0:v>185</ns0:v>
       </ns0:c>
-      <ns0:c r="DG4" s="37" t="s">
+      <ns0:c r="DL4" s="37" t="s">
         <ns0:v>186</ns0:v>
       </ns0:c>
-      <ns0:c r="DH4" s="37" t="s">
+      <ns0:c r="DM4" s="37" t="s">
         <ns0:v>268</ns0:v>
       </ns0:c>
-      <ns0:c r="DI4" s="37" t="s">
+      <ns0:c r="DN4" s="37" t="s">
         <ns0:v>187</ns0:v>
       </ns0:c>
-      <ns0:c r="DJ4" s="37" t="s">
+      <ns0:c r="DO4" s="37" t="s">
         <ns0:v>281</ns0:v>
       </ns0:c>
-      <ns0:c r="DK4" s="37" t="s">
+      <ns0:c r="DP4" s="37" t="s">
         <ns0:v>284</ns0:v>
       </ns0:c>
-      <ns0:c r="DL4" s="37" t="s">
+      <ns0:c r="DQ4" s="37" t="s">
         <ns0:v>286</ns0:v>
       </ns0:c>
-      <ns0:c r="DM4" s="37" t="s">
+      <ns0:c r="DR4" s="37" t="s">
         <ns0:v>288</ns0:v>
       </ns0:c>
-      <ns0:c r="DN4" s="37" t="s">
+      <ns0:c r="DS4" s="37" t="s">
         <ns0:v>176</ns0:v>
       </ns0:c>
-      <ns0:c r="DO4" s="37" t="s">
+      <ns0:c r="DT4" s="37" t="s">
         <ns0:v>177</ns0:v>
       </ns0:c>
-      <ns0:c r="DP4" s="37" t="s">
+      <ns0:c r="DU4" s="37" t="s">
         <ns0:v>272</ns0:v>
       </ns0:c>
-      <ns0:c r="DQ4" s="37" t="s">
+      <ns0:c r="DV4" s="37" t="s">
         <ns0:v>178</ns0:v>
       </ns0:c>
-      <ns0:c r="DR4" s="37" t="s">
+      <ns0:c r="DW4" s="37" t="s">
         <ns0:v>179</ns0:v>
       </ns0:c>
-      <ns0:c r="DS4" s="37" t="s">
+      <ns0:c r="DX4" s="37" t="s">
         <ns0:v>181</ns0:v>
       </ns0:c>
-      <ns0:c r="DT4" s="37" t="s">
+      <ns0:c r="DY4" s="37" t="s">
         <ns0:v>273</ns0:v>
       </ns0:c>
-      <ns0:c r="DU4" s="37" t="s">
+      <ns0:c r="DZ4" s="37" t="s">
         <ns0:v>180</ns0:v>
       </ns0:c>
-      <ns0:c r="DV4" s="37" t="s">
+      <ns0:c r="EA4" s="37" t="s">
         <ns0:v>292</ns0:v>
       </ns0:c>
-      <ns0:c r="DW4" s="37" t="s">
+      <ns0:c r="EB4" s="37" t="s">
         <ns0:v>294</ns0:v>
       </ns0:c>
-      <ns0:c r="DX4" s="37" t="s">
+      <ns0:c r="EC4" s="37" t="s">
         <ns0:v>296</ns0:v>
       </ns0:c>
-      <ns0:c r="DY4" s="37" t="s">
+      <ns0:c r="ED4" s="37" t="s">
         <ns0:v>298</ns0:v>
       </ns0:c>
-      <ns0:c r="EA4" s="37" t="s">
+      <ns0:c r="EE4" t="s">
+        <ns0:v>541</ns0:v>
+      </ns0:c>
+      <ns0:c r="EF4" s="37" t="s">
         <ns0:v>152</ns0:v>
       </ns0:c>
-      <ns0:c r="EB4" s="37" t="s">
+      <ns0:c r="EG4" s="37" t="s">
         <ns0:v>109</ns0:v>
       </ns0:c>
-      <ns0:c r="EC4" s="37" t="s">
+      <ns0:c r="EH4" s="37" t="s">
         <ns0:v>110</ns0:v>
       </ns0:c>
-      <ns0:c r="ED4" s="37" t="s">
+      <ns0:c r="EI4" s="37" t="s">
         <ns0:v>154</ns0:v>
       </ns0:c>
-      <ns0:c r="EE4" s="37" t="s">
+      <ns0:c r="EJ4" s="37" t="s">
         <ns0:v>153</ns0:v>
       </ns0:c>
-      <ns0:c r="EF4" s="37" t="s">
+      <ns0:c r="EK4" s="37" t="s">
         <ns0:v>111</ns0:v>
       </ns0:c>
-      <ns0:c r="EG4" s="37" t="s">
+      <ns0:c r="EL4" s="37" t="s">
         <ns0:v>112</ns0:v>
       </ns0:c>
-      <ns0:c r="EH4" s="37" t="s">
+      <ns0:c r="EM4" s="37" t="s">
         <ns0:v>155</ns0:v>
       </ns0:c>
-      <ns0:c r="EI4" s="37" t="s">
+      <ns0:c r="EN4" s="37" t="s">
         <ns0:v>45</ns0:v>
       </ns0:c>
-      <ns0:c r="EJ4" s="37" t="s">
+      <ns0:c r="EO4" s="37" t="s">
         <ns0:v>229</ns0:v>
       </ns0:c>
-      <ns0:c r="EK4" s="69" t="s">
+      <ns0:c r="EP4" s="69" t="s">
         <ns0:v>429</ns0:v>
       </ns0:c>
-      <ns0:c r="EL4" s="37" t="s">
+      <ns0:c r="EQ4" s="37" t="s">
         <ns0:v>49</ns0:v>
       </ns0:c>
-      <ns0:c r="EM4" s="37" t="s">
+      <ns0:c r="ER4" s="37" t="s">
         <ns0:v>230</ns0:v>
       </ns0:c>
-      <ns0:c r="EN4" s="69" t="s">
+      <ns0:c r="ES4" s="69" t="s">
         <ns0:v>431</ns0:v>
       </ns0:c>
-      <ns0:c r="EO4" s="37" t="s">
+      <ns0:c r="ET4" s="37" t="s">
         <ns0:v>420</ns0:v>
       </ns0:c>
-      <ns0:c r="EP4" s="37" t="s">
+      <ns0:c r="EU4" s="37" t="s">
         <ns0:v>421</ns0:v>
       </ns0:c>
-      <ns0:c r="EQ4" s="69" t="s">
+      <ns0:c r="EV4" s="69" t="s">
         <ns0:v>522</ns0:v>
       </ns0:c>
-      <ns0:c r="ER4" s="40" t="s">
+      <ns0:c r="EW4" s="40" t="s">
         <ns0:v>52</ns0:v>
       </ns0:c>
-      <ns0:c r="ES4" s="37" t="s">
+      <ns0:c r="EX4" s="37" t="s">
         <ns0:v>231</ns0:v>
       </ns0:c>
-      <ns0:c r="ET4" s="69" t="s">
+      <ns0:c r="EY4" s="69" t="s">
         <ns0:v>433</ns0:v>
       </ns0:c>
-      <ns0:c r="EU4" s="37" t="s">
+      <ns0:c r="EZ4" s="37" t="s">
         <ns0:v>47</ns0:v>
       </ns0:c>
-      <ns0:c r="EV4" s="37" t="s">
+      <ns0:c r="FA4" s="37" t="s">
         <ns0:v>232</ns0:v>
       </ns0:c>
-      <ns0:c r="EW4" s="69" t="s">
+      <ns0:c r="FB4" s="69" t="s">
         <ns0:v>435</ns0:v>
       </ns0:c>
-      <ns0:c r="EX4" s="37" t="s">
+      <ns0:c r="FC4" s="37" t="s">
         <ns0:v>48</ns0:v>
       </ns0:c>
-      <ns0:c r="EY4" s="37" t="s">
+      <ns0:c r="FD4" s="37" t="s">
         <ns0:v>233</ns0:v>
       </ns0:c>
-      <ns0:c r="EZ4" s="69" t="s">
+      <ns0:c r="FE4" s="69" t="s">
         <ns0:v>437</ns0:v>
       </ns0:c>
-      <ns0:c r="FA4" s="40" t="s">
+      <ns0:c r="FF4" s="40" t="s">
         <ns0:v>51</ns0:v>
       </ns0:c>
-      <ns0:c r="FB4" s="37" t="s">
+      <ns0:c r="FG4" s="37" t="s">
         <ns0:v>234</ns0:v>
       </ns0:c>
-      <ns0:c r="FC4" s="69" t="s">
+      <ns0:c r="FH4" s="69" t="s">
         <ns0:v>448</ns0:v>
       </ns0:c>
-      <ns0:c r="FD4" s="40" t="s">
+      <ns0:c r="FI4" s="40" t="s">
         <ns0:v>102</ns0:v>
       </ns0:c>
-      <ns0:c r="FE4" s="37" t="s">
+      <ns0:c r="FJ4" s="37" t="s">
         <ns0:v>235</ns0:v>
       </ns0:c>
-      <ns0:c r="FF4" s="69" t="s">
+      <ns0:c r="FK4" s="69" t="s">
         <ns0:v>450</ns0:v>
       </ns0:c>
-      <ns0:c r="FG4" s="40" t="s">
+      <ns0:c r="FL4" s="40" t="s">
         <ns0:v>55</ns0:v>
       </ns0:c>
-      <ns0:c r="FH4" s="37" t="s">
+      <ns0:c r="FM4" s="37" t="s">
         <ns0:v>236</ns0:v>
       </ns0:c>
-      <ns0:c r="FI4" s="69" t="s">
+      <ns0:c r="FN4" s="69" t="s">
         <ns0:v>452</ns0:v>
       </ns0:c>
-      <ns0:c r="FJ4" s="37" t="s">
+      <ns0:c r="FO4" s="37" t="s">
         <ns0:v>50</ns0:v>
       </ns0:c>
-      <ns0:c r="FK4" s="37" t="s">
+      <ns0:c r="FP4" s="37" t="s">
         <ns0:v>238</ns0:v>
       </ns0:c>
-      <ns0:c r="FL4" s="69" t="s">
+      <ns0:c r="FQ4" s="69" t="s">
         <ns0:v>454</ns0:v>
       </ns0:c>
-      <ns0:c r="FM4" s="37" t="s">
+      <ns0:c r="FR4" s="37" t="s">
         <ns0:v>103</ns0:v>
       </ns0:c>
-      <ns0:c r="FN4" s="37" t="s">
+      <ns0:c r="FS4" s="37" t="s">
         <ns0:v>239</ns0:v>
       </ns0:c>
-      <ns0:c r="FO4" s="37" t="s">
+      <ns0:c r="FT4" s="37" t="s">
         <ns0:v>104</ns0:v>
       </ns0:c>
-      <ns0:c r="FP4" s="69" t="s">
+      <ns0:c r="FU4" s="69" t="s">
         <ns0:v>462</ns0:v>
       </ns0:c>
-      <ns0:c r="FQ4" s="37" t="s">
+      <ns0:c r="FV4" s="37" t="s">
         <ns0:v>240</ns0:v>
       </ns0:c>
-      <ns0:c r="FR4" s="69" t="s">
+      <ns0:c r="FW4" s="69" t="s">
         <ns0:v>456</ns0:v>
       </ns0:c>
-      <ns0:c r="FS4" s="40" t="s">
+      <ns0:c r="FX4" s="40" t="s">
         <ns0:v>77</ns0:v>
       </ns0:c>
-      <ns0:c r="FT4" s="37" t="s">
+      <ns0:c r="FY4" s="37" t="s">
         <ns0:v>241</ns0:v>
       </ns0:c>
-      <ns0:c r="FU4" s="69" t="s">
+      <ns0:c r="FZ4" s="69" t="s">
         <ns0:v>458</ns0:v>
       </ns0:c>
-      <ns0:c r="FV4" s="37" t="s">
+      <ns0:c r="GA4" s="37" t="s">
         <ns0:v>46</ns0:v>
       </ns0:c>
-      <ns0:c r="FW4" s="37" t="s">
+      <ns0:c r="GB4" s="37" t="s">
         <ns0:v>242</ns0:v>
       </ns0:c>
-      <ns0:c r="FX4" s="69" t="s">
+      <ns0:c r="GC4" s="69" t="s">
         <ns0:v>439</ns0:v>
       </ns0:c>
-      <ns0:c r="FY4" s="40" t="s">
+      <ns0:c r="GD4" s="40" t="s">
         <ns0:v>57</ns0:v>
       </ns0:c>
-      <ns0:c r="FZ4" s="37" t="s">
+      <ns0:c r="GE4" s="37" t="s">
         <ns0:v>243</ns0:v>
       </ns0:c>
-      <ns0:c r="GA4" s="69" t="s">
+      <ns0:c r="GF4" s="69" t="s">
         <ns0:v>441</ns0:v>
       </ns0:c>
-      <ns0:c r="GB4" s="37" t="s">
+      <ns0:c r="GG4" s="37" t="s">
         <ns0:v>76</ns0:v>
       </ns0:c>
-      <ns0:c r="GC4" s="37" t="s">
+      <ns0:c r="GH4" s="37" t="s">
         <ns0:v>244</ns0:v>
       </ns0:c>
-      <ns0:c r="GD4" s="69" t="s">
+      <ns0:c r="GI4" s="69" t="s">
         <ns0:v>443</ns0:v>
       </ns0:c>
-      <ns0:c r="GE4" s="40" t="s">
+      <ns0:c r="GJ4" s="40" t="s">
         <ns0:v>56</ns0:v>
       </ns0:c>
-      <ns0:c r="GF4" s="40" t="s">
+      <ns0:c r="GK4" s="40" t="s">
         <ns0:v>245</ns0:v>
       </ns0:c>
-      <ns0:c r="GG4" s="69" t="s">
+      <ns0:c r="GL4" s="69" t="s">
         <ns0:v>445</ns0:v>
       </ns0:c>
-      <ns0:c r="GH4" s="40" t="s">
+      <ns0:c r="GM4" s="40" t="s">
         <ns0:v>54</ns0:v>
       </ns0:c>
-      <ns0:c r="GI4" s="37" t="s">
+      <ns0:c r="GN4" s="37" t="s">
         <ns0:v>246</ns0:v>
       </ns0:c>
-      <ns0:c r="GJ4" s="69" t="s">
+      <ns0:c r="GO4" s="69" t="s">
         <ns0:v>460</ns0:v>
       </ns0:c>
-      <ns0:c r="GK4" s="69" t="s">
+      <ns0:c r="GP4" s="69" t="s">
         <ns0:v>518</ns0:v>
       </ns0:c>
-      <ns0:c r="GL4" s="69" t="s">
+      <ns0:c r="GQ4" s="69" t="s">
         <ns0:v>519</ns0:v>
       </ns0:c>
-      <ns0:c r="DZ4" t="s">
-        <ns0:v>541</ns0:v>
-      </ns0:c>
     </ns0:row>
-    <ns0:row r="5" spans="1:193" ht="57.5" customHeight="1" thickTop="1" thickBot="1" ns3:dyDescent="0.25">
+    <ns0:row r="5" spans="1:198" ht="57.5" customHeight="1" thickTop="1" thickBot="1" ns3:dyDescent="0.25">
       <ns0:c r="A5" s="34" t="s">
         <ns0:v>60</ns0:v>
       </ns0:c>
@@ -4761,385 +5145,400 @@
         <ns0:v>416</ns0:v>
       </ns0:c>
       <ns0:c r="BQ5" s="4" t="s">
-        <ns0:v>505</ns0:v>
+        <ns0:v>623</ns0:v>
       </ns0:c>
       <ns0:c r="BR5" s="4" t="s">
-        <ns0:v>506</ns0:v>
+        <ns0:v>624</ns0:v>
       </ns0:c>
       <ns0:c r="BS5" s="4" t="s">
-        <ns0:v>507</ns0:v>
+        <ns0:v>625</ns0:v>
       </ns0:c>
       <ns0:c r="BT5" s="4" t="s">
-        <ns0:v>508</ns0:v>
+        <ns0:v>626</ns0:v>
       </ns0:c>
       <ns0:c r="BU5" s="4" t="s">
-        <ns0:v>509</ns0:v>
+        <ns0:v>627</ns0:v>
       </ns0:c>
       <ns0:c r="BV5" s="4" t="s">
-        <ns0:v>510</ns0:v>
+        <ns0:v>628</ns0:v>
       </ns0:c>
       <ns0:c r="BW5" s="4" t="s">
-        <ns0:v>511</ns0:v>
+        <ns0:v>629</ns0:v>
       </ns0:c>
       <ns0:c r="BX5" s="4" t="s">
-        <ns0:v>512</ns0:v>
+        <ns0:v>630</ns0:v>
       </ns0:c>
       <ns0:c r="BY5" s="4" t="s">
-        <ns0:v>513</ns0:v>
+        <ns0:v>631</ns0:v>
       </ns0:c>
       <ns0:c r="BZ5" s="4" t="s">
-        <ns0:v>514</ns0:v>
+        <ns0:v>632</ns0:v>
       </ns0:c>
       <ns0:c r="CA5" s="4" t="s">
-        <ns0:v>515</ns0:v>
+        <ns0:v>633</ns0:v>
       </ns0:c>
       <ns0:c r="CB5" s="4" t="s">
-        <ns0:v>417</ns0:v>
+        <ns0:v>634</ns0:v>
       </ns0:c>
       <ns0:c r="CC5" s="4" t="s">
-        <ns0:v>506</ns0:v>
+        <ns0:v>635</ns0:v>
       </ns0:c>
       <ns0:c r="CD5" s="4" t="s">
-        <ns0:v>507</ns0:v>
+        <ns0:v>636</ns0:v>
       </ns0:c>
       <ns0:c r="CE5" s="4" t="s">
-        <ns0:v>508</ns0:v>
+        <ns0:v>637</ns0:v>
       </ns0:c>
       <ns0:c r="CF5" s="4" t="s">
-        <ns0:v>509</ns0:v>
+        <ns0:v>638</ns0:v>
       </ns0:c>
       <ns0:c r="CG5" s="4" t="s">
-        <ns0:v>510</ns0:v>
+        <ns0:v>639</ns0:v>
       </ns0:c>
       <ns0:c r="CH5" s="4" t="s">
-        <ns0:v>511</ns0:v>
+        <ns0:v>640</ns0:v>
       </ns0:c>
       <ns0:c r="CI5" s="4" t="s">
-        <ns0:v>512</ns0:v>
+        <ns0:v>641</ns0:v>
       </ns0:c>
       <ns0:c r="CJ5" s="4" t="s">
-        <ns0:v>513</ns0:v>
+        <ns0:v>642</ns0:v>
       </ns0:c>
       <ns0:c r="CK5" s="4" t="s">
-        <ns0:v>514</ns0:v>
+        <ns0:v>643</ns0:v>
       </ns0:c>
       <ns0:c r="CL5" s="4" t="s">
+        <ns0:v>644</ns0:v>
+      </ns0:c>
+      <ns0:c r="CM5" s="4" t="s">
+        <ns0:v>645</ns0:v>
+      </ns0:c>
+      <ns0:c r="CN5" s="4" t="s">
+        <ns0:v>646</ns0:v>
+      </ns0:c>
+      <ns0:c r="CO5" s="4" t="s">
+        <ns0:v>647</ns0:v>
+      </ns0:c>
+      <ns0:c r="CP5" s="4" t="s">
+        <ns0:v>648</ns0:v>
+      </ns0:c>
+      <ns0:c r="CQ5" s="4" t="s">
         <ns0:v>249</ns0:v>
       </ns0:c>
-      <ns0:c r="CM5" s="4" t="s">
+      <ns0:c r="CR5" s="4" t="s">
         <ns0:v>256</ns0:v>
       </ns0:c>
-      <ns0:c r="CN5" s="4" t="s">
+      <ns0:c r="CS5" s="4" t="s">
         <ns0:v>263</ns0:v>
       </ns0:c>
-      <ns0:c r="CO5" s="4" t="s">
+      <ns0:c r="CT5" s="4" t="s">
         <ns0:v>258</ns0:v>
       </ns0:c>
-      <ns0:c r="CP5" s="4" t="s">
+      <ns0:c r="CU5" s="4" t="s">
         <ns0:v>250</ns0:v>
       </ns0:c>
-      <ns0:c r="CQ5" s="4" t="s">
+      <ns0:c r="CV5" s="4" t="s">
         <ns0:v>251</ns0:v>
       </ns0:c>
-      <ns0:c r="CR5" s="4" t="s">
+      <ns0:c r="CW5" s="4" t="s">
         <ns0:v>264</ns0:v>
       </ns0:c>
-      <ns0:c r="CS5" s="4" t="s">
+      <ns0:c r="CX5" s="4" t="s">
         <ns0:v>252</ns0:v>
       </ns0:c>
-      <ns0:c r="CT5" s="4" t="s">
+      <ns0:c r="CY5" s="4" t="s">
         <ns0:v>253</ns0:v>
       </ns0:c>
-      <ns0:c r="CU5" s="4" t="s">
+      <ns0:c r="CZ5" s="4" t="s">
         <ns0:v>254</ns0:v>
       </ns0:c>
-      <ns0:c r="CV5" s="4" t="s">
+      <ns0:c r="DA5" s="4" t="s">
         <ns0:v>266</ns0:v>
       </ns0:c>
-      <ns0:c r="CW5" s="4" t="s">
+      <ns0:c r="DB5" s="4" t="s">
         <ns0:v>255</ns0:v>
       </ns0:c>
-      <ns0:c r="CX5" s="4" t="s">
+      <ns0:c r="DC5" s="4" t="s">
         <ns0:v>302</ns0:v>
       </ns0:c>
-      <ns0:c r="CY5" s="4" t="s">
+      <ns0:c r="DD5" s="4" t="s">
         <ns0:v>304</ns0:v>
       </ns0:c>
-      <ns0:c r="CZ5" s="4" t="s">
+      <ns0:c r="DE5" s="4" t="s">
         <ns0:v>306</ns0:v>
       </ns0:c>
-      <ns0:c r="DA5" s="4" t="s">
+      <ns0:c r="DF5" s="4" t="s">
         <ns0:v>308</ns0:v>
       </ns0:c>
-      <ns0:c r="DB5" s="4" t="s">
+      <ns0:c r="DG5" s="4" t="s">
         <ns0:v>310</ns0:v>
       </ns0:c>
-      <ns0:c r="DC5" s="4" t="s">
+      <ns0:c r="DH5" s="4" t="s">
         <ns0:v>312</ns0:v>
       </ns0:c>
-      <ns0:c r="DD5" s="4" t="s">
+      <ns0:c r="DI5" s="4" t="s">
         <ns0:v>314</ns0:v>
       </ns0:c>
-      <ns0:c r="DE5" s="4" t="s">
+      <ns0:c r="DJ5" s="4" t="s">
         <ns0:v>316</ns0:v>
       </ns0:c>
-      <ns0:c r="DF5" s="4" t="s">
+      <ns0:c r="DK5" s="4" t="s">
         <ns0:v>277</ns0:v>
       </ns0:c>
-      <ns0:c r="DG5" s="4" t="s">
+      <ns0:c r="DL5" s="4" t="s">
         <ns0:v>278</ns0:v>
       </ns0:c>
-      <ns0:c r="DH5" s="4" t="s">
+      <ns0:c r="DM5" s="4" t="s">
         <ns0:v>279</ns0:v>
       </ns0:c>
-      <ns0:c r="DI5" s="4" t="s">
+      <ns0:c r="DN5" s="4" t="s">
         <ns0:v>280</ns0:v>
       </ns0:c>
-      <ns0:c r="DJ5" s="4" t="s">
+      <ns0:c r="DO5" s="4" t="s">
         <ns0:v>283</ns0:v>
       </ns0:c>
-      <ns0:c r="DK5" s="4" t="s">
+      <ns0:c r="DP5" s="4" t="s">
         <ns0:v>285</ns0:v>
       </ns0:c>
-      <ns0:c r="DL5" s="4" t="s">
+      <ns0:c r="DQ5" s="4" t="s">
         <ns0:v>287</ns0:v>
       </ns0:c>
-      <ns0:c r="DM5" s="4" t="s">
+      <ns0:c r="DR5" s="4" t="s">
         <ns0:v>282</ns0:v>
       </ns0:c>
-      <ns0:c r="DN5" s="4" t="s">
+      <ns0:c r="DS5" s="4" t="s">
         <ns0:v>289</ns0:v>
       </ns0:c>
-      <ns0:c r="DO5" s="4" t="s">
+      <ns0:c r="DT5" s="4" t="s">
         <ns0:v>290</ns0:v>
       </ns0:c>
-      <ns0:c r="DP5" s="4" t="s">
+      <ns0:c r="DU5" s="4" t="s">
         <ns0:v>291</ns0:v>
       </ns0:c>
-      <ns0:c r="DQ5" s="4" t="s">
+      <ns0:c r="DV5" s="4" t="s">
         <ns0:v>270</ns0:v>
       </ns0:c>
-      <ns0:c r="DR5" s="4" t="s">
+      <ns0:c r="DW5" s="4" t="s">
         <ns0:v>182</ns0:v>
       </ns0:c>
-      <ns0:c r="DS5" s="4" t="s">
+      <ns0:c r="DX5" s="4" t="s">
         <ns0:v>183</ns0:v>
       </ns0:c>
-      <ns0:c r="DT5" s="4" t="s">
+      <ns0:c r="DY5" s="4" t="s">
         <ns0:v>274</ns0:v>
       </ns0:c>
-      <ns0:c r="DU5" s="4" t="s">
+      <ns0:c r="DZ5" s="4" t="s">
         <ns0:v>257</ns0:v>
       </ns0:c>
-      <ns0:c r="DV5" s="4" t="s">
+      <ns0:c r="EA5" s="4" t="s">
         <ns0:v>293</ns0:v>
       </ns0:c>
-      <ns0:c r="DW5" s="4" t="s">
+      <ns0:c r="EB5" s="4" t="s">
         <ns0:v>295</ns0:v>
       </ns0:c>
-      <ns0:c r="DX5" s="4" t="s">
+      <ns0:c r="EC5" s="4" t="s">
         <ns0:v>297</ns0:v>
       </ns0:c>
-      <ns0:c r="DY5" s="4" t="s">
+      <ns0:c r="ED5" s="4" t="s">
         <ns0:v>299</ns0:v>
       </ns0:c>
-      <ns0:c r="EA5" s="4" t="s">
+      <ns0:c r="EE5" t="s">
+        <ns0:v>542</ns0:v>
+      </ns0:c>
+      <ns0:c r="EF5" s="4" t="s">
         <ns0:v>157</ns0:v>
       </ns0:c>
-      <ns0:c r="EB5" s="4" t="s">
+      <ns0:c r="EG5" s="4" t="s">
         <ns0:v>113</ns0:v>
       </ns0:c>
-      <ns0:c r="EC5" s="4" t="s">
+      <ns0:c r="EH5" s="4" t="s">
         <ns0:v>114</ns0:v>
       </ns0:c>
-      <ns0:c r="ED5" s="4" t="s">
+      <ns0:c r="EI5" s="4" t="s">
         <ns0:v>159</ns0:v>
       </ns0:c>
-      <ns0:c r="EE5" s="4" t="s">
+      <ns0:c r="EJ5" s="4" t="s">
         <ns0:v>158</ns0:v>
       </ns0:c>
-      <ns0:c r="EF5" s="4" t="s">
+      <ns0:c r="EK5" s="4" t="s">
         <ns0:v>115</ns0:v>
       </ns0:c>
-      <ns0:c r="EG5" s="4" t="s">
+      <ns0:c r="EL5" s="4" t="s">
         <ns0:v>116</ns0:v>
       </ns0:c>
-      <ns0:c r="EH5" s="4" t="s">
+      <ns0:c r="EM5" s="4" t="s">
         <ns0:v>156</ns0:v>
       </ns0:c>
-      <ns0:c r="EI5" s="4" t="s">
+      <ns0:c r="EN5" s="4" t="s">
         <ns0:v>35</ns0:v>
       </ns0:c>
-      <ns0:c r="EJ5" s="4" t="s">
+      <ns0:c r="EO5" s="4" t="s">
         <ns0:v>228</ns0:v>
       </ns0:c>
-      <ns0:c r="EK5" s="4" t="s">
+      <ns0:c r="EP5" s="4" t="s">
         <ns0:v>428</ns0:v>
       </ns0:c>
-      <ns0:c r="EL5" s="4" t="s">
+      <ns0:c r="EQ5" s="4" t="s">
         <ns0:v>39</ns0:v>
       </ns0:c>
-      <ns0:c r="EM5" s="4" t="s">
+      <ns0:c r="ER5" s="4" t="s">
         <ns0:v>226</ns0:v>
       </ns0:c>
-      <ns0:c r="EN5" s="4" t="s">
+      <ns0:c r="ES5" s="4" t="s">
         <ns0:v>430</ns0:v>
       </ns0:c>
-      <ns0:c r="EO5" s="4" t="s">
+      <ns0:c r="ET5" s="4" t="s">
         <ns0:v>422</ns0:v>
       </ns0:c>
-      <ns0:c r="EP5" s="4" t="s">
+      <ns0:c r="EU5" s="4" t="s">
         <ns0:v>423</ns0:v>
       </ns0:c>
-      <ns0:c r="EQ5" s="4" t="s">
+      <ns0:c r="EV5" s="4" t="s">
         <ns0:v>523</ns0:v>
       </ns0:c>
-      <ns0:c r="ER5" s="7" t="s">
+      <ns0:c r="EW5" s="7" t="s">
         <ns0:v>42</ns0:v>
       </ns0:c>
-      <ns0:c r="ES5" s="4" t="s">
+      <ns0:c r="EX5" s="4" t="s">
         <ns0:v>224</ns0:v>
       </ns0:c>
-      <ns0:c r="ET5" s="4" t="s">
+      <ns0:c r="EY5" s="4" t="s">
         <ns0:v>432</ns0:v>
       </ns0:c>
-      <ns0:c r="EU5" s="4" t="s">
+      <ns0:c r="EZ5" s="4" t="s">
         <ns0:v>69</ns0:v>
       </ns0:c>
-      <ns0:c r="EV5" s="4" t="s">
+      <ns0:c r="FA5" s="4" t="s">
         <ns0:v>222</ns0:v>
       </ns0:c>
-      <ns0:c r="EW5" s="4" t="s">
+      <ns0:c r="FB5" s="4" t="s">
         <ns0:v>434</ns0:v>
       </ns0:c>
-      <ns0:c r="EX5" s="4" t="s">
+      <ns0:c r="FC5" s="4" t="s">
         <ns0:v>38</ns0:v>
       </ns0:c>
-      <ns0:c r="EY5" s="4" t="s">
+      <ns0:c r="FD5" s="4" t="s">
         <ns0:v>220</ns0:v>
       </ns0:c>
-      <ns0:c r="EZ5" s="4" t="s">
+      <ns0:c r="FE5" s="4" t="s">
         <ns0:v>436</ns0:v>
       </ns0:c>
-      <ns0:c r="FA5" s="7" t="s">
+      <ns0:c r="FF5" s="7" t="s">
         <ns0:v>41</ns0:v>
       </ns0:c>
-      <ns0:c r="FB5" s="4" t="s">
+      <ns0:c r="FG5" s="4" t="s">
         <ns0:v>218</ns0:v>
       </ns0:c>
-      <ns0:c r="FC5" s="4" t="s">
+      <ns0:c r="FH5" s="4" t="s">
         <ns0:v>447</ns0:v>
       </ns0:c>
-      <ns0:c r="FD5" s="7" t="s">
+      <ns0:c r="FI5" s="7" t="s">
         <ns0:v>4</ns0:v>
       </ns0:c>
-      <ns0:c r="FE5" s="4" t="s">
+      <ns0:c r="FJ5" s="4" t="s">
         <ns0:v>216</ns0:v>
       </ns0:c>
-      <ns0:c r="FF5" s="4" t="s">
+      <ns0:c r="FK5" s="4" t="s">
         <ns0:v>449</ns0:v>
       </ns0:c>
-      <ns0:c r="FG5" s="7" t="s">
+      <ns0:c r="FL5" s="7" t="s">
         <ns0:v>70</ns0:v>
       </ns0:c>
-      <ns0:c r="FH5" s="4" t="s">
+      <ns0:c r="FM5" s="4" t="s">
         <ns0:v>214</ns0:v>
       </ns0:c>
-      <ns0:c r="FI5" s="4" t="s">
+      <ns0:c r="FN5" s="4" t="s">
         <ns0:v>451</ns0:v>
       </ns0:c>
-      <ns0:c r="FJ5" s="4" t="s">
+      <ns0:c r="FO5" s="4" t="s">
         <ns0:v>40</ns0:v>
       </ns0:c>
-      <ns0:c r="FK5" s="4" t="s">
+      <ns0:c r="FP5" s="4" t="s">
         <ns0:v>212</ns0:v>
       </ns0:c>
-      <ns0:c r="FL5" s="4" t="s">
+      <ns0:c r="FQ5" s="4" t="s">
         <ns0:v>453</ns0:v>
       </ns0:c>
-      <ns0:c r="FM5" s="4" t="s">
+      <ns0:c r="FR5" s="4" t="s">
         <ns0:v>134</ns0:v>
       </ns0:c>
-      <ns0:c r="FN5" s="4" t="s">
+      <ns0:c r="FS5" s="4" t="s">
         <ns0:v>210</ns0:v>
       </ns0:c>
-      <ns0:c r="FO5" s="4" t="s">
+      <ns0:c r="FT5" s="4" t="s">
         <ns0:v>105</ns0:v>
       </ns0:c>
-      <ns0:c r="FP5" s="4" t="s">
+      <ns0:c r="FU5" s="4" t="s">
         <ns0:v>461</ns0:v>
       </ns0:c>
-      <ns0:c r="FQ5" s="4" t="s">
+      <ns0:c r="FV5" s="4" t="s">
         <ns0:v>208</ns0:v>
       </ns0:c>
-      <ns0:c r="FR5" s="4" t="s">
+      <ns0:c r="FW5" s="4" t="s">
         <ns0:v>455</ns0:v>
       </ns0:c>
-      <ns0:c r="FS5" s="14" t="s">
+      <ns0:c r="FX5" s="14" t="s">
         <ns0:v>78</ns0:v>
       </ns0:c>
-      <ns0:c r="FT5" s="4" t="s">
+      <ns0:c r="FY5" s="4" t="s">
         <ns0:v>206</ns0:v>
       </ns0:c>
-      <ns0:c r="FU5" s="4" t="s">
+      <ns0:c r="FZ5" s="4" t="s">
         <ns0:v>457</ns0:v>
       </ns0:c>
-      <ns0:c r="FV5" s="4" t="s">
+      <ns0:c r="GA5" s="4" t="s">
         <ns0:v>59</ns0:v>
       </ns0:c>
-      <ns0:c r="FW5" s="4" t="s">
+      <ns0:c r="GB5" s="4" t="s">
         <ns0:v>203</ns0:v>
       </ns0:c>
-      <ns0:c r="FX5" s="4" t="s">
+      <ns0:c r="GC5" s="4" t="s">
         <ns0:v>438</ns0:v>
       </ns0:c>
-      <ns0:c r="FY5" s="7" t="s">
+      <ns0:c r="GD5" s="7" t="s">
         <ns0:v>140</ns0:v>
       </ns0:c>
-      <ns0:c r="FZ5" s="4" t="s">
+      <ns0:c r="GE5" s="4" t="s">
         <ns0:v>202</ns0:v>
       </ns0:c>
-      <ns0:c r="GA5" s="4" t="s">
+      <ns0:c r="GF5" s="4" t="s">
         <ns0:v>440</ns0:v>
       </ns0:c>
-      <ns0:c r="GB5" s="4" t="s">
+      <ns0:c r="GG5" s="4" t="s">
         <ns0:v>142</ns0:v>
       </ns0:c>
-      <ns0:c r="GC5" s="4" t="s">
+      <ns0:c r="GH5" s="4" t="s">
         <ns0:v>201</ns0:v>
       </ns0:c>
-      <ns0:c r="GD5" s="4" t="s">
+      <ns0:c r="GI5" s="4" t="s">
         <ns0:v>442</ns0:v>
       </ns0:c>
-      <ns0:c r="GE5" s="7" t="s">
+      <ns0:c r="GJ5" s="7" t="s">
         <ns0:v>144</ns0:v>
       </ns0:c>
-      <ns0:c r="GF5" s="4" t="s">
+      <ns0:c r="GK5" s="4" t="s">
         <ns0:v>198</ns0:v>
       </ns0:c>
-      <ns0:c r="GG5" s="4" t="s">
+      <ns0:c r="GL5" s="4" t="s">
         <ns0:v>444</ns0:v>
       </ns0:c>
-      <ns0:c r="GH5" s="7" t="s">
+      <ns0:c r="GM5" s="7" t="s">
         <ns0:v>146</ns0:v>
       </ns0:c>
-      <ns0:c r="GI5" s="4" t="s">
+      <ns0:c r="GN5" s="4" t="s">
         <ns0:v>196</ns0:v>
       </ns0:c>
-      <ns0:c r="GJ5" s="4" t="s">
+      <ns0:c r="GO5" s="4" t="s">
         <ns0:v>459</ns0:v>
       </ns0:c>
-      <ns0:c r="GK5" s="4" t="s">
+      <ns0:c r="GP5" s="4" t="s">
         <ns0:v>520</ns0:v>
       </ns0:c>
-      <ns0:c r="GL5" s="4" t="s">
+      <ns0:c r="GQ5" s="4" t="s">
         <ns0:v>521</ns0:v>
       </ns0:c>
-      <ns0:c r="DZ5" t="s">
-        <ns0:v>542</ns0:v>
-      </ns0:c>
     </ns0:row>
-    <ns0:row r="6" spans="1:193" ht="16" thickTop="1" ns3:dyDescent="0.2">
+    <ns0:row r="6" spans="1:198" ht="16" thickTop="1" ns3:dyDescent="0.2">
       <ns0:c r="C6" s="1" t="s">
         <ns0:v>386</ns0:v>
       </ns0:c>
@@ -5211,7 +5610,6 @@
       <ns0:c r="BQ6" s="72" t="s">
         <ns0:v>426</ns0:v>
       </ns0:c>
-      <ns0:c r="BR6"/>
       <ns0:c r="BS6"/>
       <ns0:c r="BT6"/>
       <ns0:c r="BU6"/>
@@ -5221,40 +5619,45 @@
       <ns0:c r="BY6"/>
       <ns0:c r="BZ6"/>
       <ns0:c r="CA6" s="72" t="s">
+        <ns0:v>649</ns0:v>
+      </ns0:c>
+      <ns0:c r="CC6"/>
+      <ns0:c r="CD6" s="72" t="s">
         <ns0:v>427</ns0:v>
       </ns0:c>
-      <ns0:c r="CB6"/>
-      <ns0:c r="CC6"/>
-      <ns0:c r="CD6"/>
       <ns0:c r="CE6"/>
       <ns0:c r="CF6"/>
       <ns0:c r="CG6"/>
-      <ns0:c r="CH6" t="s">
-        <ns0:v>516</ns0:v>
-      </ns0:c>
+      <ns0:c r="CH6"/>
       <ns0:c r="CI6"/>
       <ns0:c r="CJ6"/>
-      <ns0:c r="CK6"/>
-      <ns0:c r="EI6" s="1" t="s">
+      <ns0:c r="CK6" t="s">
+        <ns0:v>516</ns0:v>
+      </ns0:c>
+      <ns0:c r="CL6"/>
+      <ns0:c r="CM6"/>
+      <ns0:c r="CO6"/>
+      <ns0:c r="CP6"/>
+      <ns0:c r="EN6" s="1" t="s">
         <ns0:v>399</ns0:v>
       </ns0:c>
-      <ns0:c r="EJ6" s="1" t="b">
+      <ns0:c r="EO6" s="1" t="b">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="GB6" s="1" t="s">
+      <ns0:c r="GG6" s="1" t="s">
         <ns0:v>400</ns0:v>
       </ns0:c>
-      <ns0:c r="GC6" s="1" t="b">
+      <ns0:c r="GH6" s="1" t="b">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="GE6" s="1" t="s">
+      <ns0:c r="GJ6" s="1" t="s">
         <ns0:v>401</ns0:v>
       </ns0:c>
-      <ns0:c r="GF6" s="1" t="b">
+      <ns0:c r="GK6" s="1" t="b">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
-    <ns0:row r="7" spans="1:193" ns3:dyDescent="0.2">
+    <ns0:row r="7" spans="1:198" ns3:dyDescent="0.2">
       <ns0:c r="C7" s="1" t="s">
         <ns0:v>386</ns0:v>
       </ns0:c>
@@ -5298,21 +5701,20 @@
       <ns0:formula1>1</ns0:formula1>
       <ns0:formula2>20</ns0:formula2>
     </ns0:dataValidation>
-    <ns0:dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="K6:K1048576 GB6:GB1048576 FY6:FY1048576 FS6:FS1048576 FV6:FV1048576 EX6:EX1048576 FP6:FP1048576 FJ6:FJ1048576 FM6:FM1048576 FG6:FG1048576 FD6:FD1048576 FA6:FA1048576 GE6:GE1048576 EU6:EU1048576 ER6:ER1048576 EL6:EL1048576 Q6:Q1048576 EI6:EI1048576 U6:U1048576 GH6:GH1048576" ns2:uid="{00000000-0002-0000-0000-000004000000}">
+    <ns0:dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="K6:K1048576 GG6:GG1048576 GD6:GD1048576 FX6:FX1048576 GA6:GA1048576 FC6:FC1048576 FU6:FU1048576 FO6:FO1048576 FR6:FR1048576 FL6:FL1048576 FI6:FI1048576 FF6:FF1048576 GJ6:GJ1048576 EZ6:EZ1048576 EW6:EW1048576 EQ6:EQ1048576 Q6:Q1048576 EN6:EN1048576 U6:U1048576 GM6:GM1048576" ns2:uid="{00000000-0002-0000-0000-000004000000}">
       <ns0:formula1>"FALSE,TRUE"</ns0:formula1>
     </ns0:dataValidation>
-    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BY6:BY1005 CJ6" ns2:uid="{8E3A2B14-DC85-6C41-B4DC-2591D3302965}">
-      <ns0:formula1>"MD5,SHA-1,SHA-256,SHA-384,SHA-512"</ns0:formula1>
+    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR6:BR7 CA6:CA7 CB6:CB7 CE6:CE7 CN6:CN7 CO6:CO7">
+      <ns0:formula1>"FALSE,TRUE"</ns0:formula1>
     </ns0:dataValidation>
-    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CE6:CE1005 BT6:BT1005" ns2:uid="{9900E669-7185-CC41-A6E0-A203DC0ED362}">
+    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BT6:BT7 CG6:CG7">
+      <ns0:formula1>"none,onLoad,onRequest,other"</ns0:formula1>
+    </ns0:dataValidation>
+    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU6:BU7 CH6:CH7">
       <ns0:formula1>"embed,new,none,other,replace"</ns0:formula1>
     </ns0:dataValidation>
-    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD6:CD1005 BS6:BS1005" ns2:uid="{9839E832-5A08-8846-B820-3F904D476D10}">
-      <ns0:formula1>"none,onLoad,onRequest,other"</ns0:formula1>
-    </ns0:dataValidation>
-    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB6:CB1005 BR7:BR1005" ns2:uid="{E9039B25-3CFB-C041-BF41-ECAB4B1AF243}">
-      <ns0:formula1>"FALSE,TRUE"</ns0:formula1>
-      <ns0:formula2>0</ns0:formula2>
+    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ6:BZ7 CM6:CM7">
+      <ns0:formula1>"MD5,SHA-1,SHA-256,SHA-384,SHA-512"</ns0:formula1>
     </ns0:dataValidation>
   </ns0:dataValidations>
   <ns0:hyperlinks>
@@ -5328,7 +5730,7 @@
           <ns5:formula1>
             <ns6:f>Sheet2!$A$2:$A$4</ns6:f>
           </ns5:formula1>
-          <ns6:sqref>CN6:CN1048576 CR6:CR1048576 DH6:DH1048576 CV6:CV1048576 DT6:DT1048576 DL6:DL1048576 DP6:DP1048576 DX6:DX1048576 CZ6:CZ1048576 DD6:DD1048576</ns6:sqref>
+          <ns6:sqref>CS6:CS1048576 CW6:CW1048576 DM6:DM1048576 DA6:DA1048576 DY6:DY1048576 DQ6:DQ1048576 DU6:DU1048576 EC6:EC1048576 DE6:DE1048576 DI6:DI1048576</ns6:sqref>
         </ns5:dataValidation>
       </ns5:dataValidations>
     </ns0:ext>

</xml_diff>

<commit_message>
ANW-3030 Add a column to make the imported digital object instance representative
An archival object only shows a thumbnail through its representative digital
object instance, and the archival object import never set one. The new
digital_object_is_representative column (FALSE/TRUE, blank for FALSE) marks the
instance linking the archival object to the digital object it creates as
representative.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/spec/fixtures/bulk_import/bulk_import_VFIRST01_test01.xlsx
+++ b/backend/spec/fixtures/bulk_import/bulk_import_VFIRST01_test01.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:sst xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="650">
+<ns0:sst xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="654">
   <ns0:si>
     <ns0:t>Mapping - ArchivesSpace Resource record SECTION</ns0:t>
   </ns0:si>
@@ -1989,6 +1989,18 @@
   </ns0:si>
   <ns0:si>
     <ns0:t xml:space="preserve">TRUE</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Digital Object</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Make the instance linking the archival object to the digital object representative (FALSE/TRUE)? The archival object then shows the thumbnail of the digital object. Leave this blank to get the default value FALSE.</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">digital_object_is_representative</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t xml:space="preserve">Make Digital Object Instance Representative</ns0:t>
   </ns0:si>
 </ns0:sst>
 </file>
@@ -2943,7 +2955,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns6="http://schemas.microsoft.com/office/excel/2006/main" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
-  <ns0:dimension ref="A1:ASP7"/>
+  <ns0:dimension ref="A1:ASQ7"/>
   <ns0:sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" ns3:dyDescent="0.2"/>
   <ns0:cols>
     <ns0:col min="1" max="1" width="13.1640625" style="30" customWidth="1"/>
@@ -3021,100 +3033,101 @@
     <ns0:col min="92" max="92" width="24" customWidth="1"/>
     <ns0:col min="93" max="93" width="24" customWidth="1"/>
     <ns0:col min="94" max="94" width="24" customWidth="1"/>
-    <ns0:col min="95" max="95" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="96" max="96" width="22.6640625" style="1"/>
-    <ns0:col min="97" max="97" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="98" max="98" width="13" style="1" customWidth="1"/>
-    <ns0:col min="99" max="99" width="15.5" style="1" customWidth="1"/>
-    <ns0:col min="100" max="100" width="22.6640625" style="1"/>
-    <ns0:col min="101" max="101" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="102" max="102" width="9.1640625" style="1"/>
-    <ns0:col min="103" max="103" width="15.1640625" style="1" customWidth="1"/>
-    <ns0:col min="104" max="104" width="20.1640625" style="1" customWidth="1"/>
-    <ns0:col min="105" max="105" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="106" max="106" width="12.83203125" style="1" customWidth="1"/>
-    <ns0:col min="107" max="107" width="15.1640625" style="1" customWidth="1"/>
-    <ns0:col min="108" max="108" width="20.1640625" style="1" customWidth="1"/>
-    <ns0:col min="109" max="109" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="110" max="110" width="12.83203125" style="1" customWidth="1"/>
-    <ns0:col min="111" max="111" width="15.1640625" style="1" customWidth="1"/>
-    <ns0:col min="112" max="112" width="20.1640625" style="1" customWidth="1"/>
-    <ns0:col min="113" max="113" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="114" max="114" width="12.83203125" style="1" customWidth="1"/>
-    <ns0:col min="115" max="115" width="9.1640625" style="1"/>
-    <ns0:col min="116" max="116" width="11.5" style="1" customWidth="1"/>
-    <ns0:col min="117" max="117" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="118" max="119" width="9.1640625" style="1"/>
-    <ns0:col min="120" max="120" width="11.5" style="1" customWidth="1"/>
-    <ns0:col min="121" max="121" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="122" max="124" width="9.1640625" style="1"/>
-    <ns0:col min="125" max="125" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="126" max="128" width="9.1640625" style="1"/>
-    <ns0:col min="129" max="129" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="130" max="132" width="9.1640625" style="1"/>
-    <ns0:col min="133" max="133" width="15.33203125" style="1" customWidth="1"/>
-    <ns0:col min="134" max="134" width="9.1640625" style="1"/>
-    <ns0:col min="135" max="135" width="11.5" style="1" customWidth="1"/>
-    <ns0:col min="136" max="136" width="12.33203125" style="1" customWidth="1"/>
-    <ns0:col min="137" max="139" width="13.5" style="1" customWidth="1"/>
-    <ns0:col min="140" max="141" width="10.83203125" style="1" customWidth="1"/>
-    <ns0:col min="142" max="142" width="15.5" style="1" customWidth="1"/>
-    <ns0:col min="143" max="143" width="9.33203125" style="1"/>
-    <ns0:col min="144" max="144" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="145" max="145" width="17.6640625" customWidth="1"/>
-    <ns0:col min="146" max="146" width="17" style="1" customWidth="1"/>
-    <ns0:col min="147" max="147" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="148" max="148" width="17.6640625" customWidth="1"/>
-    <ns0:col min="149" max="150" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="151" max="152" width="12.33203125" style="1" customWidth="1"/>
-    <ns0:col min="153" max="153" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="154" max="154" width="17.6640625" customWidth="1"/>
-    <ns0:col min="155" max="155" width="11.6640625" style="1" customWidth="1"/>
-    <ns0:col min="156" max="156" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="157" max="157" width="17.6640625" customWidth="1"/>
-    <ns0:col min="158" max="158" width="16" style="1" customWidth="1"/>
-    <ns0:col min="159" max="159" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="160" max="160" width="17.6640625" customWidth="1"/>
-    <ns0:col min="161" max="161" width="9.1640625" style="1"/>
-    <ns0:col min="162" max="162" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="163" max="163" width="17.6640625" customWidth="1"/>
-    <ns0:col min="164" max="164" width="12" customWidth="1"/>
-    <ns0:col min="165" max="165" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="166" max="166" width="17.6640625" customWidth="1"/>
-    <ns0:col min="167" max="167" width="11.83203125" style="1" customWidth="1"/>
-    <ns0:col min="168" max="168" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="169" max="169" width="17.6640625" customWidth="1"/>
-    <ns0:col min="170" max="170" width="11.83203125" style="1" customWidth="1"/>
-    <ns0:col min="171" max="171" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="172" max="172" width="17.6640625" customWidth="1"/>
-    <ns0:col min="173" max="173" width="11.83203125" style="1" customWidth="1"/>
-    <ns0:col min="174" max="174" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="175" max="175" width="11.83203125" style="1" customWidth="1"/>
-    <ns0:col min="176" max="176" width="17.6640625" customWidth="1"/>
-    <ns0:col min="177" max="177" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="178" max="178" width="17.6640625" customWidth="1"/>
-    <ns0:col min="179" max="179" width="14.83203125" style="1" customWidth="1"/>
-    <ns0:col min="180" max="180" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="181" max="181" width="17.6640625" customWidth="1"/>
-    <ns0:col min="182" max="182" width="12.33203125" style="1" customWidth="1"/>
-    <ns0:col min="183" max="183" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="184" max="184" width="17.6640625" customWidth="1"/>
-    <ns0:col min="185" max="185" width="9.1640625" style="1"/>
-    <ns0:col min="186" max="186" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="187" max="187" width="17.6640625" customWidth="1"/>
-    <ns0:col min="188" max="188" width="9.1640625" style="1"/>
-    <ns0:col min="189" max="189" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="190" max="190" width="17.6640625" customWidth="1"/>
-    <ns0:col min="191" max="191" width="18.5" style="1" customWidth="1"/>
-    <ns0:col min="192" max="192" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="193" max="193" width="17.6640625" customWidth="1"/>
-    <ns0:col min="194" max="194" width="10.1640625" style="1" customWidth="1"/>
-    <ns0:col min="195" max="195" width="17.6640625" style="1" customWidth="1"/>
-    <ns0:col min="196" max="198" width="17.6640625" customWidth="1"/>
-    <ns0:col min="199" max="1185" width="9.33203125" style="1"/>
+    <ns0:col min="95" max="95" width="24" customWidth="1"/>
+    <ns0:col min="96" max="96" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="97" max="97" width="22.6640625" style="1"/>
+    <ns0:col min="98" max="98" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="99" max="99" width="13" style="1" customWidth="1"/>
+    <ns0:col min="100" max="100" width="15.5" style="1" customWidth="1"/>
+    <ns0:col min="101" max="101" width="22.6640625" style="1"/>
+    <ns0:col min="102" max="102" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="103" max="103" width="9.1640625" style="1"/>
+    <ns0:col min="104" max="104" width="15.1640625" style="1" customWidth="1"/>
+    <ns0:col min="105" max="105" width="20.1640625" style="1" customWidth="1"/>
+    <ns0:col min="106" max="106" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="107" max="107" width="12.83203125" style="1" customWidth="1"/>
+    <ns0:col min="108" max="108" width="15.1640625" style="1" customWidth="1"/>
+    <ns0:col min="109" max="109" width="20.1640625" style="1" customWidth="1"/>
+    <ns0:col min="110" max="110" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="111" max="111" width="12.83203125" style="1" customWidth="1"/>
+    <ns0:col min="112" max="112" width="15.1640625" style="1" customWidth="1"/>
+    <ns0:col min="113" max="113" width="20.1640625" style="1" customWidth="1"/>
+    <ns0:col min="114" max="114" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="115" max="115" width="12.83203125" style="1" customWidth="1"/>
+    <ns0:col min="116" max="116" width="9.1640625" style="1"/>
+    <ns0:col min="117" max="117" width="11.5" style="1" customWidth="1"/>
+    <ns0:col min="118" max="118" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="119" max="120" width="9.1640625" style="1"/>
+    <ns0:col min="121" max="121" width="11.5" style="1" customWidth="1"/>
+    <ns0:col min="122" max="122" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="123" max="125" width="9.1640625" style="1"/>
+    <ns0:col min="126" max="126" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="127" max="129" width="9.1640625" style="1"/>
+    <ns0:col min="130" max="130" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="131" max="133" width="9.1640625" style="1"/>
+    <ns0:col min="134" max="134" width="15.33203125" style="1" customWidth="1"/>
+    <ns0:col min="135" max="135" width="9.1640625" style="1"/>
+    <ns0:col min="136" max="136" width="11.5" style="1" customWidth="1"/>
+    <ns0:col min="137" max="137" width="12.33203125" style="1" customWidth="1"/>
+    <ns0:col min="138" max="140" width="13.5" style="1" customWidth="1"/>
+    <ns0:col min="141" max="142" width="10.83203125" style="1" customWidth="1"/>
+    <ns0:col min="143" max="143" width="15.5" style="1" customWidth="1"/>
+    <ns0:col min="144" max="144" width="9.33203125" style="1"/>
+    <ns0:col min="145" max="145" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="146" max="146" width="17.6640625" customWidth="1"/>
+    <ns0:col min="147" max="147" width="17" style="1" customWidth="1"/>
+    <ns0:col min="148" max="148" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="149" max="149" width="17.6640625" customWidth="1"/>
+    <ns0:col min="150" max="151" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="152" max="153" width="12.33203125" style="1" customWidth="1"/>
+    <ns0:col min="154" max="154" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="155" max="155" width="17.6640625" customWidth="1"/>
+    <ns0:col min="156" max="156" width="11.6640625" style="1" customWidth="1"/>
+    <ns0:col min="157" max="157" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="158" max="158" width="17.6640625" customWidth="1"/>
+    <ns0:col min="159" max="159" width="16" style="1" customWidth="1"/>
+    <ns0:col min="160" max="160" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="161" max="161" width="17.6640625" customWidth="1"/>
+    <ns0:col min="162" max="162" width="9.1640625" style="1"/>
+    <ns0:col min="163" max="163" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="164" max="164" width="17.6640625" customWidth="1"/>
+    <ns0:col min="165" max="165" width="12" customWidth="1"/>
+    <ns0:col min="166" max="166" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="167" max="167" width="17.6640625" customWidth="1"/>
+    <ns0:col min="168" max="168" width="11.83203125" style="1" customWidth="1"/>
+    <ns0:col min="169" max="169" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="170" max="170" width="17.6640625" customWidth="1"/>
+    <ns0:col min="171" max="171" width="11.83203125" style="1" customWidth="1"/>
+    <ns0:col min="172" max="172" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="173" max="173" width="17.6640625" customWidth="1"/>
+    <ns0:col min="174" max="174" width="11.83203125" style="1" customWidth="1"/>
+    <ns0:col min="175" max="175" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="176" max="176" width="11.83203125" style="1" customWidth="1"/>
+    <ns0:col min="177" max="177" width="17.6640625" customWidth="1"/>
+    <ns0:col min="178" max="178" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="179" max="179" width="17.6640625" customWidth="1"/>
+    <ns0:col min="180" max="180" width="14.83203125" style="1" customWidth="1"/>
+    <ns0:col min="181" max="181" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="182" max="182" width="17.6640625" customWidth="1"/>
+    <ns0:col min="183" max="183" width="12.33203125" style="1" customWidth="1"/>
+    <ns0:col min="184" max="184" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="185" max="185" width="17.6640625" customWidth="1"/>
+    <ns0:col min="186" max="186" width="9.1640625" style="1"/>
+    <ns0:col min="187" max="187" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="188" max="188" width="17.6640625" customWidth="1"/>
+    <ns0:col min="189" max="189" width="9.1640625" style="1"/>
+    <ns0:col min="190" max="190" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="191" max="191" width="17.6640625" customWidth="1"/>
+    <ns0:col min="192" max="192" width="18.5" style="1" customWidth="1"/>
+    <ns0:col min="193" max="193" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="194" max="194" width="17.6640625" customWidth="1"/>
+    <ns0:col min="195" max="195" width="10.1640625" style="1" customWidth="1"/>
+    <ns0:col min="196" max="196" width="17.6640625" style="1" customWidth="1"/>
+    <ns0:col min="197" max="199" width="17.6640625" customWidth="1"/>
+    <ns0:col min="200" max="1186" width="9.33203125" style="1"/>
   </ns0:cols>
   <ns0:sheetData>
-    <ns0:row r="1" spans="1:198" ht="16" thickBot="1" ns3:dyDescent="0.25">
+    <ns0:row r="1" spans="1:199" ht="16" thickBot="1" ns3:dyDescent="0.25">
       <ns0:c r="A1" s="30" t="s">
         <ns0:v>385</ns0:v>
       </ns0:c>
@@ -3124,27 +3137,27 @@
       <ns0:c r="R1"/>
       <ns0:c r="S1"/>
       <ns0:c r="T1"/>
-      <ns0:c r="EP1" s="1"/>
-      <ns0:c r="ES1" s="1"/>
-      <ns0:c r="EY1" s="1"/>
-      <ns0:c r="FB1" s="1"/>
-      <ns0:c r="FE1" s="1"/>
-      <ns0:c r="FH1" s="1"/>
-      <ns0:c r="FK1" s="1"/>
-      <ns0:c r="FN1" s="1"/>
-      <ns0:c r="FQ1" s="1"/>
-      <ns0:c r="FU1" s="1"/>
-      <ns0:c r="FW1" s="1"/>
-      <ns0:c r="FZ1" s="1"/>
-      <ns0:c r="GC1" s="1"/>
-      <ns0:c r="GF1" s="1"/>
-      <ns0:c r="GI1" s="1"/>
-      <ns0:c r="GL1" s="1"/>
-      <ns0:c r="GO1" s="1"/>
+      <ns0:c r="EQ1" s="1"/>
+      <ns0:c r="ET1" s="1"/>
+      <ns0:c r="EZ1" s="1"/>
+      <ns0:c r="FC1" s="1"/>
+      <ns0:c r="FF1" s="1"/>
+      <ns0:c r="FI1" s="1"/>
+      <ns0:c r="FL1" s="1"/>
+      <ns0:c r="FO1" s="1"/>
+      <ns0:c r="FR1" s="1"/>
+      <ns0:c r="FV1" s="1"/>
+      <ns0:c r="FX1" s="1"/>
+      <ns0:c r="GA1" s="1"/>
+      <ns0:c r="GD1" s="1"/>
+      <ns0:c r="GG1" s="1"/>
+      <ns0:c r="GJ1" s="1"/>
+      <ns0:c r="GM1" s="1"/>
       <ns0:c r="GP1" s="1"/>
       <ns0:c r="GQ1" s="1"/>
+      <ns0:c r="GR1" s="1"/>
     </ns0:row>
-    <ns0:row r="2" spans="1:198" s="1" customFormat="1" ht="61" thickTop="1" ns3:dyDescent="0.2">
+    <ns0:row r="2" spans="1:199" s="1" customFormat="1" ht="61" thickTop="1" ns3:dyDescent="0.2">
       <ns0:c r="A2" s="32" t="s">
         <ns0:v>0</ns0:v>
       </ns0:c>
@@ -3349,94 +3362,94 @@
       <ns0:c r="BP2" s="22" t="s">
         <ns0:v>37</ns0:v>
       </ns0:c>
-      <ns0:c r="BQ2" s="70" t="s">
+      <ns0:c r="BQ2" s="22" t="s">
+        <ns0:v>650</ns0:v>
+      </ns0:c>
+      <ns0:c r="BR2" s="70" t="s">
         <ns0:v>545</ns0:v>
       </ns0:c>
-      <ns0:c r="BR2" s="70" t="s">
+      <ns0:c r="BS2" s="70" t="s">
         <ns0:v>546</ns0:v>
       </ns0:c>
-      <ns0:c r="BS2" s="70" t="s">
+      <ns0:c r="BT2" s="70" t="s">
         <ns0:v>547</ns0:v>
       </ns0:c>
-      <ns0:c r="BT2" s="70" t="s">
+      <ns0:c r="BU2" s="70" t="s">
         <ns0:v>548</ns0:v>
       </ns0:c>
-      <ns0:c r="BU2" s="70" t="s">
+      <ns0:c r="BV2" s="70" t="s">
         <ns0:v>549</ns0:v>
       </ns0:c>
-      <ns0:c r="BV2" s="70" t="s">
+      <ns0:c r="BW2" s="70" t="s">
         <ns0:v>550</ns0:v>
       </ns0:c>
-      <ns0:c r="BW2" s="70" t="s">
+      <ns0:c r="BX2" s="70" t="s">
         <ns0:v>551</ns0:v>
       </ns0:c>
-      <ns0:c r="BX2" s="70" t="s">
+      <ns0:c r="BY2" s="70" t="s">
         <ns0:v>552</ns0:v>
       </ns0:c>
-      <ns0:c r="BY2" s="70" t="s">
+      <ns0:c r="BZ2" s="70" t="s">
         <ns0:v>553</ns0:v>
       </ns0:c>
-      <ns0:c r="BZ2" s="70" t="s">
+      <ns0:c r="CA2" s="70" t="s">
         <ns0:v>554</ns0:v>
       </ns0:c>
-      <ns0:c r="CA2" s="70" t="s">
+      <ns0:c r="CB2" s="70" t="s">
         <ns0:v>555</ns0:v>
       </ns0:c>
-      <ns0:c r="CB2" s="70" t="s">
+      <ns0:c r="CC2" s="70" t="s">
         <ns0:v>556</ns0:v>
       </ns0:c>
-      <ns0:c r="CC2" s="70" t="s">
+      <ns0:c r="CD2" s="70" t="s">
         <ns0:v>557</ns0:v>
       </ns0:c>
-      <ns0:c r="CD2" s="70" t="s">
+      <ns0:c r="CE2" s="70" t="s">
         <ns0:v>558</ns0:v>
       </ns0:c>
-      <ns0:c r="CE2" s="70" t="s">
+      <ns0:c r="CF2" s="70" t="s">
         <ns0:v>559</ns0:v>
       </ns0:c>
-      <ns0:c r="CF2" s="70" t="s">
+      <ns0:c r="CG2" s="70" t="s">
         <ns0:v>560</ns0:v>
       </ns0:c>
-      <ns0:c r="CG2" s="70" t="s">
+      <ns0:c r="CH2" s="70" t="s">
         <ns0:v>561</ns0:v>
       </ns0:c>
-      <ns0:c r="CH2" s="70" t="s">
+      <ns0:c r="CI2" s="70" t="s">
         <ns0:v>562</ns0:v>
       </ns0:c>
-      <ns0:c r="CI2" s="70" t="s">
+      <ns0:c r="CJ2" s="70" t="s">
         <ns0:v>563</ns0:v>
       </ns0:c>
-      <ns0:c r="CJ2" s="70" t="s">
+      <ns0:c r="CK2" s="70" t="s">
         <ns0:v>564</ns0:v>
       </ns0:c>
-      <ns0:c r="CK2" s="70" t="s">
+      <ns0:c r="CL2" s="70" t="s">
         <ns0:v>565</ns0:v>
       </ns0:c>
-      <ns0:c r="CL2" s="70" t="s">
+      <ns0:c r="CM2" s="70" t="s">
         <ns0:v>566</ns0:v>
       </ns0:c>
-      <ns0:c r="CM2" s="70" t="s">
+      <ns0:c r="CN2" s="70" t="s">
         <ns0:v>567</ns0:v>
       </ns0:c>
-      <ns0:c r="CN2" s="70" t="s">
+      <ns0:c r="CO2" s="70" t="s">
         <ns0:v>568</ns0:v>
       </ns0:c>
-      <ns0:c r="CO2" s="70" t="s">
+      <ns0:c r="CP2" s="70" t="s">
         <ns0:v>569</ns0:v>
       </ns0:c>
-      <ns0:c r="CP2" s="70" t="s">
+      <ns0:c r="CQ2" s="70" t="s">
         <ns0:v>570</ns0:v>
       </ns0:c>
-      <ns0:c r="CQ2" s="47" t="s">
+      <ns0:c r="CR2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="CR2" s="19" t="s">
+      <ns0:c r="CS2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="CS2" s="47" t="s">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="CT2" s="19" t="s">
+      <ns0:c r="CT2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="CU2" s="19" t="s">
@@ -3445,10 +3458,10 @@
       <ns0:c r="CV2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="CW2" s="47" t="s">
+      <ns0:c r="CW2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="CX2" s="19" t="s">
+      <ns0:c r="CX2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="CY2" s="19" t="s">
@@ -3457,10 +3470,10 @@
       <ns0:c r="CZ2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DA2" s="47" t="s">
+      <ns0:c r="DA2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DB2" s="19" t="s">
+      <ns0:c r="DB2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="DC2" s="19" t="s">
@@ -3469,10 +3482,10 @@
       <ns0:c r="DD2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DE2" s="47" t="s">
+      <ns0:c r="DE2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DF2" s="19" t="s">
+      <ns0:c r="DF2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="DG2" s="19" t="s">
@@ -3481,10 +3494,10 @@
       <ns0:c r="DH2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DI2" s="47" t="s">
+      <ns0:c r="DI2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DJ2" s="19" t="s">
+      <ns0:c r="DJ2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="DK2" s="19" t="s">
@@ -3493,10 +3506,10 @@
       <ns0:c r="DL2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DM2" s="47" t="s">
+      <ns0:c r="DM2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DN2" s="19" t="s">
+      <ns0:c r="DN2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="DO2" s="19" t="s">
@@ -3505,10 +3518,10 @@
       <ns0:c r="DP2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DQ2" s="47" t="s">
+      <ns0:c r="DQ2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DR2" s="19" t="s">
+      <ns0:c r="DR2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="DS2" s="19" t="s">
@@ -3517,10 +3530,10 @@
       <ns0:c r="DT2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DU2" s="47" t="s">
+      <ns0:c r="DU2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DV2" s="19" t="s">
+      <ns0:c r="DV2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="DW2" s="19" t="s">
@@ -3529,10 +3542,10 @@
       <ns0:c r="DX2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DY2" s="47" t="s">
+      <ns0:c r="DY2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="DZ2" s="19" t="s">
+      <ns0:c r="DZ2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="EA2" s="19" t="s">
@@ -3541,17 +3554,17 @@
       <ns0:c r="EB2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="EC2" s="47" t="s">
+      <ns0:c r="EC2" s="19" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="ED2" s="19" t="s">
+      <ns0:c r="ED2" s="47" t="s">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="EE2" t="s">
+      <ns0:c r="EE2" s="19" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="EF2" t="s">
         <ns0:v>543</ns0:v>
-      </ns0:c>
-      <ns0:c r="EF2" s="21" t="s">
-        <ns0:v>108</ns0:v>
       </ns0:c>
       <ns0:c r="EG2" s="21" t="s">
         <ns0:v>108</ns0:v>
@@ -3574,97 +3587,97 @@
       <ns0:c r="EM2" s="21" t="s">
         <ns0:v>108</ns0:v>
       </ns0:c>
-      <ns0:c r="EN2" s="28" t="s">
-        <ns0:v>58</ns0:v>
+      <ns0:c r="EN2" s="21" t="s">
+        <ns0:v>108</ns0:v>
       </ns0:c>
       <ns0:c r="EO2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EP2" s="67" t="s">
+      <ns0:c r="EP2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EQ2" s="28" t="s">
+      <ns0:c r="EQ2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="ER2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="ES2" s="67" t="s">
+      <ns0:c r="ES2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="ET2" s="66" t="s">
+      <ns0:c r="ET2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="EU2" s="66" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EV2" s="67" t="s">
+      <ns0:c r="EV2" s="66" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EW2" s="28" t="s">
+      <ns0:c r="EW2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="EX2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EY2" s="67" t="s">
+      <ns0:c r="EY2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="EZ2" s="28" t="s">
+      <ns0:c r="EZ2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FA2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FB2" s="67" t="s">
+      <ns0:c r="FB2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FC2" s="27" t="s">
+      <ns0:c r="FC2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FD2" s="28" t="s">
+      <ns0:c r="FD2" s="27" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FE2" s="67" t="s">
+      <ns0:c r="FE2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FF2" s="28" t="s">
+      <ns0:c r="FF2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FG2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FH2" s="67" t="s">
+      <ns0:c r="FH2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FI2" s="28" t="s">
+      <ns0:c r="FI2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FJ2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FK2" s="67" t="s">
+      <ns0:c r="FK2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FL2" s="28" t="s">
+      <ns0:c r="FL2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FM2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FN2" s="67" t="s">
+      <ns0:c r="FN2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FO2" s="28" t="s">
+      <ns0:c r="FO2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FP2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FQ2" s="67" t="s">
+      <ns0:c r="FQ2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FR2" s="28" t="s">
+      <ns0:c r="FR2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="FS2" s="28" t="s">
@@ -3673,67 +3686,67 @@
       <ns0:c r="FT2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FU2" s="67" t="s">
+      <ns0:c r="FU2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FV2" s="28" t="s">
+      <ns0:c r="FV2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FW2" s="67" t="s">
+      <ns0:c r="FW2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FX2" s="29" t="s">
+      <ns0:c r="FX2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FY2" s="28" t="s">
+      <ns0:c r="FY2" s="29" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="FZ2" s="67" t="s">
+      <ns0:c r="FZ2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GA2" s="28" t="s">
+      <ns0:c r="GA2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="GB2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GC2" s="67" t="s">
+      <ns0:c r="GC2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GD2" s="28" t="s">
+      <ns0:c r="GD2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="GE2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GF2" s="67" t="s">
+      <ns0:c r="GF2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GG2" s="28" t="s">
+      <ns0:c r="GG2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="GH2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GI2" s="67" t="s">
+      <ns0:c r="GI2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GJ2" s="28" t="s">
+      <ns0:c r="GJ2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="GK2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GL2" s="67" t="s">
+      <ns0:c r="GL2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GM2" s="28" t="s">
+      <ns0:c r="GM2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="GN2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
-      <ns0:c r="GO2" s="67" t="s">
+      <ns0:c r="GO2" s="28" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
       <ns0:c r="GP2" s="67" t="s">
@@ -3742,8 +3755,11 @@
       <ns0:c r="GQ2" s="67" t="s">
         <ns0:v>58</ns0:v>
       </ns0:c>
+      <ns0:c r="GR2" s="67" t="s">
+        <ns0:v>58</ns0:v>
+      </ns0:c>
     </ns0:row>
-    <ns0:row r="3" spans="1:198" ht="105.75" customHeight="1" thickBot="1" ns3:dyDescent="0.25">
+    <ns0:row r="3" spans="1:199" ht="105.75" customHeight="1" thickBot="1" ns3:dyDescent="0.25">
       <ns0:c r="A3" s="33" t="s">
         <ns0:v>61</ns0:v>
       </ns0:c>
@@ -3946,401 +3962,404 @@
       <ns0:c r="BP3" s="23" t="s">
         <ns0:v>415</ns0:v>
       </ns0:c>
-      <ns0:c r="BQ3" s="71" t="s">
+      <ns0:c r="BQ3" s="23" t="s">
+        <ns0:v>651</ns0:v>
+      </ns0:c>
+      <ns0:c r="BR3" s="71" t="s">
         <ns0:v>571</ns0:v>
       </ns0:c>
-      <ns0:c r="BR3" s="71" t="s">
+      <ns0:c r="BS3" s="71" t="s">
         <ns0:v>572</ns0:v>
       </ns0:c>
-      <ns0:c r="BS3" s="71" t="s">
+      <ns0:c r="BT3" s="71" t="s">
         <ns0:v>573</ns0:v>
       </ns0:c>
-      <ns0:c r="BT3" s="71" t="s">
+      <ns0:c r="BU3" s="71" t="s">
         <ns0:v>574</ns0:v>
       </ns0:c>
-      <ns0:c r="BU3" s="71" t="s">
+      <ns0:c r="BV3" s="71" t="s">
         <ns0:v>575</ns0:v>
       </ns0:c>
-      <ns0:c r="BV3" s="71" t="s">
+      <ns0:c r="BW3" s="71" t="s">
         <ns0:v>576</ns0:v>
       </ns0:c>
-      <ns0:c r="BW3" s="71" t="s">
+      <ns0:c r="BX3" s="71" t="s">
         <ns0:v>577</ns0:v>
       </ns0:c>
-      <ns0:c r="BX3" s="71" t="s">
+      <ns0:c r="BY3" s="71" t="s">
         <ns0:v>578</ns0:v>
       </ns0:c>
-      <ns0:c r="BY3" s="71" t="s">
+      <ns0:c r="BZ3" s="71" t="s">
         <ns0:v>579</ns0:v>
       </ns0:c>
-      <ns0:c r="BZ3" s="71" t="s">
+      <ns0:c r="CA3" s="71" t="s">
         <ns0:v>580</ns0:v>
       </ns0:c>
-      <ns0:c r="CA3" s="71" t="s">
+      <ns0:c r="CB3" s="71" t="s">
         <ns0:v>581</ns0:v>
       </ns0:c>
-      <ns0:c r="CB3" s="71" t="s">
+      <ns0:c r="CC3" s="71" t="s">
         <ns0:v>582</ns0:v>
       </ns0:c>
-      <ns0:c r="CC3" s="71" t="s">
+      <ns0:c r="CD3" s="71" t="s">
         <ns0:v>583</ns0:v>
       </ns0:c>
-      <ns0:c r="CD3" s="71" t="s">
+      <ns0:c r="CE3" s="71" t="s">
         <ns0:v>584</ns0:v>
       </ns0:c>
-      <ns0:c r="CE3" s="71" t="s">
+      <ns0:c r="CF3" s="71" t="s">
         <ns0:v>585</ns0:v>
       </ns0:c>
-      <ns0:c r="CF3" s="71" t="s">
+      <ns0:c r="CG3" s="71" t="s">
         <ns0:v>586</ns0:v>
       </ns0:c>
-      <ns0:c r="CG3" s="71" t="s">
+      <ns0:c r="CH3" s="71" t="s">
         <ns0:v>587</ns0:v>
       </ns0:c>
-      <ns0:c r="CH3" s="71" t="s">
+      <ns0:c r="CI3" s="71" t="s">
         <ns0:v>588</ns0:v>
       </ns0:c>
-      <ns0:c r="CI3" s="71" t="s">
+      <ns0:c r="CJ3" s="71" t="s">
         <ns0:v>589</ns0:v>
       </ns0:c>
-      <ns0:c r="CJ3" s="71" t="s">
+      <ns0:c r="CK3" s="71" t="s">
         <ns0:v>590</ns0:v>
       </ns0:c>
-      <ns0:c r="CK3" s="71" t="s">
+      <ns0:c r="CL3" s="71" t="s">
         <ns0:v>591</ns0:v>
       </ns0:c>
-      <ns0:c r="CL3" s="71" t="s">
+      <ns0:c r="CM3" s="71" t="s">
         <ns0:v>592</ns0:v>
       </ns0:c>
-      <ns0:c r="CM3" s="71" t="s">
+      <ns0:c r="CN3" s="71" t="s">
         <ns0:v>593</ns0:v>
       </ns0:c>
-      <ns0:c r="CN3" s="71" t="s">
+      <ns0:c r="CO3" s="71" t="s">
         <ns0:v>594</ns0:v>
       </ns0:c>
-      <ns0:c r="CO3" s="71" t="s">
+      <ns0:c r="CP3" s="71" t="s">
         <ns0:v>595</ns0:v>
       </ns0:c>
-      <ns0:c r="CP3" s="71" t="s">
+      <ns0:c r="CQ3" s="71" t="s">
         <ns0:v>596</ns0:v>
       </ns0:c>
-      <ns0:c r="CQ3" s="26" t="s">
+      <ns0:c r="CR3" s="26" t="s">
         <ns0:v>160</ns0:v>
       </ns0:c>
-      <ns0:c r="CR3" s="26" t="s">
+      <ns0:c r="CS3" s="26" t="s">
         <ns0:v>162</ns0:v>
       </ns0:c>
-      <ns0:c r="CS3" s="26" t="s">
+      <ns0:c r="CT3" s="26" t="s">
         <ns0:v>247</ns0:v>
       </ns0:c>
-      <ns0:c r="CT3" s="26" t="s">
+      <ns0:c r="CU3" s="26" t="s">
         <ns0:v>275</ns0:v>
       </ns0:c>
-      <ns0:c r="CU3" s="26" t="s">
+      <ns0:c r="CV3" s="26" t="s">
         <ns0:v>160</ns0:v>
       </ns0:c>
-      <ns0:c r="CV3" s="26" t="s">
+      <ns0:c r="CW3" s="26" t="s">
         <ns0:v>162</ns0:v>
       </ns0:c>
-      <ns0:c r="CW3" s="26" t="s">
+      <ns0:c r="CX3" s="26" t="s">
         <ns0:v>247</ns0:v>
       </ns0:c>
-      <ns0:c r="CX3" s="26" t="s">
+      <ns0:c r="CY3" s="26" t="s">
         <ns0:v>276</ns0:v>
       </ns0:c>
-      <ns0:c r="CY3" s="26" t="s">
+      <ns0:c r="CZ3" s="26" t="s">
         <ns0:v>160</ns0:v>
       </ns0:c>
-      <ns0:c r="CZ3" s="26" t="s">
+      <ns0:c r="DA3" s="26" t="s">
         <ns0:v>162</ns0:v>
       </ns0:c>
-      <ns0:c r="DA3" s="26" t="s">
+      <ns0:c r="DB3" s="26" t="s">
         <ns0:v>247</ns0:v>
       </ns0:c>
-      <ns0:c r="DB3" s="26" t="s">
+      <ns0:c r="DC3" s="26" t="s">
         <ns0:v>300</ns0:v>
       </ns0:c>
-      <ns0:c r="DC3" s="26" t="s">
+      <ns0:c r="DD3" s="26" t="s">
         <ns0:v>160</ns0:v>
       </ns0:c>
-      <ns0:c r="DD3" s="26" t="s">
+      <ns0:c r="DE3" s="26" t="s">
         <ns0:v>162</ns0:v>
       </ns0:c>
-      <ns0:c r="DE3" s="26" t="s">
+      <ns0:c r="DF3" s="26" t="s">
         <ns0:v>247</ns0:v>
       </ns0:c>
-      <ns0:c r="DF3" s="26" t="s">
+      <ns0:c r="DG3" s="26" t="s">
         <ns0:v>300</ns0:v>
       </ns0:c>
-      <ns0:c r="DG3" s="26" t="s">
+      <ns0:c r="DH3" s="26" t="s">
         <ns0:v>160</ns0:v>
       </ns0:c>
-      <ns0:c r="DH3" s="26" t="s">
+      <ns0:c r="DI3" s="26" t="s">
         <ns0:v>162</ns0:v>
       </ns0:c>
-      <ns0:c r="DI3" s="26" t="s">
+      <ns0:c r="DJ3" s="26" t="s">
         <ns0:v>247</ns0:v>
       </ns0:c>
-      <ns0:c r="DJ3" s="26" t="s">
+      <ns0:c r="DK3" s="26" t="s">
         <ns0:v>300</ns0:v>
       </ns0:c>
-      <ns0:c r="DK3" s="26" t="s">
+      <ns0:c r="DL3" s="26" t="s">
         <ns0:v>161</ns0:v>
       </ns0:c>
-      <ns0:c r="DL3" s="26" t="s">
+      <ns0:c r="DM3" s="26" t="s">
         <ns0:v>163</ns0:v>
       </ns0:c>
-      <ns0:c r="DM3" s="26" t="s">
+      <ns0:c r="DN3" s="26" t="s">
         <ns0:v>267</ns0:v>
       </ns0:c>
-      <ns0:c r="DN3" s="26" t="s">
+      <ns0:c r="DO3" s="26" t="s">
         <ns0:v>269</ns0:v>
       </ns0:c>
-      <ns0:c r="DO3" s="26" t="s">
+      <ns0:c r="DP3" s="26" t="s">
         <ns0:v>161</ns0:v>
       </ns0:c>
-      <ns0:c r="DP3" s="26" t="s">
+      <ns0:c r="DQ3" s="26" t="s">
         <ns0:v>163</ns0:v>
       </ns0:c>
-      <ns0:c r="DQ3" s="26" t="s">
+      <ns0:c r="DR3" s="26" t="s">
         <ns0:v>267</ns0:v>
       </ns0:c>
-      <ns0:c r="DR3" s="26" t="s">
+      <ns0:c r="DS3" s="26" t="s">
         <ns0:v>269</ns0:v>
       </ns0:c>
-      <ns0:c r="DS3" s="26" t="s">
+      <ns0:c r="DT3" s="26" t="s">
         <ns0:v>165</ns0:v>
       </ns0:c>
-      <ns0:c r="DT3" s="26" t="s">
+      <ns0:c r="DU3" s="26" t="s">
         <ns0:v>164</ns0:v>
       </ns0:c>
-      <ns0:c r="DU3" s="26" t="s">
+      <ns0:c r="DV3" s="26" t="s">
         <ns0:v>271</ns0:v>
       </ns0:c>
-      <ns0:c r="DV3" s="26" t="s">
+      <ns0:c r="DW3" s="26" t="s">
         <ns0:v>166</ns0:v>
       </ns0:c>
-      <ns0:c r="DW3" s="26" t="s">
+      <ns0:c r="DX3" s="26" t="s">
         <ns0:v>165</ns0:v>
       </ns0:c>
-      <ns0:c r="DX3" s="26" t="s">
+      <ns0:c r="DY3" s="26" t="s">
         <ns0:v>164</ns0:v>
       </ns0:c>
-      <ns0:c r="DY3" s="26" t="s">
+      <ns0:c r="DZ3" s="26" t="s">
         <ns0:v>271</ns0:v>
       </ns0:c>
-      <ns0:c r="DZ3" s="26" t="s">
+      <ns0:c r="EA3" s="26" t="s">
         <ns0:v>166</ns0:v>
       </ns0:c>
-      <ns0:c r="EA3" s="26" t="s">
+      <ns0:c r="EB3" s="26" t="s">
         <ns0:v>165</ns0:v>
       </ns0:c>
-      <ns0:c r="EB3" s="26" t="s">
+      <ns0:c r="EC3" s="26" t="s">
         <ns0:v>164</ns0:v>
       </ns0:c>
-      <ns0:c r="EC3" s="26" t="s">
+      <ns0:c r="ED3" s="26" t="s">
         <ns0:v>271</ns0:v>
       </ns0:c>
-      <ns0:c r="ED3" s="26" t="s">
+      <ns0:c r="EE3" s="26" t="s">
         <ns0:v>166</ns0:v>
       </ns0:c>
-      <ns0:c r="EE3" t="s">
+      <ns0:c r="EF3" t="s">
         <ns0:v>544</ns0:v>
       </ns0:c>
-      <ns0:c r="EF3" s="61" t="s">
+      <ns0:c r="EG3" s="61" t="s">
         <ns0:v>151</ns0:v>
       </ns0:c>
-      <ns0:c r="EG3" s="61" t="s">
+      <ns0:c r="EH3" s="61" t="s">
         <ns0:v>397</ns0:v>
       </ns0:c>
-      <ns0:c r="EH3" s="61" t="s">
+      <ns0:c r="EI3" s="61" t="s">
         <ns0:v>398</ns0:v>
       </ns0:c>
-      <ns0:c r="EI3" s="61" t="s">
+      <ns0:c r="EJ3" s="61" t="s">
         <ns0:v>167</ns0:v>
       </ns0:c>
-      <ns0:c r="EJ3" s="61" t="s">
+      <ns0:c r="EK3" s="61" t="s">
         <ns0:v>151</ns0:v>
       </ns0:c>
-      <ns0:c r="EK3" s="61" t="s">
+      <ns0:c r="EL3" s="61" t="s">
         <ns0:v>407</ns0:v>
       </ns0:c>
-      <ns0:c r="EL3" s="61" t="s">
+      <ns0:c r="EM3" s="61" t="s">
         <ns0:v>406</ns0:v>
       </ns0:c>
-      <ns0:c r="EM3" s="61" t="s">
+      <ns0:c r="EN3" s="61" t="s">
         <ns0:v>167</ns0:v>
       </ns0:c>
-      <ns0:c r="EN3" s="25" t="s">
+      <ns0:c r="EO3" s="25" t="s">
         <ns0:v>125</ns0:v>
       </ns0:c>
-      <ns0:c r="EO3" s="58" t="s">
+      <ns0:c r="EP3" s="58" t="s">
         <ns0:v>227</ns0:v>
       </ns0:c>
-      <ns0:c r="EP3" s="68" t="s">
+      <ns0:c r="EQ3" s="68" t="s">
         <ns0:v>428</ns0:v>
       </ns0:c>
-      <ns0:c r="EQ3" s="25" t="s">
+      <ns0:c r="ER3" s="25" t="s">
         <ns0:v>126</ns0:v>
       </ns0:c>
-      <ns0:c r="ER3" s="58" t="s">
+      <ns0:c r="ES3" s="58" t="s">
         <ns0:v>225</ns0:v>
       </ns0:c>
-      <ns0:c r="ES3" s="68" t="s">
+      <ns0:c r="ET3" s="68" t="s">
         <ns0:v>430</ns0:v>
       </ns0:c>
-      <ns0:c r="ET3" s="58" t="s">
+      <ns0:c r="EU3" s="58" t="s">
         <ns0:v>418</ns0:v>
       </ns0:c>
-      <ns0:c r="EU3" s="58" t="s">
+      <ns0:c r="EV3" s="58" t="s">
         <ns0:v>419</ns0:v>
       </ns0:c>
-      <ns0:c r="EV3" s="68" t="s">
+      <ns0:c r="EW3" s="68" t="s">
         <ns0:v>446</ns0:v>
       </ns0:c>
-      <ns0:c r="EW3" s="25" t="s">
+      <ns0:c r="EX3" s="25" t="s">
         <ns0:v>127</ns0:v>
       </ns0:c>
-      <ns0:c r="EX3" s="58" t="s">
+      <ns0:c r="EY3" s="58" t="s">
         <ns0:v>223</ns0:v>
       </ns0:c>
-      <ns0:c r="EY3" s="68" t="s">
+      <ns0:c r="EZ3" s="68" t="s">
         <ns0:v>432</ns0:v>
       </ns0:c>
-      <ns0:c r="EZ3" s="25" t="s">
+      <ns0:c r="FA3" s="25" t="s">
         <ns0:v>128</ns0:v>
       </ns0:c>
-      <ns0:c r="FA3" s="58" t="s">
+      <ns0:c r="FB3" s="58" t="s">
         <ns0:v>221</ns0:v>
       </ns0:c>
-      <ns0:c r="FB3" s="68" t="s">
+      <ns0:c r="FC3" s="68" t="s">
         <ns0:v>434</ns0:v>
       </ns0:c>
-      <ns0:c r="FC3" s="25" t="s">
+      <ns0:c r="FD3" s="25" t="s">
         <ns0:v>129</ns0:v>
       </ns0:c>
-      <ns0:c r="FD3" s="58" t="s">
+      <ns0:c r="FE3" s="58" t="s">
         <ns0:v>219</ns0:v>
       </ns0:c>
-      <ns0:c r="FE3" s="68" t="s">
+      <ns0:c r="FF3" s="68" t="s">
         <ns0:v>436</ns0:v>
       </ns0:c>
-      <ns0:c r="FF3" s="25" t="s">
+      <ns0:c r="FG3" s="25" t="s">
         <ns0:v>130</ns0:v>
       </ns0:c>
-      <ns0:c r="FG3" s="58" t="s">
+      <ns0:c r="FH3" s="58" t="s">
         <ns0:v>217</ns0:v>
       </ns0:c>
-      <ns0:c r="FH3" s="68" t="s">
+      <ns0:c r="FI3" s="68" t="s">
         <ns0:v>447</ns0:v>
       </ns0:c>
-      <ns0:c r="FI3" s="25" t="s">
+      <ns0:c r="FJ3" s="25" t="s">
         <ns0:v>131</ns0:v>
       </ns0:c>
-      <ns0:c r="FJ3" s="58" t="s">
+      <ns0:c r="FK3" s="58" t="s">
         <ns0:v>215</ns0:v>
       </ns0:c>
-      <ns0:c r="FK3" s="68" t="s">
+      <ns0:c r="FL3" s="68" t="s">
         <ns0:v>449</ns0:v>
       </ns0:c>
-      <ns0:c r="FL3" s="25" t="s">
+      <ns0:c r="FM3" s="25" t="s">
         <ns0:v>132</ns0:v>
       </ns0:c>
-      <ns0:c r="FM3" s="58" t="s">
+      <ns0:c r="FN3" s="58" t="s">
         <ns0:v>213</ns0:v>
       </ns0:c>
-      <ns0:c r="FN3" s="68" t="s">
+      <ns0:c r="FO3" s="68" t="s">
         <ns0:v>451</ns0:v>
       </ns0:c>
-      <ns0:c r="FO3" s="25" t="s">
+      <ns0:c r="FP3" s="25" t="s">
         <ns0:v>133</ns0:v>
       </ns0:c>
-      <ns0:c r="FP3" s="58" t="s">
+      <ns0:c r="FQ3" s="58" t="s">
         <ns0:v>211</ns0:v>
       </ns0:c>
-      <ns0:c r="FQ3" s="68" t="s">
+      <ns0:c r="FR3" s="68" t="s">
         <ns0:v>453</ns0:v>
       </ns0:c>
-      <ns0:c r="FR3" s="25" t="s">
+      <ns0:c r="FS3" s="25" t="s">
         <ns0:v>135</ns0:v>
       </ns0:c>
-      <ns0:c r="FS3" s="58" t="s">
+      <ns0:c r="FT3" s="58" t="s">
         <ns0:v>209</ns0:v>
       </ns0:c>
-      <ns0:c r="FT3" s="25" t="s">
+      <ns0:c r="FU3" s="25" t="s">
         <ns0:v>136</ns0:v>
       </ns0:c>
-      <ns0:c r="FU3" s="68" t="s">
+      <ns0:c r="FV3" s="68" t="s">
         <ns0:v>461</ns0:v>
       </ns0:c>
-      <ns0:c r="FV3" s="58" t="s">
+      <ns0:c r="FW3" s="58" t="s">
         <ns0:v>207</ns0:v>
       </ns0:c>
-      <ns0:c r="FW3" s="68" t="s">
+      <ns0:c r="FX3" s="68" t="s">
         <ns0:v>455</ns0:v>
       </ns0:c>
-      <ns0:c r="FX3" s="25" t="s">
+      <ns0:c r="FY3" s="25" t="s">
         <ns0:v>137</ns0:v>
       </ns0:c>
-      <ns0:c r="FY3" s="58" t="s">
+      <ns0:c r="FZ3" s="58" t="s">
         <ns0:v>205</ns0:v>
       </ns0:c>
-      <ns0:c r="FZ3" s="68" t="s">
+      <ns0:c r="GA3" s="68" t="s">
         <ns0:v>457</ns0:v>
       </ns0:c>
-      <ns0:c r="GA3" s="25" t="s">
+      <ns0:c r="GB3" s="25" t="s">
         <ns0:v>138</ns0:v>
       </ns0:c>
-      <ns0:c r="GB3" s="58" t="s">
+      <ns0:c r="GC3" s="58" t="s">
         <ns0:v>204</ns0:v>
       </ns0:c>
-      <ns0:c r="GC3" s="68" t="s">
+      <ns0:c r="GD3" s="68" t="s">
         <ns0:v>438</ns0:v>
       </ns0:c>
-      <ns0:c r="GD3" s="25" t="s">
+      <ns0:c r="GE3" s="25" t="s">
         <ns0:v>139</ns0:v>
       </ns0:c>
-      <ns0:c r="GE3" s="58" t="s">
+      <ns0:c r="GF3" s="58" t="s">
         <ns0:v>200</ns0:v>
       </ns0:c>
-      <ns0:c r="GF3" s="68" t="s">
+      <ns0:c r="GG3" s="68" t="s">
         <ns0:v>440</ns0:v>
       </ns0:c>
-      <ns0:c r="GG3" s="25" t="s">
+      <ns0:c r="GH3" s="25" t="s">
         <ns0:v>141</ns0:v>
       </ns0:c>
-      <ns0:c r="GH3" s="58" t="s">
+      <ns0:c r="GI3" s="58" t="s">
         <ns0:v>199</ns0:v>
       </ns0:c>
-      <ns0:c r="GI3" s="68" t="s">
+      <ns0:c r="GJ3" s="68" t="s">
         <ns0:v>442</ns0:v>
       </ns0:c>
-      <ns0:c r="GJ3" s="25" t="s">
+      <ns0:c r="GK3" s="25" t="s">
         <ns0:v>143</ns0:v>
       </ns0:c>
-      <ns0:c r="GK3" s="58" t="s">
+      <ns0:c r="GL3" s="58" t="s">
         <ns0:v>197</ns0:v>
       </ns0:c>
-      <ns0:c r="GL3" s="68" t="s">
+      <ns0:c r="GM3" s="68" t="s">
         <ns0:v>444</ns0:v>
       </ns0:c>
-      <ns0:c r="GM3" s="25" t="s">
+      <ns0:c r="GN3" s="25" t="s">
         <ns0:v>145</ns0:v>
       </ns0:c>
-      <ns0:c r="GN3" s="58" t="s">
+      <ns0:c r="GO3" s="58" t="s">
         <ns0:v>195</ns0:v>
       </ns0:c>
-      <ns0:c r="GO3" s="68" t="s">
+      <ns0:c r="GP3" s="68" t="s">
         <ns0:v>459</ns0:v>
       </ns0:c>
-      <ns0:c r="GP3" s="68" t="s">
+      <ns0:c r="GQ3" s="68" t="s">
         <ns0:v>520</ns0:v>
       </ns0:c>
-      <ns0:c r="GQ3" s="68" t="s">
+      <ns0:c r="GR3" s="68" t="s">
         <ns0:v>521</ns0:v>
       </ns0:c>
     </ns0:row>
-    <ns0:row r="4" spans="1:198" s="59" customFormat="1" ht="56.25" customHeight="1" thickTop="1" thickBot="1" ns3:dyDescent="0.25">
+    <ns0:row r="4" spans="1:199" s="59" customFormat="1" ht="56.25" customHeight="1" thickTop="1" thickBot="1" ns3:dyDescent="0.25">
       <ns0:c r="A4" s="35" t="s">
         <ns0:v>5</ns0:v>
       </ns0:c>
@@ -4545,401 +4564,404 @@
       <ns0:c r="BP4" s="37" t="s">
         <ns0:v>424</ns0:v>
       </ns0:c>
-      <ns0:c r="BQ4" s="69" t="s">
+      <ns0:c r="BQ4" s="37" t="s">
+        <ns0:v>652</ns0:v>
+      </ns0:c>
+      <ns0:c r="BR4" s="69" t="s">
         <ns0:v>597</ns0:v>
       </ns0:c>
-      <ns0:c r="BR4" s="69" t="s">
+      <ns0:c r="BS4" s="69" t="s">
         <ns0:v>598</ns0:v>
       </ns0:c>
-      <ns0:c r="BS4" s="69" t="s">
+      <ns0:c r="BT4" s="69" t="s">
         <ns0:v>599</ns0:v>
       </ns0:c>
-      <ns0:c r="BT4" s="69" t="s">
+      <ns0:c r="BU4" s="69" t="s">
         <ns0:v>600</ns0:v>
       </ns0:c>
-      <ns0:c r="BU4" s="69" t="s">
+      <ns0:c r="BV4" s="69" t="s">
         <ns0:v>601</ns0:v>
       </ns0:c>
-      <ns0:c r="BV4" s="69" t="s">
+      <ns0:c r="BW4" s="69" t="s">
         <ns0:v>602</ns0:v>
       </ns0:c>
-      <ns0:c r="BW4" s="69" t="s">
+      <ns0:c r="BX4" s="69" t="s">
         <ns0:v>603</ns0:v>
       </ns0:c>
-      <ns0:c r="BX4" s="69" t="s">
+      <ns0:c r="BY4" s="69" t="s">
         <ns0:v>604</ns0:v>
       </ns0:c>
-      <ns0:c r="BY4" s="69" t="s">
+      <ns0:c r="BZ4" s="69" t="s">
         <ns0:v>605</ns0:v>
       </ns0:c>
-      <ns0:c r="BZ4" s="69" t="s">
+      <ns0:c r="CA4" s="69" t="s">
         <ns0:v>606</ns0:v>
       </ns0:c>
-      <ns0:c r="CA4" s="69" t="s">
+      <ns0:c r="CB4" s="69" t="s">
         <ns0:v>607</ns0:v>
       </ns0:c>
-      <ns0:c r="CB4" s="69" t="s">
+      <ns0:c r="CC4" s="69" t="s">
         <ns0:v>608</ns0:v>
       </ns0:c>
-      <ns0:c r="CC4" s="69" t="s">
+      <ns0:c r="CD4" s="69" t="s">
         <ns0:v>609</ns0:v>
       </ns0:c>
-      <ns0:c r="CD4" s="69" t="s">
+      <ns0:c r="CE4" s="69" t="s">
         <ns0:v>610</ns0:v>
       </ns0:c>
-      <ns0:c r="CE4" s="69" t="s">
+      <ns0:c r="CF4" s="69" t="s">
         <ns0:v>611</ns0:v>
       </ns0:c>
-      <ns0:c r="CF4" s="69" t="s">
+      <ns0:c r="CG4" s="69" t="s">
         <ns0:v>612</ns0:v>
       </ns0:c>
-      <ns0:c r="CG4" s="69" t="s">
+      <ns0:c r="CH4" s="69" t="s">
         <ns0:v>613</ns0:v>
       </ns0:c>
-      <ns0:c r="CH4" s="69" t="s">
+      <ns0:c r="CI4" s="69" t="s">
         <ns0:v>614</ns0:v>
       </ns0:c>
-      <ns0:c r="CI4" s="69" t="s">
+      <ns0:c r="CJ4" s="69" t="s">
         <ns0:v>615</ns0:v>
       </ns0:c>
-      <ns0:c r="CJ4" s="69" t="s">
+      <ns0:c r="CK4" s="69" t="s">
         <ns0:v>616</ns0:v>
       </ns0:c>
-      <ns0:c r="CK4" s="69" t="s">
+      <ns0:c r="CL4" s="69" t="s">
         <ns0:v>617</ns0:v>
       </ns0:c>
-      <ns0:c r="CL4" s="69" t="s">
+      <ns0:c r="CM4" s="69" t="s">
         <ns0:v>618</ns0:v>
       </ns0:c>
-      <ns0:c r="CM4" s="69" t="s">
+      <ns0:c r="CN4" s="69" t="s">
         <ns0:v>619</ns0:v>
       </ns0:c>
-      <ns0:c r="CN4" s="69" t="s">
+      <ns0:c r="CO4" s="69" t="s">
         <ns0:v>620</ns0:v>
       </ns0:c>
-      <ns0:c r="CO4" s="69" t="s">
+      <ns0:c r="CP4" s="69" t="s">
         <ns0:v>621</ns0:v>
       </ns0:c>
-      <ns0:c r="CP4" s="69" t="s">
+      <ns0:c r="CQ4" s="69" t="s">
         <ns0:v>622</ns0:v>
       </ns0:c>
-      <ns0:c r="CQ4" s="37" t="s">
+      <ns0:c r="CR4" s="37" t="s">
         <ns0:v>184</ns0:v>
       </ns0:c>
-      <ns0:c r="CR4" s="37" t="s">
+      <ns0:c r="CS4" s="37" t="s">
         <ns0:v>168</ns0:v>
       </ns0:c>
-      <ns0:c r="CS4" s="37" t="s">
+      <ns0:c r="CT4" s="37" t="s">
         <ns0:v>248</ns0:v>
       </ns0:c>
-      <ns0:c r="CT4" s="37" t="s">
+      <ns0:c r="CU4" s="37" t="s">
         <ns0:v>169</ns0:v>
       </ns0:c>
-      <ns0:c r="CU4" s="37" t="s">
+      <ns0:c r="CV4" s="37" t="s">
         <ns0:v>170</ns0:v>
       </ns0:c>
-      <ns0:c r="CV4" s="37" t="s">
+      <ns0:c r="CW4" s="37" t="s">
         <ns0:v>171</ns0:v>
       </ns0:c>
-      <ns0:c r="CW4" s="37" t="s">
+      <ns0:c r="CX4" s="37" t="s">
         <ns0:v>262</ns0:v>
       </ns0:c>
-      <ns0:c r="CX4" s="37" t="s">
+      <ns0:c r="CY4" s="37" t="s">
         <ns0:v>172</ns0:v>
       </ns0:c>
-      <ns0:c r="CY4" s="37" t="s">
+      <ns0:c r="CZ4" s="37" t="s">
         <ns0:v>173</ns0:v>
       </ns0:c>
-      <ns0:c r="CZ4" s="37" t="s">
+      <ns0:c r="DA4" s="37" t="s">
         <ns0:v>174</ns0:v>
       </ns0:c>
-      <ns0:c r="DA4" s="37" t="s">
+      <ns0:c r="DB4" s="37" t="s">
         <ns0:v>265</ns0:v>
       </ns0:c>
-      <ns0:c r="DB4" s="37" t="s">
+      <ns0:c r="DC4" s="37" t="s">
         <ns0:v>175</ns0:v>
       </ns0:c>
-      <ns0:c r="DC4" s="37" t="s">
+      <ns0:c r="DD4" s="37" t="s">
         <ns0:v>301</ns0:v>
       </ns0:c>
-      <ns0:c r="DD4" s="37" t="s">
+      <ns0:c r="DE4" s="37" t="s">
         <ns0:v>303</ns0:v>
       </ns0:c>
-      <ns0:c r="DE4" s="37" t="s">
+      <ns0:c r="DF4" s="37" t="s">
         <ns0:v>305</ns0:v>
       </ns0:c>
-      <ns0:c r="DF4" s="37" t="s">
+      <ns0:c r="DG4" s="37" t="s">
         <ns0:v>307</ns0:v>
       </ns0:c>
-      <ns0:c r="DG4" s="37" t="s">
+      <ns0:c r="DH4" s="37" t="s">
         <ns0:v>309</ns0:v>
       </ns0:c>
-      <ns0:c r="DH4" s="37" t="s">
+      <ns0:c r="DI4" s="37" t="s">
         <ns0:v>311</ns0:v>
       </ns0:c>
-      <ns0:c r="DI4" s="37" t="s">
+      <ns0:c r="DJ4" s="37" t="s">
         <ns0:v>313</ns0:v>
       </ns0:c>
-      <ns0:c r="DJ4" s="37" t="s">
+      <ns0:c r="DK4" s="37" t="s">
         <ns0:v>315</ns0:v>
       </ns0:c>
-      <ns0:c r="DK4" s="37" t="s">
+      <ns0:c r="DL4" s="37" t="s">
         <ns0:v>185</ns0:v>
       </ns0:c>
-      <ns0:c r="DL4" s="37" t="s">
+      <ns0:c r="DM4" s="37" t="s">
         <ns0:v>186</ns0:v>
       </ns0:c>
-      <ns0:c r="DM4" s="37" t="s">
+      <ns0:c r="DN4" s="37" t="s">
         <ns0:v>268</ns0:v>
       </ns0:c>
-      <ns0:c r="DN4" s="37" t="s">
+      <ns0:c r="DO4" s="37" t="s">
         <ns0:v>187</ns0:v>
       </ns0:c>
-      <ns0:c r="DO4" s="37" t="s">
+      <ns0:c r="DP4" s="37" t="s">
         <ns0:v>281</ns0:v>
       </ns0:c>
-      <ns0:c r="DP4" s="37" t="s">
+      <ns0:c r="DQ4" s="37" t="s">
         <ns0:v>284</ns0:v>
       </ns0:c>
-      <ns0:c r="DQ4" s="37" t="s">
+      <ns0:c r="DR4" s="37" t="s">
         <ns0:v>286</ns0:v>
       </ns0:c>
-      <ns0:c r="DR4" s="37" t="s">
+      <ns0:c r="DS4" s="37" t="s">
         <ns0:v>288</ns0:v>
       </ns0:c>
-      <ns0:c r="DS4" s="37" t="s">
+      <ns0:c r="DT4" s="37" t="s">
         <ns0:v>176</ns0:v>
       </ns0:c>
-      <ns0:c r="DT4" s="37" t="s">
+      <ns0:c r="DU4" s="37" t="s">
         <ns0:v>177</ns0:v>
       </ns0:c>
-      <ns0:c r="DU4" s="37" t="s">
+      <ns0:c r="DV4" s="37" t="s">
         <ns0:v>272</ns0:v>
       </ns0:c>
-      <ns0:c r="DV4" s="37" t="s">
+      <ns0:c r="DW4" s="37" t="s">
         <ns0:v>178</ns0:v>
       </ns0:c>
-      <ns0:c r="DW4" s="37" t="s">
+      <ns0:c r="DX4" s="37" t="s">
         <ns0:v>179</ns0:v>
       </ns0:c>
-      <ns0:c r="DX4" s="37" t="s">
+      <ns0:c r="DY4" s="37" t="s">
         <ns0:v>181</ns0:v>
       </ns0:c>
-      <ns0:c r="DY4" s="37" t="s">
+      <ns0:c r="DZ4" s="37" t="s">
         <ns0:v>273</ns0:v>
       </ns0:c>
-      <ns0:c r="DZ4" s="37" t="s">
+      <ns0:c r="EA4" s="37" t="s">
         <ns0:v>180</ns0:v>
       </ns0:c>
-      <ns0:c r="EA4" s="37" t="s">
+      <ns0:c r="EB4" s="37" t="s">
         <ns0:v>292</ns0:v>
       </ns0:c>
-      <ns0:c r="EB4" s="37" t="s">
+      <ns0:c r="EC4" s="37" t="s">
         <ns0:v>294</ns0:v>
       </ns0:c>
-      <ns0:c r="EC4" s="37" t="s">
+      <ns0:c r="ED4" s="37" t="s">
         <ns0:v>296</ns0:v>
       </ns0:c>
-      <ns0:c r="ED4" s="37" t="s">
+      <ns0:c r="EE4" s="37" t="s">
         <ns0:v>298</ns0:v>
       </ns0:c>
-      <ns0:c r="EE4" t="s">
+      <ns0:c r="EF4" t="s">
         <ns0:v>541</ns0:v>
       </ns0:c>
-      <ns0:c r="EF4" s="37" t="s">
+      <ns0:c r="EG4" s="37" t="s">
         <ns0:v>152</ns0:v>
       </ns0:c>
-      <ns0:c r="EG4" s="37" t="s">
+      <ns0:c r="EH4" s="37" t="s">
         <ns0:v>109</ns0:v>
       </ns0:c>
-      <ns0:c r="EH4" s="37" t="s">
+      <ns0:c r="EI4" s="37" t="s">
         <ns0:v>110</ns0:v>
       </ns0:c>
-      <ns0:c r="EI4" s="37" t="s">
+      <ns0:c r="EJ4" s="37" t="s">
         <ns0:v>154</ns0:v>
       </ns0:c>
-      <ns0:c r="EJ4" s="37" t="s">
+      <ns0:c r="EK4" s="37" t="s">
         <ns0:v>153</ns0:v>
       </ns0:c>
-      <ns0:c r="EK4" s="37" t="s">
+      <ns0:c r="EL4" s="37" t="s">
         <ns0:v>111</ns0:v>
       </ns0:c>
-      <ns0:c r="EL4" s="37" t="s">
+      <ns0:c r="EM4" s="37" t="s">
         <ns0:v>112</ns0:v>
       </ns0:c>
-      <ns0:c r="EM4" s="37" t="s">
+      <ns0:c r="EN4" s="37" t="s">
         <ns0:v>155</ns0:v>
       </ns0:c>
-      <ns0:c r="EN4" s="37" t="s">
+      <ns0:c r="EO4" s="37" t="s">
         <ns0:v>45</ns0:v>
       </ns0:c>
-      <ns0:c r="EO4" s="37" t="s">
+      <ns0:c r="EP4" s="37" t="s">
         <ns0:v>229</ns0:v>
       </ns0:c>
-      <ns0:c r="EP4" s="69" t="s">
+      <ns0:c r="EQ4" s="69" t="s">
         <ns0:v>429</ns0:v>
       </ns0:c>
-      <ns0:c r="EQ4" s="37" t="s">
+      <ns0:c r="ER4" s="37" t="s">
         <ns0:v>49</ns0:v>
       </ns0:c>
-      <ns0:c r="ER4" s="37" t="s">
+      <ns0:c r="ES4" s="37" t="s">
         <ns0:v>230</ns0:v>
       </ns0:c>
-      <ns0:c r="ES4" s="69" t="s">
+      <ns0:c r="ET4" s="69" t="s">
         <ns0:v>431</ns0:v>
       </ns0:c>
-      <ns0:c r="ET4" s="37" t="s">
+      <ns0:c r="EU4" s="37" t="s">
         <ns0:v>420</ns0:v>
       </ns0:c>
-      <ns0:c r="EU4" s="37" t="s">
+      <ns0:c r="EV4" s="37" t="s">
         <ns0:v>421</ns0:v>
       </ns0:c>
-      <ns0:c r="EV4" s="69" t="s">
+      <ns0:c r="EW4" s="69" t="s">
         <ns0:v>522</ns0:v>
       </ns0:c>
-      <ns0:c r="EW4" s="40" t="s">
+      <ns0:c r="EX4" s="40" t="s">
         <ns0:v>52</ns0:v>
       </ns0:c>
-      <ns0:c r="EX4" s="37" t="s">
+      <ns0:c r="EY4" s="37" t="s">
         <ns0:v>231</ns0:v>
       </ns0:c>
-      <ns0:c r="EY4" s="69" t="s">
+      <ns0:c r="EZ4" s="69" t="s">
         <ns0:v>433</ns0:v>
       </ns0:c>
-      <ns0:c r="EZ4" s="37" t="s">
+      <ns0:c r="FA4" s="37" t="s">
         <ns0:v>47</ns0:v>
       </ns0:c>
-      <ns0:c r="FA4" s="37" t="s">
+      <ns0:c r="FB4" s="37" t="s">
         <ns0:v>232</ns0:v>
       </ns0:c>
-      <ns0:c r="FB4" s="69" t="s">
+      <ns0:c r="FC4" s="69" t="s">
         <ns0:v>435</ns0:v>
       </ns0:c>
-      <ns0:c r="FC4" s="37" t="s">
+      <ns0:c r="FD4" s="37" t="s">
         <ns0:v>48</ns0:v>
       </ns0:c>
-      <ns0:c r="FD4" s="37" t="s">
+      <ns0:c r="FE4" s="37" t="s">
         <ns0:v>233</ns0:v>
       </ns0:c>
-      <ns0:c r="FE4" s="69" t="s">
+      <ns0:c r="FF4" s="69" t="s">
         <ns0:v>437</ns0:v>
       </ns0:c>
-      <ns0:c r="FF4" s="40" t="s">
+      <ns0:c r="FG4" s="40" t="s">
         <ns0:v>51</ns0:v>
       </ns0:c>
-      <ns0:c r="FG4" s="37" t="s">
+      <ns0:c r="FH4" s="37" t="s">
         <ns0:v>234</ns0:v>
       </ns0:c>
-      <ns0:c r="FH4" s="69" t="s">
+      <ns0:c r="FI4" s="69" t="s">
         <ns0:v>448</ns0:v>
       </ns0:c>
-      <ns0:c r="FI4" s="40" t="s">
+      <ns0:c r="FJ4" s="40" t="s">
         <ns0:v>102</ns0:v>
       </ns0:c>
-      <ns0:c r="FJ4" s="37" t="s">
+      <ns0:c r="FK4" s="37" t="s">
         <ns0:v>235</ns0:v>
       </ns0:c>
-      <ns0:c r="FK4" s="69" t="s">
+      <ns0:c r="FL4" s="69" t="s">
         <ns0:v>450</ns0:v>
       </ns0:c>
-      <ns0:c r="FL4" s="40" t="s">
+      <ns0:c r="FM4" s="40" t="s">
         <ns0:v>55</ns0:v>
       </ns0:c>
-      <ns0:c r="FM4" s="37" t="s">
+      <ns0:c r="FN4" s="37" t="s">
         <ns0:v>236</ns0:v>
       </ns0:c>
-      <ns0:c r="FN4" s="69" t="s">
+      <ns0:c r="FO4" s="69" t="s">
         <ns0:v>452</ns0:v>
       </ns0:c>
-      <ns0:c r="FO4" s="37" t="s">
+      <ns0:c r="FP4" s="37" t="s">
         <ns0:v>50</ns0:v>
       </ns0:c>
-      <ns0:c r="FP4" s="37" t="s">
+      <ns0:c r="FQ4" s="37" t="s">
         <ns0:v>238</ns0:v>
       </ns0:c>
-      <ns0:c r="FQ4" s="69" t="s">
+      <ns0:c r="FR4" s="69" t="s">
         <ns0:v>454</ns0:v>
       </ns0:c>
-      <ns0:c r="FR4" s="37" t="s">
+      <ns0:c r="FS4" s="37" t="s">
         <ns0:v>103</ns0:v>
       </ns0:c>
-      <ns0:c r="FS4" s="37" t="s">
+      <ns0:c r="FT4" s="37" t="s">
         <ns0:v>239</ns0:v>
       </ns0:c>
-      <ns0:c r="FT4" s="37" t="s">
+      <ns0:c r="FU4" s="37" t="s">
         <ns0:v>104</ns0:v>
       </ns0:c>
-      <ns0:c r="FU4" s="69" t="s">
+      <ns0:c r="FV4" s="69" t="s">
         <ns0:v>462</ns0:v>
       </ns0:c>
-      <ns0:c r="FV4" s="37" t="s">
+      <ns0:c r="FW4" s="37" t="s">
         <ns0:v>240</ns0:v>
       </ns0:c>
-      <ns0:c r="FW4" s="69" t="s">
+      <ns0:c r="FX4" s="69" t="s">
         <ns0:v>456</ns0:v>
       </ns0:c>
-      <ns0:c r="FX4" s="40" t="s">
+      <ns0:c r="FY4" s="40" t="s">
         <ns0:v>77</ns0:v>
       </ns0:c>
-      <ns0:c r="FY4" s="37" t="s">
+      <ns0:c r="FZ4" s="37" t="s">
         <ns0:v>241</ns0:v>
       </ns0:c>
-      <ns0:c r="FZ4" s="69" t="s">
+      <ns0:c r="GA4" s="69" t="s">
         <ns0:v>458</ns0:v>
       </ns0:c>
-      <ns0:c r="GA4" s="37" t="s">
+      <ns0:c r="GB4" s="37" t="s">
         <ns0:v>46</ns0:v>
       </ns0:c>
-      <ns0:c r="GB4" s="37" t="s">
+      <ns0:c r="GC4" s="37" t="s">
         <ns0:v>242</ns0:v>
       </ns0:c>
-      <ns0:c r="GC4" s="69" t="s">
+      <ns0:c r="GD4" s="69" t="s">
         <ns0:v>439</ns0:v>
       </ns0:c>
-      <ns0:c r="GD4" s="40" t="s">
+      <ns0:c r="GE4" s="40" t="s">
         <ns0:v>57</ns0:v>
       </ns0:c>
-      <ns0:c r="GE4" s="37" t="s">
+      <ns0:c r="GF4" s="37" t="s">
         <ns0:v>243</ns0:v>
       </ns0:c>
-      <ns0:c r="GF4" s="69" t="s">
+      <ns0:c r="GG4" s="69" t="s">
         <ns0:v>441</ns0:v>
       </ns0:c>
-      <ns0:c r="GG4" s="37" t="s">
+      <ns0:c r="GH4" s="37" t="s">
         <ns0:v>76</ns0:v>
       </ns0:c>
-      <ns0:c r="GH4" s="37" t="s">
+      <ns0:c r="GI4" s="37" t="s">
         <ns0:v>244</ns0:v>
       </ns0:c>
-      <ns0:c r="GI4" s="69" t="s">
+      <ns0:c r="GJ4" s="69" t="s">
         <ns0:v>443</ns0:v>
       </ns0:c>
-      <ns0:c r="GJ4" s="40" t="s">
+      <ns0:c r="GK4" s="40" t="s">
         <ns0:v>56</ns0:v>
       </ns0:c>
-      <ns0:c r="GK4" s="40" t="s">
+      <ns0:c r="GL4" s="40" t="s">
         <ns0:v>245</ns0:v>
       </ns0:c>
-      <ns0:c r="GL4" s="69" t="s">
+      <ns0:c r="GM4" s="69" t="s">
         <ns0:v>445</ns0:v>
       </ns0:c>
-      <ns0:c r="GM4" s="40" t="s">
+      <ns0:c r="GN4" s="40" t="s">
         <ns0:v>54</ns0:v>
       </ns0:c>
-      <ns0:c r="GN4" s="37" t="s">
+      <ns0:c r="GO4" s="37" t="s">
         <ns0:v>246</ns0:v>
       </ns0:c>
-      <ns0:c r="GO4" s="69" t="s">
+      <ns0:c r="GP4" s="69" t="s">
         <ns0:v>460</ns0:v>
       </ns0:c>
-      <ns0:c r="GP4" s="69" t="s">
+      <ns0:c r="GQ4" s="69" t="s">
         <ns0:v>518</ns0:v>
       </ns0:c>
-      <ns0:c r="GQ4" s="69" t="s">
+      <ns0:c r="GR4" s="69" t="s">
         <ns0:v>519</ns0:v>
       </ns0:c>
     </ns0:row>
-    <ns0:row r="5" spans="1:198" ht="57.5" customHeight="1" thickTop="1" thickBot="1" ns3:dyDescent="0.25">
+    <ns0:row r="5" spans="1:199" ht="57.5" customHeight="1" thickTop="1" thickBot="1" ns3:dyDescent="0.25">
       <ns0:c r="A5" s="34" t="s">
         <ns0:v>60</ns0:v>
       </ns0:c>
@@ -5145,400 +5167,403 @@
         <ns0:v>416</ns0:v>
       </ns0:c>
       <ns0:c r="BQ5" s="4" t="s">
+        <ns0:v>653</ns0:v>
+      </ns0:c>
+      <ns0:c r="BR5" s="4" t="s">
         <ns0:v>623</ns0:v>
       </ns0:c>
-      <ns0:c r="BR5" s="4" t="s">
+      <ns0:c r="BS5" s="4" t="s">
         <ns0:v>624</ns0:v>
       </ns0:c>
-      <ns0:c r="BS5" s="4" t="s">
+      <ns0:c r="BT5" s="4" t="s">
         <ns0:v>625</ns0:v>
       </ns0:c>
-      <ns0:c r="BT5" s="4" t="s">
+      <ns0:c r="BU5" s="4" t="s">
         <ns0:v>626</ns0:v>
       </ns0:c>
-      <ns0:c r="BU5" s="4" t="s">
+      <ns0:c r="BV5" s="4" t="s">
         <ns0:v>627</ns0:v>
       </ns0:c>
-      <ns0:c r="BV5" s="4" t="s">
+      <ns0:c r="BW5" s="4" t="s">
         <ns0:v>628</ns0:v>
       </ns0:c>
-      <ns0:c r="BW5" s="4" t="s">
+      <ns0:c r="BX5" s="4" t="s">
         <ns0:v>629</ns0:v>
       </ns0:c>
-      <ns0:c r="BX5" s="4" t="s">
+      <ns0:c r="BY5" s="4" t="s">
         <ns0:v>630</ns0:v>
       </ns0:c>
-      <ns0:c r="BY5" s="4" t="s">
+      <ns0:c r="BZ5" s="4" t="s">
         <ns0:v>631</ns0:v>
       </ns0:c>
-      <ns0:c r="BZ5" s="4" t="s">
+      <ns0:c r="CA5" s="4" t="s">
         <ns0:v>632</ns0:v>
       </ns0:c>
-      <ns0:c r="CA5" s="4" t="s">
+      <ns0:c r="CB5" s="4" t="s">
         <ns0:v>633</ns0:v>
       </ns0:c>
-      <ns0:c r="CB5" s="4" t="s">
+      <ns0:c r="CC5" s="4" t="s">
         <ns0:v>634</ns0:v>
       </ns0:c>
-      <ns0:c r="CC5" s="4" t="s">
+      <ns0:c r="CD5" s="4" t="s">
         <ns0:v>635</ns0:v>
       </ns0:c>
-      <ns0:c r="CD5" s="4" t="s">
+      <ns0:c r="CE5" s="4" t="s">
         <ns0:v>636</ns0:v>
       </ns0:c>
-      <ns0:c r="CE5" s="4" t="s">
+      <ns0:c r="CF5" s="4" t="s">
         <ns0:v>637</ns0:v>
       </ns0:c>
-      <ns0:c r="CF5" s="4" t="s">
+      <ns0:c r="CG5" s="4" t="s">
         <ns0:v>638</ns0:v>
       </ns0:c>
-      <ns0:c r="CG5" s="4" t="s">
+      <ns0:c r="CH5" s="4" t="s">
         <ns0:v>639</ns0:v>
       </ns0:c>
-      <ns0:c r="CH5" s="4" t="s">
+      <ns0:c r="CI5" s="4" t="s">
         <ns0:v>640</ns0:v>
       </ns0:c>
-      <ns0:c r="CI5" s="4" t="s">
+      <ns0:c r="CJ5" s="4" t="s">
         <ns0:v>641</ns0:v>
       </ns0:c>
-      <ns0:c r="CJ5" s="4" t="s">
+      <ns0:c r="CK5" s="4" t="s">
         <ns0:v>642</ns0:v>
       </ns0:c>
-      <ns0:c r="CK5" s="4" t="s">
+      <ns0:c r="CL5" s="4" t="s">
         <ns0:v>643</ns0:v>
       </ns0:c>
-      <ns0:c r="CL5" s="4" t="s">
+      <ns0:c r="CM5" s="4" t="s">
         <ns0:v>644</ns0:v>
       </ns0:c>
-      <ns0:c r="CM5" s="4" t="s">
+      <ns0:c r="CN5" s="4" t="s">
         <ns0:v>645</ns0:v>
       </ns0:c>
-      <ns0:c r="CN5" s="4" t="s">
+      <ns0:c r="CO5" s="4" t="s">
         <ns0:v>646</ns0:v>
       </ns0:c>
-      <ns0:c r="CO5" s="4" t="s">
+      <ns0:c r="CP5" s="4" t="s">
         <ns0:v>647</ns0:v>
       </ns0:c>
-      <ns0:c r="CP5" s="4" t="s">
+      <ns0:c r="CQ5" s="4" t="s">
         <ns0:v>648</ns0:v>
       </ns0:c>
-      <ns0:c r="CQ5" s="4" t="s">
+      <ns0:c r="CR5" s="4" t="s">
         <ns0:v>249</ns0:v>
       </ns0:c>
-      <ns0:c r="CR5" s="4" t="s">
+      <ns0:c r="CS5" s="4" t="s">
         <ns0:v>256</ns0:v>
       </ns0:c>
-      <ns0:c r="CS5" s="4" t="s">
+      <ns0:c r="CT5" s="4" t="s">
         <ns0:v>263</ns0:v>
       </ns0:c>
-      <ns0:c r="CT5" s="4" t="s">
+      <ns0:c r="CU5" s="4" t="s">
         <ns0:v>258</ns0:v>
       </ns0:c>
-      <ns0:c r="CU5" s="4" t="s">
+      <ns0:c r="CV5" s="4" t="s">
         <ns0:v>250</ns0:v>
       </ns0:c>
-      <ns0:c r="CV5" s="4" t="s">
+      <ns0:c r="CW5" s="4" t="s">
         <ns0:v>251</ns0:v>
       </ns0:c>
-      <ns0:c r="CW5" s="4" t="s">
+      <ns0:c r="CX5" s="4" t="s">
         <ns0:v>264</ns0:v>
       </ns0:c>
-      <ns0:c r="CX5" s="4" t="s">
+      <ns0:c r="CY5" s="4" t="s">
         <ns0:v>252</ns0:v>
       </ns0:c>
-      <ns0:c r="CY5" s="4" t="s">
+      <ns0:c r="CZ5" s="4" t="s">
         <ns0:v>253</ns0:v>
       </ns0:c>
-      <ns0:c r="CZ5" s="4" t="s">
+      <ns0:c r="DA5" s="4" t="s">
         <ns0:v>254</ns0:v>
       </ns0:c>
-      <ns0:c r="DA5" s="4" t="s">
+      <ns0:c r="DB5" s="4" t="s">
         <ns0:v>266</ns0:v>
       </ns0:c>
-      <ns0:c r="DB5" s="4" t="s">
+      <ns0:c r="DC5" s="4" t="s">
         <ns0:v>255</ns0:v>
       </ns0:c>
-      <ns0:c r="DC5" s="4" t="s">
+      <ns0:c r="DD5" s="4" t="s">
         <ns0:v>302</ns0:v>
       </ns0:c>
-      <ns0:c r="DD5" s="4" t="s">
+      <ns0:c r="DE5" s="4" t="s">
         <ns0:v>304</ns0:v>
       </ns0:c>
-      <ns0:c r="DE5" s="4" t="s">
+      <ns0:c r="DF5" s="4" t="s">
         <ns0:v>306</ns0:v>
       </ns0:c>
-      <ns0:c r="DF5" s="4" t="s">
+      <ns0:c r="DG5" s="4" t="s">
         <ns0:v>308</ns0:v>
       </ns0:c>
-      <ns0:c r="DG5" s="4" t="s">
+      <ns0:c r="DH5" s="4" t="s">
         <ns0:v>310</ns0:v>
       </ns0:c>
-      <ns0:c r="DH5" s="4" t="s">
+      <ns0:c r="DI5" s="4" t="s">
         <ns0:v>312</ns0:v>
       </ns0:c>
-      <ns0:c r="DI5" s="4" t="s">
+      <ns0:c r="DJ5" s="4" t="s">
         <ns0:v>314</ns0:v>
       </ns0:c>
-      <ns0:c r="DJ5" s="4" t="s">
+      <ns0:c r="DK5" s="4" t="s">
         <ns0:v>316</ns0:v>
       </ns0:c>
-      <ns0:c r="DK5" s="4" t="s">
+      <ns0:c r="DL5" s="4" t="s">
         <ns0:v>277</ns0:v>
       </ns0:c>
-      <ns0:c r="DL5" s="4" t="s">
+      <ns0:c r="DM5" s="4" t="s">
         <ns0:v>278</ns0:v>
       </ns0:c>
-      <ns0:c r="DM5" s="4" t="s">
+      <ns0:c r="DN5" s="4" t="s">
         <ns0:v>279</ns0:v>
       </ns0:c>
-      <ns0:c r="DN5" s="4" t="s">
+      <ns0:c r="DO5" s="4" t="s">
         <ns0:v>280</ns0:v>
       </ns0:c>
-      <ns0:c r="DO5" s="4" t="s">
+      <ns0:c r="DP5" s="4" t="s">
         <ns0:v>283</ns0:v>
       </ns0:c>
-      <ns0:c r="DP5" s="4" t="s">
+      <ns0:c r="DQ5" s="4" t="s">
         <ns0:v>285</ns0:v>
       </ns0:c>
-      <ns0:c r="DQ5" s="4" t="s">
+      <ns0:c r="DR5" s="4" t="s">
         <ns0:v>287</ns0:v>
       </ns0:c>
-      <ns0:c r="DR5" s="4" t="s">
+      <ns0:c r="DS5" s="4" t="s">
         <ns0:v>282</ns0:v>
       </ns0:c>
-      <ns0:c r="DS5" s="4" t="s">
+      <ns0:c r="DT5" s="4" t="s">
         <ns0:v>289</ns0:v>
       </ns0:c>
-      <ns0:c r="DT5" s="4" t="s">
+      <ns0:c r="DU5" s="4" t="s">
         <ns0:v>290</ns0:v>
       </ns0:c>
-      <ns0:c r="DU5" s="4" t="s">
+      <ns0:c r="DV5" s="4" t="s">
         <ns0:v>291</ns0:v>
       </ns0:c>
-      <ns0:c r="DV5" s="4" t="s">
+      <ns0:c r="DW5" s="4" t="s">
         <ns0:v>270</ns0:v>
       </ns0:c>
-      <ns0:c r="DW5" s="4" t="s">
+      <ns0:c r="DX5" s="4" t="s">
         <ns0:v>182</ns0:v>
       </ns0:c>
-      <ns0:c r="DX5" s="4" t="s">
+      <ns0:c r="DY5" s="4" t="s">
         <ns0:v>183</ns0:v>
       </ns0:c>
-      <ns0:c r="DY5" s="4" t="s">
+      <ns0:c r="DZ5" s="4" t="s">
         <ns0:v>274</ns0:v>
       </ns0:c>
-      <ns0:c r="DZ5" s="4" t="s">
+      <ns0:c r="EA5" s="4" t="s">
         <ns0:v>257</ns0:v>
       </ns0:c>
-      <ns0:c r="EA5" s="4" t="s">
+      <ns0:c r="EB5" s="4" t="s">
         <ns0:v>293</ns0:v>
       </ns0:c>
-      <ns0:c r="EB5" s="4" t="s">
+      <ns0:c r="EC5" s="4" t="s">
         <ns0:v>295</ns0:v>
       </ns0:c>
-      <ns0:c r="EC5" s="4" t="s">
+      <ns0:c r="ED5" s="4" t="s">
         <ns0:v>297</ns0:v>
       </ns0:c>
-      <ns0:c r="ED5" s="4" t="s">
+      <ns0:c r="EE5" s="4" t="s">
         <ns0:v>299</ns0:v>
       </ns0:c>
-      <ns0:c r="EE5" t="s">
+      <ns0:c r="EF5" t="s">
         <ns0:v>542</ns0:v>
       </ns0:c>
-      <ns0:c r="EF5" s="4" t="s">
+      <ns0:c r="EG5" s="4" t="s">
         <ns0:v>157</ns0:v>
       </ns0:c>
-      <ns0:c r="EG5" s="4" t="s">
+      <ns0:c r="EH5" s="4" t="s">
         <ns0:v>113</ns0:v>
       </ns0:c>
-      <ns0:c r="EH5" s="4" t="s">
+      <ns0:c r="EI5" s="4" t="s">
         <ns0:v>114</ns0:v>
       </ns0:c>
-      <ns0:c r="EI5" s="4" t="s">
+      <ns0:c r="EJ5" s="4" t="s">
         <ns0:v>159</ns0:v>
       </ns0:c>
-      <ns0:c r="EJ5" s="4" t="s">
+      <ns0:c r="EK5" s="4" t="s">
         <ns0:v>158</ns0:v>
       </ns0:c>
-      <ns0:c r="EK5" s="4" t="s">
+      <ns0:c r="EL5" s="4" t="s">
         <ns0:v>115</ns0:v>
       </ns0:c>
-      <ns0:c r="EL5" s="4" t="s">
+      <ns0:c r="EM5" s="4" t="s">
         <ns0:v>116</ns0:v>
       </ns0:c>
-      <ns0:c r="EM5" s="4" t="s">
+      <ns0:c r="EN5" s="4" t="s">
         <ns0:v>156</ns0:v>
       </ns0:c>
-      <ns0:c r="EN5" s="4" t="s">
+      <ns0:c r="EO5" s="4" t="s">
         <ns0:v>35</ns0:v>
       </ns0:c>
-      <ns0:c r="EO5" s="4" t="s">
+      <ns0:c r="EP5" s="4" t="s">
         <ns0:v>228</ns0:v>
       </ns0:c>
-      <ns0:c r="EP5" s="4" t="s">
+      <ns0:c r="EQ5" s="4" t="s">
         <ns0:v>428</ns0:v>
       </ns0:c>
-      <ns0:c r="EQ5" s="4" t="s">
+      <ns0:c r="ER5" s="4" t="s">
         <ns0:v>39</ns0:v>
       </ns0:c>
-      <ns0:c r="ER5" s="4" t="s">
+      <ns0:c r="ES5" s="4" t="s">
         <ns0:v>226</ns0:v>
       </ns0:c>
-      <ns0:c r="ES5" s="4" t="s">
+      <ns0:c r="ET5" s="4" t="s">
         <ns0:v>430</ns0:v>
       </ns0:c>
-      <ns0:c r="ET5" s="4" t="s">
+      <ns0:c r="EU5" s="4" t="s">
         <ns0:v>422</ns0:v>
       </ns0:c>
-      <ns0:c r="EU5" s="4" t="s">
+      <ns0:c r="EV5" s="4" t="s">
         <ns0:v>423</ns0:v>
       </ns0:c>
-      <ns0:c r="EV5" s="4" t="s">
+      <ns0:c r="EW5" s="4" t="s">
         <ns0:v>523</ns0:v>
       </ns0:c>
-      <ns0:c r="EW5" s="7" t="s">
+      <ns0:c r="EX5" s="7" t="s">
         <ns0:v>42</ns0:v>
       </ns0:c>
-      <ns0:c r="EX5" s="4" t="s">
+      <ns0:c r="EY5" s="4" t="s">
         <ns0:v>224</ns0:v>
       </ns0:c>
-      <ns0:c r="EY5" s="4" t="s">
+      <ns0:c r="EZ5" s="4" t="s">
         <ns0:v>432</ns0:v>
       </ns0:c>
-      <ns0:c r="EZ5" s="4" t="s">
+      <ns0:c r="FA5" s="4" t="s">
         <ns0:v>69</ns0:v>
       </ns0:c>
-      <ns0:c r="FA5" s="4" t="s">
+      <ns0:c r="FB5" s="4" t="s">
         <ns0:v>222</ns0:v>
       </ns0:c>
-      <ns0:c r="FB5" s="4" t="s">
+      <ns0:c r="FC5" s="4" t="s">
         <ns0:v>434</ns0:v>
       </ns0:c>
-      <ns0:c r="FC5" s="4" t="s">
+      <ns0:c r="FD5" s="4" t="s">
         <ns0:v>38</ns0:v>
       </ns0:c>
-      <ns0:c r="FD5" s="4" t="s">
+      <ns0:c r="FE5" s="4" t="s">
         <ns0:v>220</ns0:v>
       </ns0:c>
-      <ns0:c r="FE5" s="4" t="s">
+      <ns0:c r="FF5" s="4" t="s">
         <ns0:v>436</ns0:v>
       </ns0:c>
-      <ns0:c r="FF5" s="7" t="s">
+      <ns0:c r="FG5" s="7" t="s">
         <ns0:v>41</ns0:v>
       </ns0:c>
-      <ns0:c r="FG5" s="4" t="s">
+      <ns0:c r="FH5" s="4" t="s">
         <ns0:v>218</ns0:v>
       </ns0:c>
-      <ns0:c r="FH5" s="4" t="s">
+      <ns0:c r="FI5" s="4" t="s">
         <ns0:v>447</ns0:v>
       </ns0:c>
-      <ns0:c r="FI5" s="7" t="s">
+      <ns0:c r="FJ5" s="7" t="s">
         <ns0:v>4</ns0:v>
       </ns0:c>
-      <ns0:c r="FJ5" s="4" t="s">
+      <ns0:c r="FK5" s="4" t="s">
         <ns0:v>216</ns0:v>
       </ns0:c>
-      <ns0:c r="FK5" s="4" t="s">
+      <ns0:c r="FL5" s="4" t="s">
         <ns0:v>449</ns0:v>
       </ns0:c>
-      <ns0:c r="FL5" s="7" t="s">
+      <ns0:c r="FM5" s="7" t="s">
         <ns0:v>70</ns0:v>
       </ns0:c>
-      <ns0:c r="FM5" s="4" t="s">
+      <ns0:c r="FN5" s="4" t="s">
         <ns0:v>214</ns0:v>
       </ns0:c>
-      <ns0:c r="FN5" s="4" t="s">
+      <ns0:c r="FO5" s="4" t="s">
         <ns0:v>451</ns0:v>
       </ns0:c>
-      <ns0:c r="FO5" s="4" t="s">
+      <ns0:c r="FP5" s="4" t="s">
         <ns0:v>40</ns0:v>
       </ns0:c>
-      <ns0:c r="FP5" s="4" t="s">
+      <ns0:c r="FQ5" s="4" t="s">
         <ns0:v>212</ns0:v>
       </ns0:c>
-      <ns0:c r="FQ5" s="4" t="s">
+      <ns0:c r="FR5" s="4" t="s">
         <ns0:v>453</ns0:v>
       </ns0:c>
-      <ns0:c r="FR5" s="4" t="s">
+      <ns0:c r="FS5" s="4" t="s">
         <ns0:v>134</ns0:v>
       </ns0:c>
-      <ns0:c r="FS5" s="4" t="s">
+      <ns0:c r="FT5" s="4" t="s">
         <ns0:v>210</ns0:v>
       </ns0:c>
-      <ns0:c r="FT5" s="4" t="s">
+      <ns0:c r="FU5" s="4" t="s">
         <ns0:v>105</ns0:v>
       </ns0:c>
-      <ns0:c r="FU5" s="4" t="s">
+      <ns0:c r="FV5" s="4" t="s">
         <ns0:v>461</ns0:v>
       </ns0:c>
-      <ns0:c r="FV5" s="4" t="s">
+      <ns0:c r="FW5" s="4" t="s">
         <ns0:v>208</ns0:v>
       </ns0:c>
-      <ns0:c r="FW5" s="4" t="s">
+      <ns0:c r="FX5" s="4" t="s">
         <ns0:v>455</ns0:v>
       </ns0:c>
-      <ns0:c r="FX5" s="14" t="s">
+      <ns0:c r="FY5" s="14" t="s">
         <ns0:v>78</ns0:v>
       </ns0:c>
-      <ns0:c r="FY5" s="4" t="s">
+      <ns0:c r="FZ5" s="4" t="s">
         <ns0:v>206</ns0:v>
       </ns0:c>
-      <ns0:c r="FZ5" s="4" t="s">
+      <ns0:c r="GA5" s="4" t="s">
         <ns0:v>457</ns0:v>
       </ns0:c>
-      <ns0:c r="GA5" s="4" t="s">
+      <ns0:c r="GB5" s="4" t="s">
         <ns0:v>59</ns0:v>
       </ns0:c>
-      <ns0:c r="GB5" s="4" t="s">
+      <ns0:c r="GC5" s="4" t="s">
         <ns0:v>203</ns0:v>
       </ns0:c>
-      <ns0:c r="GC5" s="4" t="s">
+      <ns0:c r="GD5" s="4" t="s">
         <ns0:v>438</ns0:v>
       </ns0:c>
-      <ns0:c r="GD5" s="7" t="s">
+      <ns0:c r="GE5" s="7" t="s">
         <ns0:v>140</ns0:v>
       </ns0:c>
-      <ns0:c r="GE5" s="4" t="s">
+      <ns0:c r="GF5" s="4" t="s">
         <ns0:v>202</ns0:v>
       </ns0:c>
-      <ns0:c r="GF5" s="4" t="s">
+      <ns0:c r="GG5" s="4" t="s">
         <ns0:v>440</ns0:v>
       </ns0:c>
-      <ns0:c r="GG5" s="4" t="s">
+      <ns0:c r="GH5" s="4" t="s">
         <ns0:v>142</ns0:v>
       </ns0:c>
-      <ns0:c r="GH5" s="4" t="s">
+      <ns0:c r="GI5" s="4" t="s">
         <ns0:v>201</ns0:v>
       </ns0:c>
-      <ns0:c r="GI5" s="4" t="s">
+      <ns0:c r="GJ5" s="4" t="s">
         <ns0:v>442</ns0:v>
       </ns0:c>
-      <ns0:c r="GJ5" s="7" t="s">
+      <ns0:c r="GK5" s="7" t="s">
         <ns0:v>144</ns0:v>
       </ns0:c>
-      <ns0:c r="GK5" s="4" t="s">
+      <ns0:c r="GL5" s="4" t="s">
         <ns0:v>198</ns0:v>
       </ns0:c>
-      <ns0:c r="GL5" s="4" t="s">
+      <ns0:c r="GM5" s="4" t="s">
         <ns0:v>444</ns0:v>
       </ns0:c>
-      <ns0:c r="GM5" s="7" t="s">
+      <ns0:c r="GN5" s="7" t="s">
         <ns0:v>146</ns0:v>
       </ns0:c>
-      <ns0:c r="GN5" s="4" t="s">
+      <ns0:c r="GO5" s="4" t="s">
         <ns0:v>196</ns0:v>
       </ns0:c>
-      <ns0:c r="GO5" s="4" t="s">
+      <ns0:c r="GP5" s="4" t="s">
         <ns0:v>459</ns0:v>
       </ns0:c>
-      <ns0:c r="GP5" s="4" t="s">
+      <ns0:c r="GQ5" s="4" t="s">
         <ns0:v>520</ns0:v>
       </ns0:c>
-      <ns0:c r="GQ5" s="4" t="s">
+      <ns0:c r="GR5" s="4" t="s">
         <ns0:v>521</ns0:v>
       </ns0:c>
     </ns0:row>
-    <ns0:row r="6" spans="1:198" ht="16" thickTop="1" ns3:dyDescent="0.2">
+    <ns0:row r="6" spans="1:199" ht="16" thickTop="1" ns3:dyDescent="0.2">
       <ns0:c r="C6" s="1" t="s">
         <ns0:v>386</ns0:v>
       </ns0:c>
@@ -5607,10 +5632,9 @@
       <ns0:c r="BO6" s="1" t="s">
         <ns0:v>101</ns0:v>
       </ns0:c>
-      <ns0:c r="BQ6" s="72" t="s">
+      <ns0:c r="BR6" s="72" t="s">
         <ns0:v>426</ns0:v>
       </ns0:c>
-      <ns0:c r="BS6"/>
       <ns0:c r="BT6"/>
       <ns0:c r="BU6"/>
       <ns0:c r="BV6"/>
@@ -5618,46 +5642,47 @@
       <ns0:c r="BX6"/>
       <ns0:c r="BY6"/>
       <ns0:c r="BZ6"/>
-      <ns0:c r="CA6" s="72" t="s">
+      <ns0:c r="CA6"/>
+      <ns0:c r="CB6" s="72" t="s">
         <ns0:v>649</ns0:v>
       </ns0:c>
-      <ns0:c r="CC6"/>
-      <ns0:c r="CD6" s="72" t="s">
+      <ns0:c r="CD6"/>
+      <ns0:c r="CE6" s="72" t="s">
         <ns0:v>427</ns0:v>
       </ns0:c>
-      <ns0:c r="CE6"/>
       <ns0:c r="CF6"/>
       <ns0:c r="CG6"/>
       <ns0:c r="CH6"/>
       <ns0:c r="CI6"/>
       <ns0:c r="CJ6"/>
-      <ns0:c r="CK6" t="s">
+      <ns0:c r="CK6"/>
+      <ns0:c r="CL6" t="s">
         <ns0:v>516</ns0:v>
       </ns0:c>
-      <ns0:c r="CL6"/>
       <ns0:c r="CM6"/>
-      <ns0:c r="CO6"/>
+      <ns0:c r="CN6"/>
       <ns0:c r="CP6"/>
-      <ns0:c r="EN6" s="1" t="s">
+      <ns0:c r="CQ6"/>
+      <ns0:c r="EO6" s="1" t="s">
         <ns0:v>399</ns0:v>
       </ns0:c>
-      <ns0:c r="EO6" s="1" t="b">
+      <ns0:c r="EP6" s="1" t="b">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="GG6" s="1" t="s">
+      <ns0:c r="GH6" s="1" t="s">
         <ns0:v>400</ns0:v>
       </ns0:c>
-      <ns0:c r="GH6" s="1" t="b">
+      <ns0:c r="GI6" s="1" t="b">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="GJ6" s="1" t="s">
+      <ns0:c r="GK6" s="1" t="s">
         <ns0:v>401</ns0:v>
       </ns0:c>
-      <ns0:c r="GK6" s="1" t="b">
+      <ns0:c r="GL6" s="1" t="b">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
-    <ns0:row r="7" spans="1:198" ns3:dyDescent="0.2">
+    <ns0:row r="7" spans="1:199" ns3:dyDescent="0.2">
       <ns0:c r="C7" s="1" t="s">
         <ns0:v>386</ns0:v>
       </ns0:c>
@@ -5687,7 +5712,7 @@
       </ns0:c>
     </ns0:row>
   </ns0:sheetData>
-  <ns0:dataValidations count="9">
+  <ns0:dataValidations count="10">
     <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I6:I1048576" ns2:uid="{00000000-0002-0000-0000-000000000000}">
       <ns0:formula1>"Class,Collection,File,Fonds,Item,Other Level,Record Group,Series,Sub-Fonds,Sub-Group,Sub-Series"</ns0:formula1>
     </ns0:dataValidation>
@@ -5701,20 +5726,23 @@
       <ns0:formula1>1</ns0:formula1>
       <ns0:formula2>20</ns0:formula2>
     </ns0:dataValidation>
-    <ns0:dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="K6:K1048576 GG6:GG1048576 GD6:GD1048576 FX6:FX1048576 GA6:GA1048576 FC6:FC1048576 FU6:FU1048576 FO6:FO1048576 FR6:FR1048576 FL6:FL1048576 FI6:FI1048576 FF6:FF1048576 GJ6:GJ1048576 EZ6:EZ1048576 EW6:EW1048576 EQ6:EQ1048576 Q6:Q1048576 EN6:EN1048576 U6:U1048576 GM6:GM1048576" ns2:uid="{00000000-0002-0000-0000-000004000000}">
+    <ns0:dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="K6:K1048576 GH6:GH1048576 GE6:GE1048576 FY6:FY1048576 GB6:GB1048576 FD6:FD1048576 FV6:FV1048576 FP6:FP1048576 FS6:FS1048576 FM6:FM1048576 FJ6:FJ1048576 FG6:FG1048576 GK6:GK1048576 FA6:FA1048576 EX6:EX1048576 ER6:ER1048576 Q6:Q1048576 EO6:EO1048576 U6:U1048576 GN6:GN1048576" ns2:uid="{00000000-0002-0000-0000-000004000000}">
       <ns0:formula1>"FALSE,TRUE"</ns0:formula1>
     </ns0:dataValidation>
-    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR6:BR7 CA6:CA7 CB6:CB7 CE6:CE7 CN6:CN7 CO6:CO7">
+    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BS6:BS7 CB6:CB7 CC6:CC7 CF6:CF7 CO6:CO7 CP6:CP7">
       <ns0:formula1>"FALSE,TRUE"</ns0:formula1>
     </ns0:dataValidation>
-    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BT6:BT7 CG6:CG7">
+    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU6:BU7 CH6:CH7">
       <ns0:formula1>"none,onLoad,onRequest,other"</ns0:formula1>
     </ns0:dataValidation>
-    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU6:BU7 CH6:CH7">
+    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BV6:BV7 CI6:CI7">
       <ns0:formula1>"embed,new,none,other,replace"</ns0:formula1>
     </ns0:dataValidation>
-    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ6:BZ7 CM6:CM7">
+    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA6:CA7 CN6:CN7">
       <ns0:formula1>"MD5,SHA-1,SHA-256,SHA-384,SHA-512"</ns0:formula1>
+    </ns0:dataValidation>
+    <ns0:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ6:BQ7">
+      <ns0:formula1>"FALSE,TRUE"</ns0:formula1>
     </ns0:dataValidation>
   </ns0:dataValidations>
   <ns0:hyperlinks>
@@ -5730,7 +5758,7 @@
           <ns5:formula1>
             <ns6:f>Sheet2!$A$2:$A$4</ns6:f>
           </ns5:formula1>
-          <ns6:sqref>CS6:CS1048576 CW6:CW1048576 DM6:DM1048576 DA6:DA1048576 DY6:DY1048576 DQ6:DQ1048576 DU6:DU1048576 EC6:EC1048576 DE6:DE1048576 DI6:DI1048576</ns6:sqref>
+          <ns6:sqref>CT6:CT1048576 CX6:CX1048576 DN6:DN1048576 DB6:DB1048576 DZ6:DZ1048576 DR6:DR1048576 DV6:DV1048576 ED6:ED1048576 DF6:DF1048576 DJ6:DJ1048576</ns6:sqref>
         </ns5:dataValidation>
       </ns5:dataValidations>
     </ns0:ext>

</xml_diff>